<commit_message>
feat: publish PTO ISA 0.58.0
</commit_message>
<xml_diff>
--- a/spec/encoding/PTO-ISA-Encoding.xlsx
+++ b/spec/encoding/PTO-ISA-Encoding.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7be91cb1db834a9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="R88f3fdf121894f82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="Rf386aba083e6451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6f8d8ab6d45b4199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rce61c905a5d940fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R691a09b226ca4fbe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7154,7 +7154,7 @@
 D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
 Cooperative form 中 C/D、RowMaxIn/Out、GroupMaxOut 为 MShard4；Bias、vector QuantParam、vector PReLU 是四 PE 上内容相同的完整 Local N-vector；scalar GPR 参数也必须在四 PE 上相等。
 D==C 仅在 D 保持 TileAcc role 且 dtype、shape、layout、allocation 完全相同时合法；实现必须 read-old/rename-new，禁止物理原地覆盖。C 不携带 partial-sum provenance 要求。
-Cooperative TMATMUL 要求所有 Shared value fully-defined、四 PE 静态收敛并以相同动态顺序到达；该 rendezvous 不建立 GM ordering。
+Cooperative TMATMUL 的 Shared read 不修改 descriptor/payload；并发 overlap 由程序避免，且该 rendezvous 不建立 GM ordering。
 一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
@@ -7218,7 +7218,7 @@
 D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
 Cooperative form 中 C/D、RowMaxIn/Out、GroupMaxOut 为 MShard4；Bias、vector QuantParam、vector PReLU 是四 PE 上内容相同的完整 Local N-vector；scalar GPR 参数也必须在四 PE 上相等。
 D 必须是显式 ordinary physical Local destination。
-Cooperative TMATMUL 要求所有 Shared value fully-defined、四 PE 静态收敛并以相同动态顺序到达；该 rendezvous 不建立 GM ordering。
+Cooperative TMATMUL 的 Shared read 不修改 descriptor/payload；并发 overlap 由程序避免，且该 rendezvous 不建立 GM ordering。
 一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
@@ -7304,9 +7304,9 @@
       <x:c r="L107" s="91" t="str">
         <x:v>Shared→Shared TMOV is absent in v5; copy/transform through Local Tile.
 Runtime mode, owner or size is illegal.
-Partial Shared values may be moved or partition-stored but not used by CUBE compute or Broadcast.
-PE_MASK selects destination/local payloads but does not reduce Shared source-ready or collective participation requirements.
-Shared IDs and versions are compiler-managed; C++ cannot specify S#n.
+PE_MASK is a four-bit quarter predicate; multiple bits are allowed and
+  0000 is a no-op.
+Absolute Shared registers are compiler-managed; C++ cannot specify Sx.
 RecordEvent is reused; there is no SharedEvent, and event completion is not a cross-PE GM fence.</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
docs: publish complete PTO ISA 0.58 reference
</commit_message>
<xml_diff>
--- a/spec/encoding/PTO-ISA-Encoding.xlsx
+++ b/spec/encoding/PTO-ISA-Encoding.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6f8d8ab6d45b4199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rce61c905a5d940fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R691a09b226ca4fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R77efea90e68d4cb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rd5d2a39aebb44e71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="Rfc64d61f63034444"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1134,32 +1134,6 @@
 3. Destination layout restrictions are target/profile-defined; some targets require row-major dst.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TRANDOM</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">dst random tile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TRandomKey via B.IOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TRandomCounter via B.IOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">S32, U32</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TEPL Mode 3, Function 9, TileOp 0x69;</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Generate counter-based pseudo-random values into dst.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1. A5 dst dtype must be S32 or U32 and dst must be row-major.
-2. Rounds must be 7 or 10; default is 10.
-3. Key and counter operands must be valid and non-null.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">TFILLPAD</x:t>
   </x:si>
   <x:si>
@@ -1403,35 +1377,6 @@
     <x:t xml:space="preserve">1. Supported tile types, layout, padding, repeat, and config fields are target/implementation-defined.
 2. posM/posK select the convolution window position consumed by the opcode profile.
 3. A2/A3 and A5 differ in how img2col repeat/padding state is configured.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">排序</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TSORT32</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">dst sorted value/index pairs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">src value tile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">idx tile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">values: F16, F32; idx: U32</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TEPL Mode 3, Function 12, TileOp 0x6C;</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sort each 32-element block and carry indices along with values.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1. TSORT32 does not take WaitEvents and does not implicitly call TSYNC.
-2. dst/src value dtype must be F16 or F32; idx dtype must be U32.
-3. dst/src/idx must be Vec row-major; sorting is independent per 32-element block.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TMRGSORT</x:t>
@@ -2339,7 +2284,7 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="125">
+  <x:cellXfs count="128">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -2713,6 +2658,15 @@
       <x:alignment horizontal="center" vertical="top"/>
     </x:xf>
     <x:xf fontId="3" borderId="23" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="3" fillId="0" borderId="23" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf fontId="3" fillId="0" borderId="23" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top"/>
+    </x:xf>
+    <x:xf fontId="3" fillId="0" borderId="23" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -6049,7 +6003,7 @@
 C.B.IOS
 B.IOR
 Shared pe_scope form
-BSTART.TLSU Function 12
+BSTART.TLSU Function 14
 C.B.IOS
 B.IOR</x:v>
       </x:c>
@@ -6071,7 +6025,7 @@
         <x:v>PTO TSTORE dtype/layout combinations supported by the v5 TLSU profile</x:v>
       </x:c>
       <x:c r="J77" s="41" t="str">
-        <x:v>TLSU Function 1; Shared pe_scope Function 12;</x:v>
+        <x:v>TLSU Function 1; Shared pe_scope Function 14;</x:v>
       </x:c>
       <x:c r="K77" s="2" t="s">
         <x:v>313</x:v>
@@ -6306,184 +6260,186 @@
         <x:v>358</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" ht="101">
+    <x:row r="84" ht="84.75">
       <x:c r="A84" s="53"/>
-      <x:c r="B84" s="54"/>
-      <x:c r="C84" s="16" t="s">
+      <x:c r="B84" s="55"/>
+      <x:c r="C84" s="24" t="s">
         <x:v>359</x:v>
       </x:c>
-      <x:c r="D84" s="17" t="str">
-        <x:v>BSTART.TEPL TRANDOM, DataType
+      <x:c r="D84" s="25" t="str">
+        <x:v>BSTART.TEPL TFILLPAD, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E84" s="25" t="s">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="F84" s="25" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G84" s="25" t="s">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="H84" s="25"/>
+      <x:c r="I84" s="25" t="s">
+        <x:v>362</x:v>
+      </x:c>
+      <x:c r="J84" s="43" t="s">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="K84" s="2" t="s">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="L84" s="3" t="s">
+        <x:v>365</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="118">
+      <x:c r="A85" s="53"/>
+      <x:c r="B85" s="52" t="s">
+        <x:v>366</x:v>
+      </x:c>
+      <x:c r="C85" s="13" t="s">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="D85" s="17" t="str">
+        <x:v>BSTART.TEPL TCVT, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E85" s="17" t="s">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="F85" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G85" s="17" t="s">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="H85" s="17"/>
+      <x:c r="I85" s="17" t="s">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="J85" s="41" t="s">
+        <x:v>371</x:v>
+      </x:c>
+      <x:c r="K85" s="2" t="s">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="L85" s="3" t="s">
+        <x:v>373</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="84">
+      <x:c r="A86" s="53"/>
+      <x:c r="B86" s="54"/>
+      <x:c r="C86" s="16" t="s">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="D86" s="17" t="str">
+        <x:v>BSTART.TEPL TQUANT, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E86" s="17" t="s">
+        <x:v>375</x:v>
+      </x:c>
+      <x:c r="F86" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G86" s="17" t="s">
+        <x:v>376</x:v>
+      </x:c>
+      <x:c r="H86" s="17" t="str">
+        <x:v>offset/scaling/index Tile (optional)</x:v>
+      </x:c>
+      <x:c r="I86" s="17" t="s">
+        <x:v>377</x:v>
+      </x:c>
+      <x:c r="J86" s="41" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="K86" s="2" t="s">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="L86" s="3" t="s">
+        <x:v>380</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="84.75">
+      <x:c r="A87" s="53"/>
+      <x:c r="B87" s="55"/>
+      <x:c r="C87" s="16" t="s">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="D87" s="17" t="str">
+        <x:v>BSTART.TEPL TDEQUANT, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E87" s="17" t="s">
+        <x:v>382</x:v>
+      </x:c>
+      <x:c r="F87" s="17" t="s">
+        <x:v>383</x:v>
+      </x:c>
+      <x:c r="G87" s="17" t="s">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="H87" s="17" t="s">
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="I87" s="17" t="s">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="J87" s="41" t="s">
+        <x:v>387</x:v>
+      </x:c>
+      <x:c r="K87" s="2" t="s">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="L87" s="3" t="s">
+        <x:v>389</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="101">
+      <x:c r="A88" s="53"/>
+      <x:c r="B88" s="52" t="s">
+        <x:v>390</x:v>
+      </x:c>
+      <x:c r="C88" s="56" t="s">
+        <x:v>391</x:v>
+      </x:c>
+      <x:c r="D88" s="56" t="str">
+        <x:v>BSTART.TEPL TEXTRACT, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT
 B.IOR</x:v>
       </x:c>
-      <x:c r="E84" s="17" t="s">
-        <x:v>360</x:v>
-      </x:c>
-      <x:c r="F84" s="17" t="s">
-        <x:v>361</x:v>
-      </x:c>
-      <x:c r="G84" s="17" t="s">
-        <x:v>362</x:v>
-      </x:c>
-      <x:c r="H84" s="17"/>
-      <x:c r="I84" s="17" t="s">
-        <x:v>363</x:v>
-      </x:c>
-      <x:c r="J84" s="41" t="s">
-        <x:v>364</x:v>
-      </x:c>
-      <x:c r="K84" s="2" t="s">
-        <x:v>365</x:v>
-      </x:c>
-      <x:c r="L84" s="3" t="s">
-        <x:v>366</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="85" ht="84.75">
-      <x:c r="A85" s="53"/>
-      <x:c r="B85" s="55"/>
-      <x:c r="C85" s="24" t="s">
-        <x:v>367</x:v>
-      </x:c>
-      <x:c r="D85" s="25" t="str">
-        <x:v>BSTART.TEPL TFILLPAD, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E85" s="25" t="s">
-        <x:v>368</x:v>
-      </x:c>
-      <x:c r="F85" s="25" t="s">
+      <x:c r="E88" s="9" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="F88" s="9" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="G85" s="25" t="s">
-        <x:v>369</x:v>
-      </x:c>
-      <x:c r="H85" s="25"/>
-      <x:c r="I85" s="25" t="s">
-        <x:v>370</x:v>
-      </x:c>
-      <x:c r="J85" s="43" t="s">
-        <x:v>371</x:v>
-      </x:c>
-      <x:c r="K85" s="2" t="s">
-        <x:v>372</x:v>
-      </x:c>
-      <x:c r="L85" s="3" t="s">
-        <x:v>373</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="86" ht="118">
-      <x:c r="A86" s="53"/>
-      <x:c r="B86" s="52" t="s">
-        <x:v>374</x:v>
-      </x:c>
-      <x:c r="C86" s="13" t="s">
-        <x:v>375</x:v>
-      </x:c>
-      <x:c r="D86" s="17" t="str">
-        <x:v>BSTART.TEPL TCVT, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E86" s="17" t="s">
-        <x:v>376</x:v>
-      </x:c>
-      <x:c r="F86" s="17" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="G86" s="17" t="s">
-        <x:v>377</x:v>
-      </x:c>
-      <x:c r="H86" s="17"/>
-      <x:c r="I86" s="17" t="s">
-        <x:v>378</x:v>
-      </x:c>
-      <x:c r="J86" s="41" t="s">
-        <x:v>379</x:v>
-      </x:c>
-      <x:c r="K86" s="2" t="s">
-        <x:v>380</x:v>
-      </x:c>
-      <x:c r="L86" s="3" t="s">
-        <x:v>381</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="87" ht="84">
-      <x:c r="A87" s="53"/>
-      <x:c r="B87" s="54"/>
-      <x:c r="C87" s="16" t="s">
-        <x:v>382</x:v>
-      </x:c>
-      <x:c r="D87" s="17" t="str">
-        <x:v>BSTART.TEPL TQUANT, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E87" s="17" t="s">
-        <x:v>383</x:v>
-      </x:c>
-      <x:c r="F87" s="17" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="G87" s="17" t="s">
-        <x:v>384</x:v>
-      </x:c>
-      <x:c r="H87" s="17" t="str">
-        <x:v>offset/scaling/index Tile (optional)</x:v>
-      </x:c>
-      <x:c r="I87" s="17" t="s">
-        <x:v>385</x:v>
-      </x:c>
-      <x:c r="J87" s="41" t="s">
-        <x:v>386</x:v>
-      </x:c>
-      <x:c r="K87" s="2" t="s">
-        <x:v>387</x:v>
-      </x:c>
-      <x:c r="L87" s="3" t="s">
-        <x:v>388</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="88" ht="84.75">
-      <x:c r="A88" s="53"/>
-      <x:c r="B88" s="55"/>
-      <x:c r="C88" s="16" t="s">
-        <x:v>389</x:v>
-      </x:c>
-      <x:c r="D88" s="17" t="str">
-        <x:v>BSTART.TEPL TDEQUANT, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E88" s="17" t="s">
-        <x:v>390</x:v>
-      </x:c>
-      <x:c r="F88" s="17" t="s">
-        <x:v>391</x:v>
-      </x:c>
-      <x:c r="G88" s="17" t="s">
-        <x:v>392</x:v>
-      </x:c>
-      <x:c r="H88" s="17" t="s">
+      <x:c r="G88" s="9" t="s">
         <x:v>393</x:v>
       </x:c>
-      <x:c r="I88" s="17" t="s">
+      <x:c r="H88" s="9"/>
+      <x:c r="I88" s="9" t="s">
         <x:v>394</x:v>
       </x:c>
-      <x:c r="J88" s="41" t="s">
+      <x:c r="J88" s="40" t="s">
         <x:v>395</x:v>
       </x:c>
       <x:c r="K88" s="2" t="s">
@@ -6495,230 +6451,228 @@
     </x:row>
     <x:row r="89" ht="101">
       <x:c r="A89" s="53"/>
-      <x:c r="B89" s="52" t="s">
+      <x:c r="B89" s="54"/>
+      <x:c r="C89" s="57" t="s">
         <x:v>398</x:v>
       </x:c>
-      <x:c r="C89" s="56" t="s">
-        <x:v>399</x:v>
-      </x:c>
-      <x:c r="D89" s="56" t="str">
-        <x:v>BSTART.TEPL TEXTRACT, DataType
+      <x:c r="D89" s="57" t="str">
+        <x:v>BSTART.TEPL TINSERT, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT
 B.IOR</x:v>
       </x:c>
-      <x:c r="E89" s="9" t="s">
+      <x:c r="E89" s="17" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F89" s="17" t="s">
+        <x:v>399</x:v>
+      </x:c>
+      <x:c r="G89" s="17" t="s">
+        <x:v>393</x:v>
+      </x:c>
+      <x:c r="H89" s="17"/>
+      <x:c r="I89" s="17" t="s">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="F89" s="9" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="G89" s="9" t="s">
+      <x:c r="J89" s="41" t="s">
         <x:v>401</x:v>
       </x:c>
-      <x:c r="H89" s="9"/>
-      <x:c r="I89" s="9" t="s">
+      <x:c r="K89" s="2" t="s">
         <x:v>402</x:v>
       </x:c>
-      <x:c r="J89" s="40" t="s">
+      <x:c r="L89" s="3" t="s">
         <x:v>403</x:v>
-      </x:c>
-      <x:c r="K89" s="2" t="s">
-        <x:v>404</x:v>
-      </x:c>
-      <x:c r="L89" s="3" t="s">
-        <x:v>405</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="101">
       <x:c r="A90" s="53"/>
       <x:c r="B90" s="54"/>
       <x:c r="C90" s="57" t="s">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="D90" s="57" t="str">
+        <x:v>BSTART.TEPL TGATHER, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E90" s="17" t="s">
+        <x:v>405</x:v>
+      </x:c>
+      <x:c r="F90" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G90" s="17" t="s">
         <x:v>406</x:v>
-      </x:c>
-      <x:c r="D90" s="57" t="str">
-        <x:v>BSTART.TEPL TINSERT, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT
-B.IOR</x:v>
-      </x:c>
-      <x:c r="E90" s="17" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F90" s="17" t="s">
-        <x:v>407</x:v>
-      </x:c>
-      <x:c r="G90" s="17" t="s">
-        <x:v>401</x:v>
       </x:c>
       <x:c r="H90" s="17"/>
       <x:c r="I90" s="17" t="s">
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="J90" s="41" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="J90" s="41" t="s">
+      <x:c r="K90" s="2" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="K90" s="2" t="s">
+      <x:c r="L90" s="3" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="L90" s="3" t="s">
-        <x:v>411</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91" ht="101">
+    </x:row>
+    <x:row r="91" ht="84">
       <x:c r="A91" s="53"/>
       <x:c r="B91" s="54"/>
       <x:c r="C91" s="57" t="s">
+        <x:v>411</x:v>
+      </x:c>
+      <x:c r="D91" s="57" t="str">
+        <x:v>BSTART.TEPL TSCATTER, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E91" s="17" t="s">
         <x:v>412</x:v>
-      </x:c>
-      <x:c r="D91" s="57" t="str">
-        <x:v>BSTART.TEPL TGATHER, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E91" s="17" t="s">
-        <x:v>413</x:v>
       </x:c>
       <x:c r="F91" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G91" s="17" t="s">
-        <x:v>414</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="H91" s="17"/>
       <x:c r="I91" s="17" t="s">
+        <x:v>414</x:v>
+      </x:c>
+      <x:c r="J91" s="41" t="s">
         <x:v>415</x:v>
       </x:c>
-      <x:c r="J91" s="41" t="s">
+      <x:c r="K91" s="2" t="s">
         <x:v>416</x:v>
       </x:c>
-      <x:c r="K91" s="2" t="s">
+      <x:c r="L91" s="3" t="s">
         <x:v>417</x:v>
-      </x:c>
-      <x:c r="L91" s="3" t="s">
-        <x:v>418</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="84">
       <x:c r="A92" s="53"/>
       <x:c r="B92" s="54"/>
       <x:c r="C92" s="57" t="s">
-        <x:v>419</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="D92" s="57" t="str">
-        <x:v>BSTART.TEPL TSCATTER, DataType
+        <x:v>BSTART.TEPL TCONCAT, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
       <x:c r="E92" s="17" t="s">
-        <x:v>420</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F92" s="17" t="s">
-        <x:v>74</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G92" s="17" t="s">
-        <x:v>421</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H92" s="17"/>
       <x:c r="I92" s="17" t="s">
-        <x:v>422</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="J92" s="41" t="s">
-        <x:v>423</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="K92" s="2" t="s">
-        <x:v>424</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="L92" s="3" t="s">
-        <x:v>425</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="84">
       <x:c r="A93" s="53"/>
       <x:c r="B93" s="54"/>
       <x:c r="C93" s="57" t="s">
-        <x:v>426</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="D93" s="57" t="str">
-        <x:v>BSTART.TEPL TCONCAT, DataType
+        <x:v>BSTART.TEPL TTRANS, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
       <x:c r="E93" s="17" t="s">
-        <x:v>15</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="F93" s="17" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G93" s="17" t="s">
-        <x:v>17</x:v>
-      </x:c>
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G93" s="17"/>
       <x:c r="H93" s="17"/>
       <x:c r="I93" s="17" t="s">
-        <x:v>18</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="J93" s="41" t="s">
+        <x:v>424</x:v>
+      </x:c>
+      <x:c r="K93" s="2" t="s">
+        <x:v>425</x:v>
+      </x:c>
+      <x:c r="L93" s="3" t="s">
+        <x:v>426</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="101.75">
+      <x:c r="A94" s="53"/>
+      <x:c r="B94" s="55"/>
+      <x:c r="C94" s="58" t="s">
         <x:v>427</x:v>
       </x:c>
-      <x:c r="K93" s="2" t="s">
+      <x:c r="D94" s="58" t="str">
+        <x:v>BSTART.TEPL TIMG2COL, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT
+B.IOR</x:v>
+      </x:c>
+      <x:c r="E94" s="25" t="s">
         <x:v>428</x:v>
       </x:c>
-      <x:c r="L93" s="3" t="s">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="94" ht="84">
-      <x:c r="A94" s="53"/>
-      <x:c r="B94" s="54"/>
-      <x:c r="C94" s="57" t="s">
+      <x:c r="F94" s="25" t="s">
         <x:v>429</x:v>
       </x:c>
-      <x:c r="D94" s="57" t="str">
-        <x:v>BSTART.TEPL TTRANS, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E94" s="17" t="s">
+      <x:c r="G94" s="25" t="s">
         <x:v>430</x:v>
       </x:c>
-      <x:c r="F94" s="17" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="G94" s="17"/>
-      <x:c r="H94" s="17"/>
-      <x:c r="I94" s="17" t="s">
+      <x:c r="H94" s="25"/>
+      <x:c r="I94" s="25" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="J94" s="43" t="s">
         <x:v>431</x:v>
       </x:c>
-      <x:c r="J94" s="41" t="s">
+      <x:c r="K94" s="2" t="s">
         <x:v>432</x:v>
       </x:c>
-      <x:c r="K94" s="2" t="s">
+      <x:c r="L94" s="3" t="s">
         <x:v>433</x:v>
-      </x:c>
-      <x:c r="L94" s="3" t="s">
-        <x:v>434</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="101.75">
       <x:c r="A95" s="53"/>
       <x:c r="B95" s="55"/>
-      <x:c r="C95" s="58" t="s">
-        <x:v>435</x:v>
+      <x:c r="C95" s="43" t="s">
+        <x:v>434</x:v>
       </x:c>
       <x:c r="D95" s="58" t="str">
-        <x:v>BSTART.TEPL TIMG2COL, DataType
+        <x:v>BSTART.TEPL TMRGSORT, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
@@ -6726,261 +6680,186 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E95" s="25" t="s">
+        <x:v>435</x:v>
+      </x:c>
+      <x:c r="F95" s="25" t="s">
         <x:v>436</x:v>
       </x:c>
-      <x:c r="F95" s="25" t="s">
+      <x:c r="G95" s="25" t="s">
         <x:v>437</x:v>
-      </x:c>
-      <x:c r="G95" s="25" t="s">
-        <x:v>438</x:v>
       </x:c>
       <x:c r="H95" s="25"/>
       <x:c r="I95" s="25" t="s">
-        <x:v>223</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="J95" s="43" t="s">
+        <x:v>438</x:v>
+      </x:c>
+      <x:c r="K95" s="2" t="s">
         <x:v>439</x:v>
       </x:c>
-      <x:c r="K95" s="2" t="s">
+      <x:c r="L95" s="3" t="s">
         <x:v>440</x:v>
-      </x:c>
-      <x:c r="L95" s="3" t="s">
-        <x:v>441</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="84">
       <x:c r="A96" s="53"/>
       <x:c r="B96" s="52" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="C96" s="40" t="s">
         <x:v>442</x:v>
       </x:c>
-      <x:c r="C96" s="40" t="s">
-        <x:v>443</x:v>
-      </x:c>
       <x:c r="D96" s="56" t="str">
-        <x:v>BSTART.TEPL TSORT32, DataType
+        <x:v>BSTART.TEPL TPARTADD, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
       <x:c r="E96" s="9" t="s">
-        <x:v>444</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F96" s="9" t="s">
-        <x:v>445</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G96" s="9" t="s">
-        <x:v>446</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H96" s="9"/>
       <x:c r="I96" s="9" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="J96" s="40" t="s">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="K96" s="2" t="s">
+        <x:v>444</x:v>
+      </x:c>
+      <x:c r="L96" s="3" t="s">
+        <x:v>26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="84">
+      <x:c r="A97" s="53"/>
+      <x:c r="B97" s="54"/>
+      <x:c r="C97" s="41" t="s">
+        <x:v>445</x:v>
+      </x:c>
+      <x:c r="D97" s="57" t="str">
+        <x:v>BSTART.TEPL TPARTMUL, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E97" s="17" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F97" s="17" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G97" s="17" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H97" s="17"/>
+      <x:c r="I97" s="17" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J97" s="41" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="K97" s="2" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="J96" s="40" t="s">
-        <x:v>448</x:v>
-      </x:c>
-      <x:c r="K96" s="2" t="s">
-        <x:v>449</x:v>
-      </x:c>
-      <x:c r="L96" s="3" t="s">
-        <x:v>450</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="97" ht="101.75">
-      <x:c r="A97" s="53"/>
-      <x:c r="B97" s="55"/>
-      <x:c r="C97" s="43" t="s">
-        <x:v>451</x:v>
-      </x:c>
-      <x:c r="D97" s="58" t="str">
-        <x:v>BSTART.TEPL TMRGSORT, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT
-B.IOR</x:v>
-      </x:c>
-      <x:c r="E97" s="25" t="s">
-        <x:v>452</x:v>
-      </x:c>
-      <x:c r="F97" s="25" t="s">
-        <x:v>453</x:v>
-      </x:c>
-      <x:c r="G97" s="25" t="s">
-        <x:v>454</x:v>
-      </x:c>
-      <x:c r="H97" s="25"/>
-      <x:c r="I97" s="25" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="J97" s="43" t="s">
-        <x:v>455</x:v>
-      </x:c>
-      <x:c r="K97" s="2" t="s">
-        <x:v>456</x:v>
-      </x:c>
       <x:c r="L97" s="3" t="s">
-        <x:v>457</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="84">
       <x:c r="A98" s="53"/>
-      <x:c r="B98" s="52" t="s">
-        <x:v>458</x:v>
-      </x:c>
-      <x:c r="C98" s="40" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="D98" s="56" t="str">
-        <x:v>BSTART.TEPL TPARTADD, DataType
+      <x:c r="B98" s="54"/>
+      <x:c r="C98" s="41" t="s">
+        <x:v>448</x:v>
+      </x:c>
+      <x:c r="D98" s="57" t="str">
+        <x:v>BSTART.TEPL TPARTMAX, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
-      <x:c r="E98" s="9" t="s">
+      <x:c r="E98" s="17" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F98" s="9" t="s">
+      <x:c r="F98" s="17" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G98" s="9" t="s">
+      <x:c r="G98" s="17" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H98" s="9"/>
-      <x:c r="I98" s="9" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="J98" s="40" t="s">
-        <x:v>460</x:v>
+      <x:c r="H98" s="17"/>
+      <x:c r="I98" s="17" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="J98" s="41" t="s">
+        <x:v>449</x:v>
       </x:c>
       <x:c r="K98" s="2" t="s">
-        <x:v>461</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="L98" s="3" t="s">
         <x:v>26</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" ht="84">
-      <x:c r="A99" s="53"/>
-      <x:c r="B99" s="54"/>
-      <x:c r="C99" s="41" t="s">
-        <x:v>462</x:v>
-      </x:c>
-      <x:c r="D99" s="57" t="str">
-        <x:v>BSTART.TEPL TPARTMUL, DataType
+    <x:row r="99" ht="84.75">
+      <x:c r="A99" s="59"/>
+      <x:c r="B99" s="55"/>
+      <x:c r="C99" s="43" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="D99" s="58" t="str">
+        <x:v>BSTART.TEPL TPARTMIN, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
-      <x:c r="E99" s="17" t="s">
+      <x:c r="E99" s="25" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F99" s="17" t="s">
+      <x:c r="F99" s="25" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G99" s="17" t="s">
+      <x:c r="G99" s="25" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H99" s="17"/>
-      <x:c r="I99" s="17" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="J99" s="41" t="s">
-        <x:v>463</x:v>
+      <x:c r="H99" s="25"/>
+      <x:c r="I99" s="25" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="J99" s="43" t="s">
+        <x:v>452</x:v>
       </x:c>
       <x:c r="K99" s="2" t="s">
-        <x:v>464</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="L99" s="3" t="s">
         <x:v>26</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" ht="84">
-      <x:c r="A100" s="53"/>
-      <x:c r="B100" s="54"/>
-      <x:c r="C100" s="41" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="D100" s="57" t="str">
-        <x:v>BSTART.TEPL TPARTMAX, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E100" s="17" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F100" s="17" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G100" s="17" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H100" s="17"/>
-      <x:c r="I100" s="17" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="J100" s="41" t="s">
-        <x:v>466</x:v>
-      </x:c>
-      <x:c r="K100" s="2" t="s">
-        <x:v>467</x:v>
-      </x:c>
-      <x:c r="L100" s="3" t="s">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="101" ht="84.75">
-      <x:c r="A101" s="59"/>
-      <x:c r="B101" s="55"/>
-      <x:c r="C101" s="43" t="s">
-        <x:v>468</x:v>
-      </x:c>
-      <x:c r="D101" s="58" t="str">
-        <x:v>BSTART.TEPL TPARTMIN, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E101" s="25" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F101" s="25" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G101" s="25" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H101" s="25"/>
-      <x:c r="I101" s="25" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="J101" s="43" t="s">
-        <x:v>469</x:v>
-      </x:c>
-      <x:c r="K101" s="2" t="s">
-        <x:v>470</x:v>
-      </x:c>
-      <x:c r="L101" s="3" t="s">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="102" ht="101" customHeight="1">
-      <x:c r="A102" s="66" t="str">
+    <x:row r="100" ht="101" customHeight="1">
+      <x:c r="A100" s="66" t="str">
         <x:v>MATRIX Operation
 矩阵乘操作</x:v>
       </x:c>
-      <x:c r="B102" s="66" t="str">
+      <x:c r="B100" s="66" t="str">
         <x:v>矩阵乘向量</x:v>
       </x:c>
-      <x:c r="C102" s="73" t="str">
+      <x:c r="C100" s="73" t="str">
         <x:v>TGEMV_MX_ACC</x:v>
       </x:c>
-      <x:c r="D102" s="78" t="str">
+      <x:c r="D100" s="78" t="str">
         <x:v>BSTART.CUBE TGEMVMX.ACC AType
 B.DATR BType RMode Sat
 B.FPATR
@@ -6990,35 +6869,35 @@
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
-      <x:c r="E102" s="78" t="str">
+      <x:c r="E100" s="78" t="str">
         <x:v>D Tile
 RowMaxOut Tile (optional)
 GroupMaxOut Tile (optional)</x:v>
       </x:c>
-      <x:c r="F102" s="78" t="str">
+      <x:c r="F100" s="78" t="str">
         <x:v>A Tile
 ScaleA Tile</x:v>
       </x:c>
-      <x:c r="G102" s="78" t="str">
+      <x:c r="G100" s="78" t="str">
         <x:v>B/Right Tile
 ScaleB/ScaleRight Tile</x:v>
       </x:c>
-      <x:c r="H102" s="78" t="str">
+      <x:c r="H100" s="78" t="str">
         <x:v>C Tile
 RowMaxIn Tile (optional)
 Quant parameter Tile or GPR (optional)
 ReLU parameter Tile or GPR (optional)</x:v>
       </x:c>
-      <x:c r="I102" s="78" t="str">
+      <x:c r="I100" s="78" t="str">
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
-      <x:c r="J102" s="83" t="str">
+      <x:c r="J100" s="83" t="str">
         <x:v>CUBE Mode 0, Function 22;</x:v>
       </x:c>
-      <x:c r="K102" s="90" t="str">
+      <x:c r="K100" s="90" t="str">
         <x:v>C 是显式 Local AccType Tile input，并在 K 乘积累加前读入 P；它不是隐式 ACC。 PostProcess 只在完整 K 累加后执行一次。</x:v>
       </x:c>
-      <x:c r="L102" s="91" t="str">
+      <x:c r="L100" s="91" t="str">
         <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
 canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
 任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
@@ -7032,18 +6911,18 @@
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" ht="101" customHeight="1">
-      <x:c r="A103" s="66" t="str">
+    <x:row r="101" ht="101" customHeight="1">
+      <x:c r="A101" s="66" t="str">
         <x:v>MATRIX Operation
 矩阵乘操作</x:v>
       </x:c>
-      <x:c r="B103" s="66" t="str">
+      <x:c r="B101" s="66" t="str">
         <x:v>矩阵乘向量</x:v>
       </x:c>
-      <x:c r="C103" s="73" t="str">
+      <x:c r="C101" s="73" t="str">
         <x:v>TGEMV_MX_BIAS</x:v>
       </x:c>
-      <x:c r="D103" s="78" t="str">
+      <x:c r="D101" s="78" t="str">
         <x:v>BSTART.CUBE TGEMVMX.BIAS AType
 B.DATR BType RMode Sat
 B.FPATR
@@ -7053,35 +6932,35 @@
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
-      <x:c r="E103" s="78" t="str">
+      <x:c r="E101" s="78" t="str">
         <x:v>D Tile
 RowMaxOut Tile (optional)
 GroupMaxOut Tile (optional)</x:v>
       </x:c>
-      <x:c r="F103" s="78" t="str">
+      <x:c r="F101" s="78" t="str">
         <x:v>A Tile
 ScaleA Tile</x:v>
       </x:c>
-      <x:c r="G103" s="78" t="str">
+      <x:c r="G101" s="78" t="str">
         <x:v>B/Right Tile
 ScaleB/ScaleRight Tile</x:v>
       </x:c>
-      <x:c r="H103" s="78" t="str">
+      <x:c r="H101" s="78" t="str">
         <x:v>Bias Tile
 RowMaxIn Tile (optional)
 Quant parameter Tile or GPR (optional)
 ReLU parameter Tile or GPR (optional)</x:v>
       </x:c>
-      <x:c r="I103" s="78" t="str">
+      <x:c r="I101" s="78" t="str">
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
-      <x:c r="J103" s="83" t="str">
+      <x:c r="J101" s="83" t="str">
         <x:v>CUBE Mode 0, Function 21;</x:v>
       </x:c>
-      <x:c r="K103" s="90" t="str">
+      <x:c r="K101" s="90" t="str">
         <x:v>Bias 是显式 Local Tile input，并在 K 乘积累加前预装入 P。 PostProcess 只在完整 K 累加后执行一次。</x:v>
       </x:c>
-      <x:c r="L103" s="91" t="str">
+      <x:c r="L101" s="91" t="str">
         <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
 canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
 任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
@@ -7095,18 +6974,18 @@
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
-    <x:row r="104" ht="101" customHeight="1">
-      <x:c r="A104" s="96" t="str">
+    <x:row r="102" ht="101" customHeight="1">
+      <x:c r="A102" s="96" t="str">
         <x:v>MATRIX Operation
 矩阵乘操作</x:v>
       </x:c>
-      <x:c r="B104" s="96" t="str">
+      <x:c r="B102" s="96" t="str">
         <x:v>矩阵乘矩阵</x:v>
       </x:c>
-      <x:c r="C104" s="73" t="str">
+      <x:c r="C102" s="73" t="str">
         <x:v>TMATMUL_MX_ACC</x:v>
       </x:c>
-      <x:c r="D104" s="78" t="str">
+      <x:c r="D102" s="78" t="str">
         <x:v>BSTART.CUBE TMATMULMX.ACC AType
 B.DATR BType RMode Sat
 B.FPATR
@@ -7117,35 +6996,35 @@
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
-      <x:c r="E104" s="78" t="str">
+      <x:c r="E102" s="78" t="str">
         <x:v>D Tile
 RowMaxOut Tile (optional)
 GroupMaxOut Tile (optional)</x:v>
       </x:c>
-      <x:c r="F104" s="78" t="str">
+      <x:c r="F102" s="78" t="str">
         <x:v>A Tile
 ScaleA Tile</x:v>
       </x:c>
-      <x:c r="G104" s="78" t="str">
+      <x:c r="G102" s="78" t="str">
         <x:v>B/Right Tile
 ScaleB/ScaleRight Tile</x:v>
       </x:c>
-      <x:c r="H104" s="78" t="str">
+      <x:c r="H102" s="78" t="str">
         <x:v>C Tile
 RowMaxIn Tile (optional)
 Quant parameter Tile or GPR (optional)
 ReLU parameter Tile or GPR (optional)</x:v>
       </x:c>
-      <x:c r="I104" s="78" t="str">
+      <x:c r="I102" s="78" t="str">
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
-      <x:c r="J104" s="83" t="str">
+      <x:c r="J102" s="83" t="str">
         <x:v>CUBE Mode 0, Function 6;</x:v>
       </x:c>
-      <x:c r="K104" s="90" t="str">
+      <x:c r="K102" s="90" t="str">
         <x:v>C 是显式 Local AccType Tile input，并在 K 乘积累加前读入 P；它不是隐式 ACC。 PostProcess 只在完整 K 累加后执行一次。</x:v>
       </x:c>
-      <x:c r="L104" s="91" t="str">
+      <x:c r="L102" s="91" t="str">
         <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
 canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
 任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
@@ -7159,18 +7038,18 @@
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
-    <x:row r="105" ht="101" customHeight="1">
-      <x:c r="A105" s="96" t="str">
+    <x:row r="103" ht="101" customHeight="1">
+      <x:c r="A103" s="96" t="str">
         <x:v>MATRIX Operation
 矩阵乘操作</x:v>
       </x:c>
-      <x:c r="B105" s="96" t="str">
+      <x:c r="B103" s="96" t="str">
         <x:v>矩阵乘矩阵</x:v>
       </x:c>
-      <x:c r="C105" s="73" t="str">
+      <x:c r="C103" s="73" t="str">
         <x:v>TMATMUL_MX_BIAS</x:v>
       </x:c>
-      <x:c r="D105" s="78" t="str">
+      <x:c r="D103" s="78" t="str">
         <x:v>BSTART.CUBE TMATMULMX.BIAS AType
 B.DATR BType RMode Sat
 B.FPATR
@@ -7181,35 +7060,35 @@
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
-      <x:c r="E105" s="78" t="str">
+      <x:c r="E103" s="78" t="str">
         <x:v>D Tile
 RowMaxOut Tile (optional)
 GroupMaxOut Tile (optional)</x:v>
       </x:c>
-      <x:c r="F105" s="78" t="str">
+      <x:c r="F103" s="78" t="str">
         <x:v>A Tile
 ScaleA Tile</x:v>
       </x:c>
-      <x:c r="G105" s="78" t="str">
+      <x:c r="G103" s="78" t="str">
         <x:v>B/Right Tile
 ScaleB/ScaleRight Tile</x:v>
       </x:c>
-      <x:c r="H105" s="78" t="str">
+      <x:c r="H103" s="78" t="str">
         <x:v>Bias Tile
 RowMaxIn Tile (optional)
 Quant parameter Tile or GPR (optional)
 ReLU parameter Tile or GPR (optional)</x:v>
       </x:c>
-      <x:c r="I105" s="78" t="str">
+      <x:c r="I103" s="78" t="str">
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
-      <x:c r="J105" s="83" t="str">
+      <x:c r="J103" s="83" t="str">
         <x:v>CUBE Mode 0, Function 5;</x:v>
       </x:c>
-      <x:c r="K105" s="90" t="str">
+      <x:c r="K103" s="90" t="str">
         <x:v>Bias 是显式 Local Tile input，并在 K 乘积累加前预装入 P。 PostProcess 只在完整 K 累加后执行一次。</x:v>
       </x:c>
-      <x:c r="L105" s="91" t="str">
+      <x:c r="L103" s="91" t="str">
         <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
 canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
 任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
@@ -7223,91 +7102,327 @@
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
-    <x:row r="106" ht="101" customHeight="1">
-      <x:c r="A106" s="96" t="str">
+    <x:row r="104" ht="101" customHeight="1">
+      <x:c r="A104" s="96" t="str">
         <x:v>Tile Memory Operation
 Tile级访存操作</x:v>
       </x:c>
-      <x:c r="B106" s="96" t="str">
+      <x:c r="B104" s="96" t="str">
         <x:v>PE间搬运</x:v>
       </x:c>
-      <x:c r="C106" s="73" t="str">
+      <x:c r="C104" s="73" t="str">
         <x:v>GMOV</x:v>
       </x:c>
-      <x:c r="D106" s="78" t="str">
+      <x:c r="D104" s="78" t="str">
         <x:v>BSTART.TLSU GMOV, DataType
 B.IOT source, destination, PE_MASK, TSize
 B.IOR peer_tid</x:v>
       </x:c>
-      <x:c r="E106" s="78" t="str">
+      <x:c r="E104" s="78" t="str">
         <x:v>destination Local Tile</x:v>
       </x:c>
-      <x:c r="F106" s="78" t="str">
+      <x:c r="F104" s="78" t="str">
         <x:v>source Local Tile</x:v>
       </x:c>
-      <x:c r="G106" s="78" t="str">
+      <x:c r="G104" s="78" t="str">
         <x:v>peer_tid GPR</x:v>
       </x:c>
-      <x:c r="H106" s="78"/>
-      <x:c r="I106" s="78" t="str">
+      <x:c r="H104" s="78"/>
+      <x:c r="I104" s="78" t="str">
         <x:v>byte-preserving; source and destination descriptors must match</x:v>
       </x:c>
-      <x:c r="J106" s="83" t="str">
+      <x:c r="J104" s="83" t="str">
         <x:v>TLSU Function 13;</x:v>
       </x:c>
-      <x:c r="K106" s="90" t="str">
+      <x:c r="K104" s="90" t="str">
         <x:v>GMOV 是 DavinciOO v5 的 Core 内 PE 间 Local Tile 搬运扩展，公开接口为：</x:v>
       </x:c>
-      <x:c r="L106" s="91" t="str">
+      <x:c r="L104" s="91" t="str">
         <x:v>source/destination 必须是 descriptor-compatible ordinary Local Tile；同一物理输入输出采用 read-old/write-new。
 所有四个 PE 必须以相同动态顺序到达 collective；不收敛或 participant 不一致非法。
 SharedTile、Tile role 转换及跨 Core peer_tid 不受支持。
 逻辑 TileAcc role 仍映射到 ordinary physical TReg；GMOV 不访问任何 hidden accumulator state。</x:v>
       </x:c>
     </x:row>
-    <x:row r="107" ht="101" customHeight="1">
-      <x:c r="A107" s="124" t="str">
+    <x:row r="105" ht="101" customHeight="1">
+      <x:c r="A105" s="124" t="str">
         <x:v>Complex Layout Transformation
 复杂变换操作</x:v>
       </x:c>
-      <x:c r="B107" s="96" t="str">
+      <x:c r="B105" s="96" t="str">
         <x:v>Tile搬运</x:v>
       </x:c>
-      <x:c r="C107" s="73" t="str">
+      <x:c r="C105" s="73" t="str">
         <x:v>TMOV</x:v>
       </x:c>
-      <x:c r="D107" s="78" t="str">
+      <x:c r="D105" s="78" t="str">
         <x:v>BSTART.TLSU TMOV, DataType
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
-      <x:c r="E107" s="78" t="str">
+      <x:c r="E105" s="78" t="str">
         <x:v>destination Local or Shared Tile</x:v>
       </x:c>
-      <x:c r="F107" s="78" t="str">
+      <x:c r="F105" s="78" t="str">
         <x:v>source Local or Shared Tile</x:v>
       </x:c>
-      <x:c r="G107" s="78" t="str">
+      <x:c r="G105" s="78" t="str">
         <x:v>compile-time SharedMoveMode when Shared participates</x:v>
       </x:c>
-      <x:c r="H107" s="78"/>
-      <x:c r="I107" s="78" t="str">
+      <x:c r="H105" s="78"/>
+      <x:c r="I105" s="78" t="str">
         <x:v>byte-preserving; descriptors must be compatible</x:v>
       </x:c>
-      <x:c r="J107" s="83" t="str">
+      <x:c r="J105" s="83" t="str">
         <x:v>TLSU Function 2, Shared Functions 8–11;</x:v>
       </x:c>
-      <x:c r="K107" s="90" t="str">
+      <x:c r="K105" s="90" t="str">
         <x:v>Ordinary PTO TMOV(dst,src) remains a Local Tile move/conversion. DavinciOO v5 adds strongly typed Local↔Shared forms under the same intrinsic name; no _SHARED operation is introduced.</x:v>
       </x:c>
-      <x:c r="L107" s="91" t="str">
+      <x:c r="L105" s="91" t="str">
         <x:v>Shared→Shared TMOV is absent in v5; copy/transform through Local Tile.
 Runtime mode, owner or size is illegal.
 PE_MASK is a four-bit quarter predicate; multiple bits are allowed and
   0000 is a no-op.
 Absolute Shared registers are compiler-managed; C++ cannot specify Sx.
 RecordEvent is reused; there is no SharedEvent, and event completion is not a cross-PE GM fence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="101" customHeight="1">
+      <x:c r="A106" s="101" t="str">
+        <x:v>Tile Memory Operation
+Tile级访存操作</x:v>
+      </x:c>
+      <x:c r="B106" s="101" t="str">
+        <x:v>原子不规则访存</x:v>
+      </x:c>
+      <x:c r="C106" s="106" t="str">
+        <x:v>MGATHER_CAS</x:v>
+      </x:c>
+      <x:c r="D106" s="111" t="str">
+        <x:v>BSTART.MGATHER.CAS DataType
+B.IOT
+B.IOR base_address</x:v>
+      </x:c>
+      <x:c r="E106" s="111" t="str">
+        <x:v>old-value destination tile</x:v>
+      </x:c>
+      <x:c r="F106" s="111" t="str">
+        <x:v>base address
+indices tile</x:v>
+      </x:c>
+      <x:c r="G106" s="111" t="str">
+        <x:v>expected tile</x:v>
+      </x:c>
+      <x:c r="H106" s="111" t="str">
+        <x:v>replacement tile</x:v>
+      </x:c>
+      <x:c r="I106" s="111" t="str">
+        <x:v>TLSU atomic data types accepted by BSTART.MGATHER.CAS</x:v>
+      </x:c>
+      <x:c r="J106" s="116" t="str">
+        <x:v>TLSU Function 8;</x:v>
+      </x:c>
+      <x:c r="K106" s="120" t="str">
+        <x:v>MGATHER_CAS performs an atomic compare-and-swap for every indexed lane. The old memory value is always returned in the destination Tile. Memory is replaced only when the old value equals the lane's expected value, and an atomic event is recorded for both successful and failed comparisons.</x:v>
+      </x:c>
+      <x:c r="L106" s="121" t="str">
+        <x:v>Destination and index Tiles must have equal logical shape.
+Expected and replacement Tiles must match the destination shape and dtype.
+Read and write translation must resolve to the same address for each lane;
+  otherwise the operation raises a precise data-page fault.
+Each lane is an atomic read-modify-write using the current bundle memory-order
+  attribute. No stronger order between different lanes or PEs is guaranteed.
+BSTART.MGATHER.CAS is an accepted PTO ISA 0.58.0 command form.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="101" customHeight="1">
+      <x:c r="A107" s="101" t="str">
+        <x:v>Tile Memory Operation
+Tile级访存操作</x:v>
+      </x:c>
+      <x:c r="B107" s="101" t="str">
+        <x:v>不规则访存</x:v>
+      </x:c>
+      <x:c r="C107" s="106" t="str">
+        <x:v>MGATHER_MASK</x:v>
+      </x:c>
+      <x:c r="D107" s="111" t="str">
+        <x:v>BSTART.MGATHER.MASK DataType
+B.DATR PadValue (optional)
+B.IOT
+B.IOR base_address</x:v>
+      </x:c>
+      <x:c r="E107" s="111" t="str">
+        <x:v>destination tile</x:v>
+      </x:c>
+      <x:c r="F107" s="111" t="str">
+        <x:v>base address
+indices tile</x:v>
+      </x:c>
+      <x:c r="G107" s="111" t="str">
+        <x:v>mask tile</x:v>
+      </x:c>
+      <x:c r="H107" s="111" t="str">
+        <x:v>masked-off pad value</x:v>
+      </x:c>
+      <x:c r="I107" s="111" t="str">
+        <x:v>TLSU data types accepted by BSTART.MGATHER.MASK</x:v>
+      </x:c>
+      <x:c r="J107" s="116" t="str">
+        <x:v>TLSU Function 6;</x:v>
+      </x:c>
+      <x:c r="K107" s="120" t="str">
+        <x:v>MGATHER_MASK gathers indexed memory elements for nonzero mask lanes. A zero mask lane performs no memory access and writes the current bundle pad value to the corresponding destination element. All selected addresses are probed before any load event or destination update, preserving precise faults.</x:v>
+      </x:c>
+      <x:c r="L107" s="121" t="str">
+        <x:v>Destination, index, and mask Tiles must have equal logical shape.
+Index and mask contents must be defined before execution.
+Masked-off lanes do not access memory; selected lanes use the current bundle
+  memory-order attribute.
+BSTART.MGATHER.MASK is an accepted PTO ISA 0.58.0 command form, not a
+  future-reserved encoding.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="101" customHeight="1">
+      <x:c r="A108" s="101" t="str">
+        <x:v>Tile Memory Operation
+Tile级访存操作</x:v>
+      </x:c>
+      <x:c r="B108" s="101" t="str">
+        <x:v>不规则访存</x:v>
+      </x:c>
+      <x:c r="C108" s="106" t="str">
+        <x:v>MSCATTER_MASK</x:v>
+      </x:c>
+      <x:c r="D108" s="111" t="str">
+        <x:v>BSTART.MSCATTER.MASK DataType
+B.IOT
+B.IOR base_address</x:v>
+      </x:c>
+      <x:c r="E108" s="111" t="str">
+        <x:v>indexed memory locations</x:v>
+      </x:c>
+      <x:c r="F108" s="111" t="str">
+        <x:v>source tile
+indices tile</x:v>
+      </x:c>
+      <x:c r="G108" s="111" t="str">
+        <x:v>mask tile</x:v>
+      </x:c>
+      <x:c r="H108" s="111"/>
+      <x:c r="I108" s="111" t="str">
+        <x:v>TLSU data types accepted by BSTART.MSCATTER.MASK</x:v>
+      </x:c>
+      <x:c r="J108" s="116" t="str">
+        <x:v>TLSU Function 7;</x:v>
+      </x:c>
+      <x:c r="K108" s="120" t="str">
+        <x:v>MSCATTER_MASK scatters source elements to indexed memory locations for nonzero mask lanes. Zero mask lanes have no memory side effect. All selected addresses are probed before the scatter commit phase so a failing footprint does not produce a partial event prefix.</x:v>
+      </x:c>
+      <x:c r="L108" s="121" t="str">
+        <x:v>Source, index, and mask Tiles must have equal logical shape and defined
+  contents.
+Selected lanes obey the current bundle memory-order attribute.
+Conflicting selected addresses follow the architectural scatter commit
+  policy; programmers must not infer a stronger lane order.
+BSTART.MSCATTER.MASK is an accepted PTO ISA 0.58.0 command form.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="101" customHeight="1">
+      <x:c r="A109" s="127" t="str">
+        <x:v>Complex Layout Transformation
+复杂变换操作</x:v>
+      </x:c>
+      <x:c r="B109" s="101" t="str">
+        <x:v>直方图</x:v>
+      </x:c>
+      <x:c r="C109" s="106" t="str">
+        <x:v>THISTOGRAM</x:v>
+      </x:c>
+      <x:c r="D109" s="111" t="str">
+        <x:v>BSTART.TEPL THISTOGRAM, DataType
+B.DATR selected_byte
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E109" s="111" t="str">
+        <x:v>per-row cumulative 256-bin histogram</x:v>
+      </x:c>
+      <x:c r="F109" s="111" t="str">
+        <x:v>U16 or U32 source tile</x:v>
+      </x:c>
+      <x:c r="G109" s="111" t="str">
+        <x:v>filter/index tile</x:v>
+      </x:c>
+      <x:c r="H109" s="111" t="str">
+        <x:v>selected_byte 0..3</x:v>
+      </x:c>
+      <x:c r="I109" s="111" t="str">
+        <x:v>source: U16, U32</x:v>
+      </x:c>
+      <x:c r="J109" s="116" t="str">
+        <x:v>TEPL Mode 3, Function 8, TileOp 0x68;</x:v>
+      </x:c>
+      <x:c r="K109" s="120" t="str">
+        <x:v>THISTOGRAM selects one byte from each U16 or U32 source element, optionally filters higher bytes through the index Tile, counts 256 byte values per row, and writes the cumulative bin counts to the destination. selected_byte is encoded through the B.DATR.PadValueOrByteId union for this operation.</x:v>
+      </x:c>
+      <x:c r="L109" s="121" t="str">
+        <x:v>Destination and source row counts must match; destination valid columns must
+  be at least 256.
+U16 sources allow byte 0 or 1. U32 sources allow byte 0 through 3.
+The index Tile must supply the filter rows required by the selected byte.
+The destination valid region becomes defined after successful completion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="101" customHeight="1">
+      <x:c r="A110" s="127" t="str">
+        <x:v>Complex Layout Transformation
+复杂变换操作</x:v>
+      </x:c>
+      <x:c r="B110" s="101" t="str">
+        <x:v>排序</x:v>
+      </x:c>
+      <x:c r="C110" s="106" t="str">
+        <x:v>TSORT</x:v>
+      </x:c>
+      <x:c r="D110" s="111" t="str">
+        <x:v>BSTART.TEPL TSORT, DataType
+B.DIM sort_width -&gt; LB0
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E110" s="111" t="str">
+        <x:v>sorted values tile
+original-index U32 tile</x:v>
+      </x:c>
+      <x:c r="F110" s="111" t="str">
+        <x:v>source values tile</x:v>
+      </x:c>
+      <x:c r="G110" s="111" t="str">
+        <x:v>sort_width 1..64</x:v>
+      </x:c>
+      <x:c r="H110" s="111" t="str">
+        <x:v>descending control</x:v>
+      </x:c>
+      <x:c r="I110" s="111" t="str">
+        <x:v>values: source/destination dtype match, indices: U32</x:v>
+      </x:c>
+      <x:c r="J110" s="116" t="str">
+        <x:v>TEPL Mode 3, Function 12, TileOp 0x6C;</x:v>
+      </x:c>
+      <x:c r="K110" s="120" t="str">
+        <x:v>TSORT sorts each consecutive group of sort_width elements from the source Tile, writes the ordered values to destination0, and writes each value's original group-relative index to the U32 destination1 Tile. sort_width is in 1..64; the canonical bundle decoder obtains it from LB0 and defaults to 32 when no nonzero width is supplied. The semantic descending operand selects ascending or descending order; the current PTO block transport supplies the operation default (false, ascending).</x:v>
+      </x:c>
+      <x:c r="L110" s="121" t="str">
+        <x:v>The two destinations must be distinct and must have the same element count
+  as the source.
+The values destination dtype must equal the source dtype; the index
+  destination dtype is U32.
+Sorting is stable only where the selected numeric profile defines equal-value
+  ordering; no memory or cross-PE ordering is implied.
+TSORT32 is not an ISA identity in PTO ISA 0.58.0. It is replaced by
+  TSORT with explicit sort_width; the old PTO source page is retained only
+  as provenance for the operation family.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7320,7 +7435,7 @@
     <x:mergeCell ref="A52:A67"/>
     <x:mergeCell ref="A68:A75"/>
     <x:mergeCell ref="A76:A80"/>
-    <x:mergeCell ref="A81:A101"/>
+    <x:mergeCell ref="A81:A99"/>
     <x:mergeCell ref="B2:B6"/>
     <x:mergeCell ref="B8:B14"/>
     <x:mergeCell ref="B15:B18"/>
@@ -7335,10 +7450,10 @@
     <x:mergeCell ref="B72:B75"/>
     <x:mergeCell ref="B76:B78"/>
     <x:mergeCell ref="B79:B80"/>
-    <x:mergeCell ref="B81:B85"/>
-    <x:mergeCell ref="B86:B88"/>
-    <x:mergeCell ref="B89:B95"/>
-    <x:mergeCell ref="B98:B101"/>
+    <x:mergeCell ref="B81:B84"/>
+    <x:mergeCell ref="B85:B87"/>
+    <x:mergeCell ref="B88:B94"/>
+    <x:mergeCell ref="B96:B99"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7354,106 +7469,106 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>471</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>472</x:v>
+        <x:v>455</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26.399999618530273" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>473</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>474</x:v>
+        <x:v>457</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="26.399999618530273" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>475</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>476</x:v>
+        <x:v>459</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" customHeight="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>477</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>478</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.399999618530273" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>479</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>480</x:v>
+        <x:v>463</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>481</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>482</x:v>
+        <x:v>465</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>483</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>484</x:v>
+        <x:v>467</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>485</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>486</x:v>
+        <x:v>469</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>487</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>488</x:v>
+        <x:v>471</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40.5" customHeight="1">
       <x:c r="A10" s="3" t="s">
-        <x:v>489</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
-        <x:v>490</x:v>
+        <x:v>473</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40.5" customHeight="1">
       <x:c r="A11" s="3" t="s">
-        <x:v>491</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>475</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40.5" customHeight="1">
       <x:c r="A12" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>477</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="40.5" customHeight="1">
       <x:c r="A13" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
-        <x:v>496</x:v>
+        <x:v>479</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7471,98 +7586,98 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>497</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>498</x:v>
+        <x:v>481</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="14" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>499</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>500</x:v>
+        <x:v>483</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="14" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>501</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>502</x:v>
+        <x:v>485</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="14" customHeight="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>503</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>504</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="14" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>505</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>506</x:v>
+        <x:v>489</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="14" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>507</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>508</x:v>
+        <x:v>491</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>509</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>510</x:v>
+        <x:v>493</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="14" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>511</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>512</x:v>
+        <x:v>495</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="14" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>513</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>514</x:v>
+        <x:v>497</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="14" customHeight="1">
       <x:c r="A10" s="2" t="s">
-        <x:v>515</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
-        <x:v>516</x:v>
+        <x:v>499</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="14" customHeight="1">
       <x:c r="A11" s="2" t="s">
-        <x:v>517</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>518</x:v>
+        <x:v>501</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="14" customHeight="1">
       <x:c r="A12" s="2" t="s">
-        <x:v>519</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>520</x:v>
+        <x:v>503</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Align PTO ISA 0.58 retained operations (#46)
Align the PTO ISA 0.58 catalog with the reviewed retained operation set
and Shared tile contract.\n\n- restore BSTART.MGATHER.MASK,
BSTART.MSCATTER.MASK, and BSTART.MGATHER.CAS\n- restore THISTOGRAM,
retain TSORT with explicit sort_width, and reserve the removed TRANDOM
selector\n- rename the direct memory family from TMA to TLSU\n- move
Shared TLSU variants after retained Functions 6 through 8\n- preserve
exact 474-form scalar ABI and clarify scalar count terminology\n-
regenerate ASL decoders, references, evidence, and release
identity\n\nLocal verification: repo-check, release-check, binary
closure, ASL shard checks, scalar-base, scalar-alu-bru, tile operations,
TEPL totality, TLSU totality, CUBE totality, and focused Shared TLSU
execution.

---------

Co-authored-by: Codex Review <codex-review@example.invalid>
</commit_message>
<xml_diff>
--- a/spec/encoding/PTO-ISA-Encoding.xlsx
+++ b/spec/encoding/PTO-ISA-Encoding.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6f8d8ab6d45b4199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rce61c905a5d940fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R691a09b226ca4fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R77efea90e68d4cb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rd5d2a39aebb44e71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="Rfc64d61f63034444"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1134,32 +1134,6 @@
 3. Destination layout restrictions are target/profile-defined; some targets require row-major dst.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">TRANDOM</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">dst random tile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TRandomKey via B.IOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TRandomCounter via B.IOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">S32, U32</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TEPL Mode 3, Function 9, TileOp 0x69;</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Generate counter-based pseudo-random values into dst.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1. A5 dst dtype must be S32 or U32 and dst must be row-major.
-2. Rounds must be 7 or 10; default is 10.
-3. Key and counter operands must be valid and non-null.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">TFILLPAD</x:t>
   </x:si>
   <x:si>
@@ -1403,35 +1377,6 @@
     <x:t xml:space="preserve">1. Supported tile types, layout, padding, repeat, and config fields are target/implementation-defined.
 2. posM/posK select the convolution window position consumed by the opcode profile.
 3. A2/A3 and A5 differ in how img2col repeat/padding state is configured.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">排序</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TSORT32</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">dst sorted value/index pairs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">src value tile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">idx tile</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">values: F16, F32; idx: U32</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TEPL Mode 3, Function 12, TileOp 0x6C;</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sort each 32-element block and carry indices along with values.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1. TSORT32 does not take WaitEvents and does not implicitly call TSYNC.
-2. dst/src value dtype must be F16 or F32; idx dtype must be U32.
-3. dst/src/idx must be Vec row-major; sorting is independent per 32-element block.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TMRGSORT</x:t>
@@ -2339,7 +2284,7 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="125">
+  <x:cellXfs count="128">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -2713,6 +2658,15 @@
       <x:alignment horizontal="center" vertical="top"/>
     </x:xf>
     <x:xf fontId="3" borderId="23" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="3" fillId="0" borderId="23" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf fontId="3" fillId="0" borderId="23" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top"/>
+    </x:xf>
+    <x:xf fontId="3" fillId="0" borderId="23" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -6049,7 +6003,7 @@
 C.B.IOS
 B.IOR
 Shared pe_scope form
-BSTART.TLSU Function 12
+BSTART.TLSU Function 14
 C.B.IOS
 B.IOR</x:v>
       </x:c>
@@ -6071,7 +6025,7 @@
         <x:v>PTO TSTORE dtype/layout combinations supported by the v5 TLSU profile</x:v>
       </x:c>
       <x:c r="J77" s="41" t="str">
-        <x:v>TLSU Function 1; Shared pe_scope Function 12;</x:v>
+        <x:v>TLSU Function 1; Shared pe_scope Function 14;</x:v>
       </x:c>
       <x:c r="K77" s="2" t="s">
         <x:v>313</x:v>
@@ -6306,184 +6260,186 @@
         <x:v>358</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" ht="101">
+    <x:row r="84" ht="84.75">
       <x:c r="A84" s="53"/>
-      <x:c r="B84" s="54"/>
-      <x:c r="C84" s="16" t="s">
+      <x:c r="B84" s="55"/>
+      <x:c r="C84" s="24" t="s">
         <x:v>359</x:v>
       </x:c>
-      <x:c r="D84" s="17" t="str">
-        <x:v>BSTART.TEPL TRANDOM, DataType
+      <x:c r="D84" s="25" t="str">
+        <x:v>BSTART.TEPL TFILLPAD, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E84" s="25" t="s">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="F84" s="25" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G84" s="25" t="s">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="H84" s="25"/>
+      <x:c r="I84" s="25" t="s">
+        <x:v>362</x:v>
+      </x:c>
+      <x:c r="J84" s="43" t="s">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="K84" s="2" t="s">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="L84" s="3" t="s">
+        <x:v>365</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="118">
+      <x:c r="A85" s="53"/>
+      <x:c r="B85" s="52" t="s">
+        <x:v>366</x:v>
+      </x:c>
+      <x:c r="C85" s="13" t="s">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="D85" s="17" t="str">
+        <x:v>BSTART.TEPL TCVT, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E85" s="17" t="s">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="F85" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G85" s="17" t="s">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="H85" s="17"/>
+      <x:c r="I85" s="17" t="s">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="J85" s="41" t="s">
+        <x:v>371</x:v>
+      </x:c>
+      <x:c r="K85" s="2" t="s">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="L85" s="3" t="s">
+        <x:v>373</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="84">
+      <x:c r="A86" s="53"/>
+      <x:c r="B86" s="54"/>
+      <x:c r="C86" s="16" t="s">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="D86" s="17" t="str">
+        <x:v>BSTART.TEPL TQUANT, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E86" s="17" t="s">
+        <x:v>375</x:v>
+      </x:c>
+      <x:c r="F86" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G86" s="17" t="s">
+        <x:v>376</x:v>
+      </x:c>
+      <x:c r="H86" s="17" t="str">
+        <x:v>offset/scaling/index Tile (optional)</x:v>
+      </x:c>
+      <x:c r="I86" s="17" t="s">
+        <x:v>377</x:v>
+      </x:c>
+      <x:c r="J86" s="41" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="K86" s="2" t="s">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="L86" s="3" t="s">
+        <x:v>380</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="84.75">
+      <x:c r="A87" s="53"/>
+      <x:c r="B87" s="55"/>
+      <x:c r="C87" s="16" t="s">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="D87" s="17" t="str">
+        <x:v>BSTART.TEPL TDEQUANT, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E87" s="17" t="s">
+        <x:v>382</x:v>
+      </x:c>
+      <x:c r="F87" s="17" t="s">
+        <x:v>383</x:v>
+      </x:c>
+      <x:c r="G87" s="17" t="s">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="H87" s="17" t="s">
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="I87" s="17" t="s">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="J87" s="41" t="s">
+        <x:v>387</x:v>
+      </x:c>
+      <x:c r="K87" s="2" t="s">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="L87" s="3" t="s">
+        <x:v>389</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="101">
+      <x:c r="A88" s="53"/>
+      <x:c r="B88" s="52" t="s">
+        <x:v>390</x:v>
+      </x:c>
+      <x:c r="C88" s="56" t="s">
+        <x:v>391</x:v>
+      </x:c>
+      <x:c r="D88" s="56" t="str">
+        <x:v>BSTART.TEPL TEXTRACT, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT
 B.IOR</x:v>
       </x:c>
-      <x:c r="E84" s="17" t="s">
-        <x:v>360</x:v>
-      </x:c>
-      <x:c r="F84" s="17" t="s">
-        <x:v>361</x:v>
-      </x:c>
-      <x:c r="G84" s="17" t="s">
-        <x:v>362</x:v>
-      </x:c>
-      <x:c r="H84" s="17"/>
-      <x:c r="I84" s="17" t="s">
-        <x:v>363</x:v>
-      </x:c>
-      <x:c r="J84" s="41" t="s">
-        <x:v>364</x:v>
-      </x:c>
-      <x:c r="K84" s="2" t="s">
-        <x:v>365</x:v>
-      </x:c>
-      <x:c r="L84" s="3" t="s">
-        <x:v>366</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="85" ht="84.75">
-      <x:c r="A85" s="53"/>
-      <x:c r="B85" s="55"/>
-      <x:c r="C85" s="24" t="s">
-        <x:v>367</x:v>
-      </x:c>
-      <x:c r="D85" s="25" t="str">
-        <x:v>BSTART.TEPL TFILLPAD, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E85" s="25" t="s">
-        <x:v>368</x:v>
-      </x:c>
-      <x:c r="F85" s="25" t="s">
+      <x:c r="E88" s="9" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="F88" s="9" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="G85" s="25" t="s">
-        <x:v>369</x:v>
-      </x:c>
-      <x:c r="H85" s="25"/>
-      <x:c r="I85" s="25" t="s">
-        <x:v>370</x:v>
-      </x:c>
-      <x:c r="J85" s="43" t="s">
-        <x:v>371</x:v>
-      </x:c>
-      <x:c r="K85" s="2" t="s">
-        <x:v>372</x:v>
-      </x:c>
-      <x:c r="L85" s="3" t="s">
-        <x:v>373</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="86" ht="118">
-      <x:c r="A86" s="53"/>
-      <x:c r="B86" s="52" t="s">
-        <x:v>374</x:v>
-      </x:c>
-      <x:c r="C86" s="13" t="s">
-        <x:v>375</x:v>
-      </x:c>
-      <x:c r="D86" s="17" t="str">
-        <x:v>BSTART.TEPL TCVT, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E86" s="17" t="s">
-        <x:v>376</x:v>
-      </x:c>
-      <x:c r="F86" s="17" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="G86" s="17" t="s">
-        <x:v>377</x:v>
-      </x:c>
-      <x:c r="H86" s="17"/>
-      <x:c r="I86" s="17" t="s">
-        <x:v>378</x:v>
-      </x:c>
-      <x:c r="J86" s="41" t="s">
-        <x:v>379</x:v>
-      </x:c>
-      <x:c r="K86" s="2" t="s">
-        <x:v>380</x:v>
-      </x:c>
-      <x:c r="L86" s="3" t="s">
-        <x:v>381</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="87" ht="84">
-      <x:c r="A87" s="53"/>
-      <x:c r="B87" s="54"/>
-      <x:c r="C87" s="16" t="s">
-        <x:v>382</x:v>
-      </x:c>
-      <x:c r="D87" s="17" t="str">
-        <x:v>BSTART.TEPL TQUANT, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E87" s="17" t="s">
-        <x:v>383</x:v>
-      </x:c>
-      <x:c r="F87" s="17" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="G87" s="17" t="s">
-        <x:v>384</x:v>
-      </x:c>
-      <x:c r="H87" s="17" t="str">
-        <x:v>offset/scaling/index Tile (optional)</x:v>
-      </x:c>
-      <x:c r="I87" s="17" t="s">
-        <x:v>385</x:v>
-      </x:c>
-      <x:c r="J87" s="41" t="s">
-        <x:v>386</x:v>
-      </x:c>
-      <x:c r="K87" s="2" t="s">
-        <x:v>387</x:v>
-      </x:c>
-      <x:c r="L87" s="3" t="s">
-        <x:v>388</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="88" ht="84.75">
-      <x:c r="A88" s="53"/>
-      <x:c r="B88" s="55"/>
-      <x:c r="C88" s="16" t="s">
-        <x:v>389</x:v>
-      </x:c>
-      <x:c r="D88" s="17" t="str">
-        <x:v>BSTART.TEPL TDEQUANT, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E88" s="17" t="s">
-        <x:v>390</x:v>
-      </x:c>
-      <x:c r="F88" s="17" t="s">
-        <x:v>391</x:v>
-      </x:c>
-      <x:c r="G88" s="17" t="s">
-        <x:v>392</x:v>
-      </x:c>
-      <x:c r="H88" s="17" t="s">
+      <x:c r="G88" s="9" t="s">
         <x:v>393</x:v>
       </x:c>
-      <x:c r="I88" s="17" t="s">
+      <x:c r="H88" s="9"/>
+      <x:c r="I88" s="9" t="s">
         <x:v>394</x:v>
       </x:c>
-      <x:c r="J88" s="41" t="s">
+      <x:c r="J88" s="40" t="s">
         <x:v>395</x:v>
       </x:c>
       <x:c r="K88" s="2" t="s">
@@ -6495,230 +6451,228 @@
     </x:row>
     <x:row r="89" ht="101">
       <x:c r="A89" s="53"/>
-      <x:c r="B89" s="52" t="s">
+      <x:c r="B89" s="54"/>
+      <x:c r="C89" s="57" t="s">
         <x:v>398</x:v>
       </x:c>
-      <x:c r="C89" s="56" t="s">
-        <x:v>399</x:v>
-      </x:c>
-      <x:c r="D89" s="56" t="str">
-        <x:v>BSTART.TEPL TEXTRACT, DataType
+      <x:c r="D89" s="57" t="str">
+        <x:v>BSTART.TEPL TINSERT, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT
 B.IOR</x:v>
       </x:c>
-      <x:c r="E89" s="9" t="s">
+      <x:c r="E89" s="17" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F89" s="17" t="s">
+        <x:v>399</x:v>
+      </x:c>
+      <x:c r="G89" s="17" t="s">
+        <x:v>393</x:v>
+      </x:c>
+      <x:c r="H89" s="17"/>
+      <x:c r="I89" s="17" t="s">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="F89" s="9" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="G89" s="9" t="s">
+      <x:c r="J89" s="41" t="s">
         <x:v>401</x:v>
       </x:c>
-      <x:c r="H89" s="9"/>
-      <x:c r="I89" s="9" t="s">
+      <x:c r="K89" s="2" t="s">
         <x:v>402</x:v>
       </x:c>
-      <x:c r="J89" s="40" t="s">
+      <x:c r="L89" s="3" t="s">
         <x:v>403</x:v>
-      </x:c>
-      <x:c r="K89" s="2" t="s">
-        <x:v>404</x:v>
-      </x:c>
-      <x:c r="L89" s="3" t="s">
-        <x:v>405</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="101">
       <x:c r="A90" s="53"/>
       <x:c r="B90" s="54"/>
       <x:c r="C90" s="57" t="s">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="D90" s="57" t="str">
+        <x:v>BSTART.TEPL TGATHER, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E90" s="17" t="s">
+        <x:v>405</x:v>
+      </x:c>
+      <x:c r="F90" s="17" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G90" s="17" t="s">
         <x:v>406</x:v>
-      </x:c>
-      <x:c r="D90" s="57" t="str">
-        <x:v>BSTART.TEPL TINSERT, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT
-B.IOR</x:v>
-      </x:c>
-      <x:c r="E90" s="17" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F90" s="17" t="s">
-        <x:v>407</x:v>
-      </x:c>
-      <x:c r="G90" s="17" t="s">
-        <x:v>401</x:v>
       </x:c>
       <x:c r="H90" s="17"/>
       <x:c r="I90" s="17" t="s">
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="J90" s="41" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="J90" s="41" t="s">
+      <x:c r="K90" s="2" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="K90" s="2" t="s">
+      <x:c r="L90" s="3" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="L90" s="3" t="s">
-        <x:v>411</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91" ht="101">
+    </x:row>
+    <x:row r="91" ht="84">
       <x:c r="A91" s="53"/>
       <x:c r="B91" s="54"/>
       <x:c r="C91" s="57" t="s">
+        <x:v>411</x:v>
+      </x:c>
+      <x:c r="D91" s="57" t="str">
+        <x:v>BSTART.TEPL TSCATTER, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E91" s="17" t="s">
         <x:v>412</x:v>
-      </x:c>
-      <x:c r="D91" s="57" t="str">
-        <x:v>BSTART.TEPL TGATHER, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E91" s="17" t="s">
-        <x:v>413</x:v>
       </x:c>
       <x:c r="F91" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G91" s="17" t="s">
-        <x:v>414</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="H91" s="17"/>
       <x:c r="I91" s="17" t="s">
+        <x:v>414</x:v>
+      </x:c>
+      <x:c r="J91" s="41" t="s">
         <x:v>415</x:v>
       </x:c>
-      <x:c r="J91" s="41" t="s">
+      <x:c r="K91" s="2" t="s">
         <x:v>416</x:v>
       </x:c>
-      <x:c r="K91" s="2" t="s">
+      <x:c r="L91" s="3" t="s">
         <x:v>417</x:v>
-      </x:c>
-      <x:c r="L91" s="3" t="s">
-        <x:v>418</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="84">
       <x:c r="A92" s="53"/>
       <x:c r="B92" s="54"/>
       <x:c r="C92" s="57" t="s">
-        <x:v>419</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="D92" s="57" t="str">
-        <x:v>BSTART.TEPL TSCATTER, DataType
+        <x:v>BSTART.TEPL TCONCAT, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
       <x:c r="E92" s="17" t="s">
-        <x:v>420</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F92" s="17" t="s">
-        <x:v>74</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G92" s="17" t="s">
-        <x:v>421</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H92" s="17"/>
       <x:c r="I92" s="17" t="s">
-        <x:v>422</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="J92" s="41" t="s">
-        <x:v>423</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="K92" s="2" t="s">
-        <x:v>424</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="L92" s="3" t="s">
-        <x:v>425</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="84">
       <x:c r="A93" s="53"/>
       <x:c r="B93" s="54"/>
       <x:c r="C93" s="57" t="s">
-        <x:v>426</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="D93" s="57" t="str">
-        <x:v>BSTART.TEPL TCONCAT, DataType
+        <x:v>BSTART.TEPL TTRANS, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
       <x:c r="E93" s="17" t="s">
-        <x:v>15</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="F93" s="17" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G93" s="17" t="s">
-        <x:v>17</x:v>
-      </x:c>
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G93" s="17"/>
       <x:c r="H93" s="17"/>
       <x:c r="I93" s="17" t="s">
-        <x:v>18</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="J93" s="41" t="s">
+        <x:v>424</x:v>
+      </x:c>
+      <x:c r="K93" s="2" t="s">
+        <x:v>425</x:v>
+      </x:c>
+      <x:c r="L93" s="3" t="s">
+        <x:v>426</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="101.75">
+      <x:c r="A94" s="53"/>
+      <x:c r="B94" s="55"/>
+      <x:c r="C94" s="58" t="s">
         <x:v>427</x:v>
       </x:c>
-      <x:c r="K93" s="2" t="s">
+      <x:c r="D94" s="58" t="str">
+        <x:v>BSTART.TEPL TIMG2COL, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT
+B.IOR</x:v>
+      </x:c>
+      <x:c r="E94" s="25" t="s">
         <x:v>428</x:v>
       </x:c>
-      <x:c r="L93" s="3" t="s">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="94" ht="84">
-      <x:c r="A94" s="53"/>
-      <x:c r="B94" s="54"/>
-      <x:c r="C94" s="57" t="s">
+      <x:c r="F94" s="25" t="s">
         <x:v>429</x:v>
       </x:c>
-      <x:c r="D94" s="57" t="str">
-        <x:v>BSTART.TEPL TTRANS, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E94" s="17" t="s">
+      <x:c r="G94" s="25" t="s">
         <x:v>430</x:v>
       </x:c>
-      <x:c r="F94" s="17" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="G94" s="17"/>
-      <x:c r="H94" s="17"/>
-      <x:c r="I94" s="17" t="s">
+      <x:c r="H94" s="25"/>
+      <x:c r="I94" s="25" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="J94" s="43" t="s">
         <x:v>431</x:v>
       </x:c>
-      <x:c r="J94" s="41" t="s">
+      <x:c r="K94" s="2" t="s">
         <x:v>432</x:v>
       </x:c>
-      <x:c r="K94" s="2" t="s">
+      <x:c r="L94" s="3" t="s">
         <x:v>433</x:v>
-      </x:c>
-      <x:c r="L94" s="3" t="s">
-        <x:v>434</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="101.75">
       <x:c r="A95" s="53"/>
       <x:c r="B95" s="55"/>
-      <x:c r="C95" s="58" t="s">
-        <x:v>435</x:v>
+      <x:c r="C95" s="43" t="s">
+        <x:v>434</x:v>
       </x:c>
       <x:c r="D95" s="58" t="str">
-        <x:v>BSTART.TEPL TIMG2COL, DataType
+        <x:v>BSTART.TEPL TMRGSORT, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
@@ -6726,261 +6680,186 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E95" s="25" t="s">
+        <x:v>435</x:v>
+      </x:c>
+      <x:c r="F95" s="25" t="s">
         <x:v>436</x:v>
       </x:c>
-      <x:c r="F95" s="25" t="s">
+      <x:c r="G95" s="25" t="s">
         <x:v>437</x:v>
-      </x:c>
-      <x:c r="G95" s="25" t="s">
-        <x:v>438</x:v>
       </x:c>
       <x:c r="H95" s="25"/>
       <x:c r="I95" s="25" t="s">
-        <x:v>223</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="J95" s="43" t="s">
+        <x:v>438</x:v>
+      </x:c>
+      <x:c r="K95" s="2" t="s">
         <x:v>439</x:v>
       </x:c>
-      <x:c r="K95" s="2" t="s">
+      <x:c r="L95" s="3" t="s">
         <x:v>440</x:v>
-      </x:c>
-      <x:c r="L95" s="3" t="s">
-        <x:v>441</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="84">
       <x:c r="A96" s="53"/>
       <x:c r="B96" s="52" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="C96" s="40" t="s">
         <x:v>442</x:v>
       </x:c>
-      <x:c r="C96" s="40" t="s">
-        <x:v>443</x:v>
-      </x:c>
       <x:c r="D96" s="56" t="str">
-        <x:v>BSTART.TEPL TSORT32, DataType
+        <x:v>BSTART.TEPL TPARTADD, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
       <x:c r="E96" s="9" t="s">
-        <x:v>444</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F96" s="9" t="s">
-        <x:v>445</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G96" s="9" t="s">
-        <x:v>446</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H96" s="9"/>
       <x:c r="I96" s="9" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="J96" s="40" t="s">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="K96" s="2" t="s">
+        <x:v>444</x:v>
+      </x:c>
+      <x:c r="L96" s="3" t="s">
+        <x:v>26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="84">
+      <x:c r="A97" s="53"/>
+      <x:c r="B97" s="54"/>
+      <x:c r="C97" s="41" t="s">
+        <x:v>445</x:v>
+      </x:c>
+      <x:c r="D97" s="57" t="str">
+        <x:v>BSTART.TEPL TPARTMUL, DataType
+B.DATR (optional)
+B.DIM LB0
+B.DIM (LB1/LB2 for 2D)
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E97" s="17" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F97" s="17" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G97" s="17" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H97" s="17"/>
+      <x:c r="I97" s="17" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J97" s="41" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="K97" s="2" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="J96" s="40" t="s">
-        <x:v>448</x:v>
-      </x:c>
-      <x:c r="K96" s="2" t="s">
-        <x:v>449</x:v>
-      </x:c>
-      <x:c r="L96" s="3" t="s">
-        <x:v>450</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="97" ht="101.75">
-      <x:c r="A97" s="53"/>
-      <x:c r="B97" s="55"/>
-      <x:c r="C97" s="43" t="s">
-        <x:v>451</x:v>
-      </x:c>
-      <x:c r="D97" s="58" t="str">
-        <x:v>BSTART.TEPL TMRGSORT, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT
-B.IOR</x:v>
-      </x:c>
-      <x:c r="E97" s="25" t="s">
-        <x:v>452</x:v>
-      </x:c>
-      <x:c r="F97" s="25" t="s">
-        <x:v>453</x:v>
-      </x:c>
-      <x:c r="G97" s="25" t="s">
-        <x:v>454</x:v>
-      </x:c>
-      <x:c r="H97" s="25"/>
-      <x:c r="I97" s="25" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="J97" s="43" t="s">
-        <x:v>455</x:v>
-      </x:c>
-      <x:c r="K97" s="2" t="s">
-        <x:v>456</x:v>
-      </x:c>
       <x:c r="L97" s="3" t="s">
-        <x:v>457</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="84">
       <x:c r="A98" s="53"/>
-      <x:c r="B98" s="52" t="s">
-        <x:v>458</x:v>
-      </x:c>
-      <x:c r="C98" s="40" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="D98" s="56" t="str">
-        <x:v>BSTART.TEPL TPARTADD, DataType
+      <x:c r="B98" s="54"/>
+      <x:c r="C98" s="41" t="s">
+        <x:v>448</x:v>
+      </x:c>
+      <x:c r="D98" s="57" t="str">
+        <x:v>BSTART.TEPL TPARTMAX, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
-      <x:c r="E98" s="9" t="s">
+      <x:c r="E98" s="17" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F98" s="9" t="s">
+      <x:c r="F98" s="17" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G98" s="9" t="s">
+      <x:c r="G98" s="17" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H98" s="9"/>
-      <x:c r="I98" s="9" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="J98" s="40" t="s">
-        <x:v>460</x:v>
+      <x:c r="H98" s="17"/>
+      <x:c r="I98" s="17" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="J98" s="41" t="s">
+        <x:v>449</x:v>
       </x:c>
       <x:c r="K98" s="2" t="s">
-        <x:v>461</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="L98" s="3" t="s">
         <x:v>26</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" ht="84">
-      <x:c r="A99" s="53"/>
-      <x:c r="B99" s="54"/>
-      <x:c r="C99" s="41" t="s">
-        <x:v>462</x:v>
-      </x:c>
-      <x:c r="D99" s="57" t="str">
-        <x:v>BSTART.TEPL TPARTMUL, DataType
+    <x:row r="99" ht="84.75">
+      <x:c r="A99" s="59"/>
+      <x:c r="B99" s="55"/>
+      <x:c r="C99" s="43" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="D99" s="58" t="str">
+        <x:v>BSTART.TEPL TPARTMIN, DataType
 B.DATR (optional)
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
-      <x:c r="E99" s="17" t="s">
+      <x:c r="E99" s="25" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F99" s="17" t="s">
+      <x:c r="F99" s="25" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G99" s="17" t="s">
+      <x:c r="G99" s="25" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H99" s="17"/>
-      <x:c r="I99" s="17" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="J99" s="41" t="s">
-        <x:v>463</x:v>
+      <x:c r="H99" s="25"/>
+      <x:c r="I99" s="25" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="J99" s="43" t="s">
+        <x:v>452</x:v>
       </x:c>
       <x:c r="K99" s="2" t="s">
-        <x:v>464</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="L99" s="3" t="s">
         <x:v>26</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" ht="84">
-      <x:c r="A100" s="53"/>
-      <x:c r="B100" s="54"/>
-      <x:c r="C100" s="41" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="D100" s="57" t="str">
-        <x:v>BSTART.TEPL TPARTMAX, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E100" s="17" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F100" s="17" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G100" s="17" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H100" s="17"/>
-      <x:c r="I100" s="17" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="J100" s="41" t="s">
-        <x:v>466</x:v>
-      </x:c>
-      <x:c r="K100" s="2" t="s">
-        <x:v>467</x:v>
-      </x:c>
-      <x:c r="L100" s="3" t="s">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="101" ht="84.75">
-      <x:c r="A101" s="59"/>
-      <x:c r="B101" s="55"/>
-      <x:c r="C101" s="43" t="s">
-        <x:v>468</x:v>
-      </x:c>
-      <x:c r="D101" s="58" t="str">
-        <x:v>BSTART.TEPL TPARTMIN, DataType
-B.DATR (optional)
-B.DIM LB0
-B.DIM (LB1/LB2 for 2D)
-B.IOT</x:v>
-      </x:c>
-      <x:c r="E101" s="25" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F101" s="25" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G101" s="25" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H101" s="25"/>
-      <x:c r="I101" s="25" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="J101" s="43" t="s">
-        <x:v>469</x:v>
-      </x:c>
-      <x:c r="K101" s="2" t="s">
-        <x:v>470</x:v>
-      </x:c>
-      <x:c r="L101" s="3" t="s">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="102" ht="101" customHeight="1">
-      <x:c r="A102" s="66" t="str">
+    <x:row r="100" ht="101" customHeight="1">
+      <x:c r="A100" s="66" t="str">
         <x:v>MATRIX Operation
 矩阵乘操作</x:v>
       </x:c>
-      <x:c r="B102" s="66" t="str">
+      <x:c r="B100" s="66" t="str">
         <x:v>矩阵乘向量</x:v>
       </x:c>
-      <x:c r="C102" s="73" t="str">
+      <x:c r="C100" s="73" t="str">
         <x:v>TGEMV_MX_ACC</x:v>
       </x:c>
-      <x:c r="D102" s="78" t="str">
+      <x:c r="D100" s="78" t="str">
         <x:v>BSTART.CUBE TGEMVMX.ACC AType
 B.DATR BType RMode Sat
 B.FPATR
@@ -6990,35 +6869,35 @@
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
-      <x:c r="E102" s="78" t="str">
+      <x:c r="E100" s="78" t="str">
         <x:v>D Tile
 RowMaxOut Tile (optional)
 GroupMaxOut Tile (optional)</x:v>
       </x:c>
-      <x:c r="F102" s="78" t="str">
+      <x:c r="F100" s="78" t="str">
         <x:v>A Tile
 ScaleA Tile</x:v>
       </x:c>
-      <x:c r="G102" s="78" t="str">
+      <x:c r="G100" s="78" t="str">
         <x:v>B/Right Tile
 ScaleB/ScaleRight Tile</x:v>
       </x:c>
-      <x:c r="H102" s="78" t="str">
+      <x:c r="H100" s="78" t="str">
         <x:v>C Tile
 RowMaxIn Tile (optional)
 Quant parameter Tile or GPR (optional)
 ReLU parameter Tile or GPR (optional)</x:v>
       </x:c>
-      <x:c r="I102" s="78" t="str">
+      <x:c r="I100" s="78" t="str">
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
-      <x:c r="J102" s="83" t="str">
+      <x:c r="J100" s="83" t="str">
         <x:v>CUBE Mode 0, Function 22;</x:v>
       </x:c>
-      <x:c r="K102" s="90" t="str">
+      <x:c r="K100" s="90" t="str">
         <x:v>C 是显式 Local AccType Tile input，并在 K 乘积累加前读入 P；它不是隐式 ACC。 PostProcess 只在完整 K 累加后执行一次。</x:v>
       </x:c>
-      <x:c r="L102" s="91" t="str">
+      <x:c r="L100" s="91" t="str">
         <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
 canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
 任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
@@ -7032,18 +6911,18 @@
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" ht="101" customHeight="1">
-      <x:c r="A103" s="66" t="str">
+    <x:row r="101" ht="101" customHeight="1">
+      <x:c r="A101" s="66" t="str">
         <x:v>MATRIX Operation
 矩阵乘操作</x:v>
       </x:c>
-      <x:c r="B103" s="66" t="str">
+      <x:c r="B101" s="66" t="str">
         <x:v>矩阵乘向量</x:v>
       </x:c>
-      <x:c r="C103" s="73" t="str">
+      <x:c r="C101" s="73" t="str">
         <x:v>TGEMV_MX_BIAS</x:v>
       </x:c>
-      <x:c r="D103" s="78" t="str">
+      <x:c r="D101" s="78" t="str">
         <x:v>BSTART.CUBE TGEMVMX.BIAS AType
 B.DATR BType RMode Sat
 B.FPATR
@@ -7053,35 +6932,35 @@
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
-      <x:c r="E103" s="78" t="str">
+      <x:c r="E101" s="78" t="str">
         <x:v>D Tile
 RowMaxOut Tile (optional)
 GroupMaxOut Tile (optional)</x:v>
       </x:c>
-      <x:c r="F103" s="78" t="str">
+      <x:c r="F101" s="78" t="str">
         <x:v>A Tile
 ScaleA Tile</x:v>
       </x:c>
-      <x:c r="G103" s="78" t="str">
+      <x:c r="G101" s="78" t="str">
         <x:v>B/Right Tile
 ScaleB/ScaleRight Tile</x:v>
       </x:c>
-      <x:c r="H103" s="78" t="str">
+      <x:c r="H101" s="78" t="str">
         <x:v>Bias Tile
 RowMaxIn Tile (optional)
 Quant parameter Tile or GPR (optional)
 ReLU parameter Tile or GPR (optional)</x:v>
       </x:c>
-      <x:c r="I103" s="78" t="str">
+      <x:c r="I101" s="78" t="str">
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
-      <x:c r="J103" s="83" t="str">
+      <x:c r="J101" s="83" t="str">
         <x:v>CUBE Mode 0, Function 21;</x:v>
       </x:c>
-      <x:c r="K103" s="90" t="str">
+      <x:c r="K101" s="90" t="str">
         <x:v>Bias 是显式 Local Tile input，并在 K 乘积累加前预装入 P。 PostProcess 只在完整 K 累加后执行一次。</x:v>
       </x:c>
-      <x:c r="L103" s="91" t="str">
+      <x:c r="L101" s="91" t="str">
         <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
 canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
 任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
@@ -7095,18 +6974,18 @@
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
-    <x:row r="104" ht="101" customHeight="1">
-      <x:c r="A104" s="96" t="str">
+    <x:row r="102" ht="101" customHeight="1">
+      <x:c r="A102" s="96" t="str">
         <x:v>MATRIX Operation
 矩阵乘操作</x:v>
       </x:c>
-      <x:c r="B104" s="96" t="str">
+      <x:c r="B102" s="96" t="str">
         <x:v>矩阵乘矩阵</x:v>
       </x:c>
-      <x:c r="C104" s="73" t="str">
+      <x:c r="C102" s="73" t="str">
         <x:v>TMATMUL_MX_ACC</x:v>
       </x:c>
-      <x:c r="D104" s="78" t="str">
+      <x:c r="D102" s="78" t="str">
         <x:v>BSTART.CUBE TMATMULMX.ACC AType
 B.DATR BType RMode Sat
 B.FPATR
@@ -7117,35 +6996,35 @@
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
-      <x:c r="E104" s="78" t="str">
+      <x:c r="E102" s="78" t="str">
         <x:v>D Tile
 RowMaxOut Tile (optional)
 GroupMaxOut Tile (optional)</x:v>
       </x:c>
-      <x:c r="F104" s="78" t="str">
+      <x:c r="F102" s="78" t="str">
         <x:v>A Tile
 ScaleA Tile</x:v>
       </x:c>
-      <x:c r="G104" s="78" t="str">
+      <x:c r="G102" s="78" t="str">
         <x:v>B/Right Tile
 ScaleB/ScaleRight Tile</x:v>
       </x:c>
-      <x:c r="H104" s="78" t="str">
+      <x:c r="H102" s="78" t="str">
         <x:v>C Tile
 RowMaxIn Tile (optional)
 Quant parameter Tile or GPR (optional)
 ReLU parameter Tile or GPR (optional)</x:v>
       </x:c>
-      <x:c r="I104" s="78" t="str">
+      <x:c r="I102" s="78" t="str">
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
-      <x:c r="J104" s="83" t="str">
+      <x:c r="J102" s="83" t="str">
         <x:v>CUBE Mode 0, Function 6;</x:v>
       </x:c>
-      <x:c r="K104" s="90" t="str">
+      <x:c r="K102" s="90" t="str">
         <x:v>C 是显式 Local AccType Tile input，并在 K 乘积累加前读入 P；它不是隐式 ACC。 PostProcess 只在完整 K 累加后执行一次。</x:v>
       </x:c>
-      <x:c r="L104" s="91" t="str">
+      <x:c r="L102" s="91" t="str">
         <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
 canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
 任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
@@ -7159,18 +7038,18 @@
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
-    <x:row r="105" ht="101" customHeight="1">
-      <x:c r="A105" s="96" t="str">
+    <x:row r="103" ht="101" customHeight="1">
+      <x:c r="A103" s="96" t="str">
         <x:v>MATRIX Operation
 矩阵乘操作</x:v>
       </x:c>
-      <x:c r="B105" s="96" t="str">
+      <x:c r="B103" s="96" t="str">
         <x:v>矩阵乘矩阵</x:v>
       </x:c>
-      <x:c r="C105" s="73" t="str">
+      <x:c r="C103" s="73" t="str">
         <x:v>TMATMUL_MX_BIAS</x:v>
       </x:c>
-      <x:c r="D105" s="78" t="str">
+      <x:c r="D103" s="78" t="str">
         <x:v>BSTART.CUBE TMATMULMX.BIAS AType
 B.DATR BType RMode Sat
 B.FPATR
@@ -7181,35 +7060,35 @@
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
-      <x:c r="E105" s="78" t="str">
+      <x:c r="E103" s="78" t="str">
         <x:v>D Tile
 RowMaxOut Tile (optional)
 GroupMaxOut Tile (optional)</x:v>
       </x:c>
-      <x:c r="F105" s="78" t="str">
+      <x:c r="F103" s="78" t="str">
         <x:v>A Tile
 ScaleA Tile</x:v>
       </x:c>
-      <x:c r="G105" s="78" t="str">
+      <x:c r="G103" s="78" t="str">
         <x:v>B/Right Tile
 ScaleB/ScaleRight Tile</x:v>
       </x:c>
-      <x:c r="H105" s="78" t="str">
+      <x:c r="H103" s="78" t="str">
         <x:v>Bias Tile
 RowMaxIn Tile (optional)
 Quant parameter Tile or GPR (optional)
 ReLU parameter Tile or GPR (optional)</x:v>
       </x:c>
-      <x:c r="I105" s="78" t="str">
+      <x:c r="I103" s="78" t="str">
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
-      <x:c r="J105" s="83" t="str">
+      <x:c r="J103" s="83" t="str">
         <x:v>CUBE Mode 0, Function 5;</x:v>
       </x:c>
-      <x:c r="K105" s="90" t="str">
+      <x:c r="K103" s="90" t="str">
         <x:v>Bias 是显式 Local Tile input，并在 K 乘积累加前预装入 P。 PostProcess 只在完整 K 累加后执行一次。</x:v>
       </x:c>
-      <x:c r="L105" s="91" t="str">
+      <x:c r="L103" s="91" t="str">
         <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
 canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
 任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
@@ -7223,91 +7102,327 @@
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
-    <x:row r="106" ht="101" customHeight="1">
-      <x:c r="A106" s="96" t="str">
+    <x:row r="104" ht="101" customHeight="1">
+      <x:c r="A104" s="96" t="str">
         <x:v>Tile Memory Operation
 Tile级访存操作</x:v>
       </x:c>
-      <x:c r="B106" s="96" t="str">
+      <x:c r="B104" s="96" t="str">
         <x:v>PE间搬运</x:v>
       </x:c>
-      <x:c r="C106" s="73" t="str">
+      <x:c r="C104" s="73" t="str">
         <x:v>GMOV</x:v>
       </x:c>
-      <x:c r="D106" s="78" t="str">
+      <x:c r="D104" s="78" t="str">
         <x:v>BSTART.TLSU GMOV, DataType
 B.IOT source, destination, PE_MASK, TSize
 B.IOR peer_tid</x:v>
       </x:c>
-      <x:c r="E106" s="78" t="str">
+      <x:c r="E104" s="78" t="str">
         <x:v>destination Local Tile</x:v>
       </x:c>
-      <x:c r="F106" s="78" t="str">
+      <x:c r="F104" s="78" t="str">
         <x:v>source Local Tile</x:v>
       </x:c>
-      <x:c r="G106" s="78" t="str">
+      <x:c r="G104" s="78" t="str">
         <x:v>peer_tid GPR</x:v>
       </x:c>
-      <x:c r="H106" s="78"/>
-      <x:c r="I106" s="78" t="str">
+      <x:c r="H104" s="78"/>
+      <x:c r="I104" s="78" t="str">
         <x:v>byte-preserving; source and destination descriptors must match</x:v>
       </x:c>
-      <x:c r="J106" s="83" t="str">
+      <x:c r="J104" s="83" t="str">
         <x:v>TLSU Function 13;</x:v>
       </x:c>
-      <x:c r="K106" s="90" t="str">
+      <x:c r="K104" s="90" t="str">
         <x:v>GMOV 是 DavinciOO v5 的 Core 内 PE 间 Local Tile 搬运扩展，公开接口为：</x:v>
       </x:c>
-      <x:c r="L106" s="91" t="str">
+      <x:c r="L104" s="91" t="str">
         <x:v>source/destination 必须是 descriptor-compatible ordinary Local Tile；同一物理输入输出采用 read-old/write-new。
 所有四个 PE 必须以相同动态顺序到达 collective；不收敛或 participant 不一致非法。
 SharedTile、Tile role 转换及跨 Core peer_tid 不受支持。
 逻辑 TileAcc role 仍映射到 ordinary physical TReg；GMOV 不访问任何 hidden accumulator state。</x:v>
       </x:c>
     </x:row>
-    <x:row r="107" ht="101" customHeight="1">
-      <x:c r="A107" s="124" t="str">
+    <x:row r="105" ht="101" customHeight="1">
+      <x:c r="A105" s="124" t="str">
         <x:v>Complex Layout Transformation
 复杂变换操作</x:v>
       </x:c>
-      <x:c r="B107" s="96" t="str">
+      <x:c r="B105" s="96" t="str">
         <x:v>Tile搬运</x:v>
       </x:c>
-      <x:c r="C107" s="73" t="str">
+      <x:c r="C105" s="73" t="str">
         <x:v>TMOV</x:v>
       </x:c>
-      <x:c r="D107" s="78" t="str">
+      <x:c r="D105" s="78" t="str">
         <x:v>BSTART.TLSU TMOV, DataType
 B.DIM LB0
 B.DIM (LB1/LB2 for 2D)
 B.IOT</x:v>
       </x:c>
-      <x:c r="E107" s="78" t="str">
+      <x:c r="E105" s="78" t="str">
         <x:v>destination Local or Shared Tile</x:v>
       </x:c>
-      <x:c r="F107" s="78" t="str">
+      <x:c r="F105" s="78" t="str">
         <x:v>source Local or Shared Tile</x:v>
       </x:c>
-      <x:c r="G107" s="78" t="str">
+      <x:c r="G105" s="78" t="str">
         <x:v>compile-time SharedMoveMode when Shared participates</x:v>
       </x:c>
-      <x:c r="H107" s="78"/>
-      <x:c r="I107" s="78" t="str">
+      <x:c r="H105" s="78"/>
+      <x:c r="I105" s="78" t="str">
         <x:v>byte-preserving; descriptors must be compatible</x:v>
       </x:c>
-      <x:c r="J107" s="83" t="str">
+      <x:c r="J105" s="83" t="str">
         <x:v>TLSU Function 2, Shared Functions 8–11;</x:v>
       </x:c>
-      <x:c r="K107" s="90" t="str">
+      <x:c r="K105" s="90" t="str">
         <x:v>Ordinary PTO TMOV(dst,src) remains a Local Tile move/conversion. DavinciOO v5 adds strongly typed Local↔Shared forms under the same intrinsic name; no _SHARED operation is introduced.</x:v>
       </x:c>
-      <x:c r="L107" s="91" t="str">
+      <x:c r="L105" s="91" t="str">
         <x:v>Shared→Shared TMOV is absent in v5; copy/transform through Local Tile.
 Runtime mode, owner or size is illegal.
 PE_MASK is a four-bit quarter predicate; multiple bits are allowed and
   0000 is a no-op.
 Absolute Shared registers are compiler-managed; C++ cannot specify Sx.
 RecordEvent is reused; there is no SharedEvent, and event completion is not a cross-PE GM fence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="101" customHeight="1">
+      <x:c r="A106" s="101" t="str">
+        <x:v>Tile Memory Operation
+Tile级访存操作</x:v>
+      </x:c>
+      <x:c r="B106" s="101" t="str">
+        <x:v>原子不规则访存</x:v>
+      </x:c>
+      <x:c r="C106" s="106" t="str">
+        <x:v>MGATHER_CAS</x:v>
+      </x:c>
+      <x:c r="D106" s="111" t="str">
+        <x:v>BSTART.MGATHER.CAS DataType
+B.IOT
+B.IOR base_address</x:v>
+      </x:c>
+      <x:c r="E106" s="111" t="str">
+        <x:v>old-value destination tile</x:v>
+      </x:c>
+      <x:c r="F106" s="111" t="str">
+        <x:v>base address
+indices tile</x:v>
+      </x:c>
+      <x:c r="G106" s="111" t="str">
+        <x:v>expected tile</x:v>
+      </x:c>
+      <x:c r="H106" s="111" t="str">
+        <x:v>replacement tile</x:v>
+      </x:c>
+      <x:c r="I106" s="111" t="str">
+        <x:v>TLSU atomic data types accepted by BSTART.MGATHER.CAS</x:v>
+      </x:c>
+      <x:c r="J106" s="116" t="str">
+        <x:v>TLSU Function 8;</x:v>
+      </x:c>
+      <x:c r="K106" s="120" t="str">
+        <x:v>MGATHER_CAS performs an atomic compare-and-swap for every indexed lane. The old memory value is always returned in the destination Tile. Memory is replaced only when the old value equals the lane's expected value, and an atomic event is recorded for both successful and failed comparisons.</x:v>
+      </x:c>
+      <x:c r="L106" s="121" t="str">
+        <x:v>Destination and index Tiles must have equal logical shape.
+Expected and replacement Tiles must match the destination shape and dtype.
+Read and write translation must resolve to the same address for each lane;
+  otherwise the operation raises a precise data-page fault.
+Each lane is an atomic read-modify-write using the current bundle memory-order
+  attribute. No stronger order between different lanes or PEs is guaranteed.
+BSTART.MGATHER.CAS is an accepted PTO ISA 0.58.0 command form.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="101" customHeight="1">
+      <x:c r="A107" s="101" t="str">
+        <x:v>Tile Memory Operation
+Tile级访存操作</x:v>
+      </x:c>
+      <x:c r="B107" s="101" t="str">
+        <x:v>不规则访存</x:v>
+      </x:c>
+      <x:c r="C107" s="106" t="str">
+        <x:v>MGATHER_MASK</x:v>
+      </x:c>
+      <x:c r="D107" s="111" t="str">
+        <x:v>BSTART.MGATHER.MASK DataType
+B.DATR PadValue (optional)
+B.IOT
+B.IOR base_address</x:v>
+      </x:c>
+      <x:c r="E107" s="111" t="str">
+        <x:v>destination tile</x:v>
+      </x:c>
+      <x:c r="F107" s="111" t="str">
+        <x:v>base address
+indices tile</x:v>
+      </x:c>
+      <x:c r="G107" s="111" t="str">
+        <x:v>mask tile</x:v>
+      </x:c>
+      <x:c r="H107" s="111" t="str">
+        <x:v>masked-off pad value</x:v>
+      </x:c>
+      <x:c r="I107" s="111" t="str">
+        <x:v>TLSU data types accepted by BSTART.MGATHER.MASK</x:v>
+      </x:c>
+      <x:c r="J107" s="116" t="str">
+        <x:v>TLSU Function 6;</x:v>
+      </x:c>
+      <x:c r="K107" s="120" t="str">
+        <x:v>MGATHER_MASK gathers indexed memory elements for nonzero mask lanes. A zero mask lane performs no memory access and writes the current bundle pad value to the corresponding destination element. All selected addresses are probed before any load event or destination update, preserving precise faults.</x:v>
+      </x:c>
+      <x:c r="L107" s="121" t="str">
+        <x:v>Destination, index, and mask Tiles must have equal logical shape.
+Index and mask contents must be defined before execution.
+Masked-off lanes do not access memory; selected lanes use the current bundle
+  memory-order attribute.
+BSTART.MGATHER.MASK is an accepted PTO ISA 0.58.0 command form, not a
+  future-reserved encoding.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="101" customHeight="1">
+      <x:c r="A108" s="101" t="str">
+        <x:v>Tile Memory Operation
+Tile级访存操作</x:v>
+      </x:c>
+      <x:c r="B108" s="101" t="str">
+        <x:v>不规则访存</x:v>
+      </x:c>
+      <x:c r="C108" s="106" t="str">
+        <x:v>MSCATTER_MASK</x:v>
+      </x:c>
+      <x:c r="D108" s="111" t="str">
+        <x:v>BSTART.MSCATTER.MASK DataType
+B.IOT
+B.IOR base_address</x:v>
+      </x:c>
+      <x:c r="E108" s="111" t="str">
+        <x:v>indexed memory locations</x:v>
+      </x:c>
+      <x:c r="F108" s="111" t="str">
+        <x:v>source tile
+indices tile</x:v>
+      </x:c>
+      <x:c r="G108" s="111" t="str">
+        <x:v>mask tile</x:v>
+      </x:c>
+      <x:c r="H108" s="111"/>
+      <x:c r="I108" s="111" t="str">
+        <x:v>TLSU data types accepted by BSTART.MSCATTER.MASK</x:v>
+      </x:c>
+      <x:c r="J108" s="116" t="str">
+        <x:v>TLSU Function 7;</x:v>
+      </x:c>
+      <x:c r="K108" s="120" t="str">
+        <x:v>MSCATTER_MASK scatters source elements to indexed memory locations for nonzero mask lanes. Zero mask lanes have no memory side effect. All selected addresses are probed before the scatter commit phase so a failing footprint does not produce a partial event prefix.</x:v>
+      </x:c>
+      <x:c r="L108" s="121" t="str">
+        <x:v>Source, index, and mask Tiles must have equal logical shape and defined
+  contents.
+Selected lanes obey the current bundle memory-order attribute.
+Conflicting selected addresses follow the architectural scatter commit
+  policy; programmers must not infer a stronger lane order.
+BSTART.MSCATTER.MASK is an accepted PTO ISA 0.58.0 command form.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="101" customHeight="1">
+      <x:c r="A109" s="127" t="str">
+        <x:v>Complex Layout Transformation
+复杂变换操作</x:v>
+      </x:c>
+      <x:c r="B109" s="101" t="str">
+        <x:v>直方图</x:v>
+      </x:c>
+      <x:c r="C109" s="106" t="str">
+        <x:v>THISTOGRAM</x:v>
+      </x:c>
+      <x:c r="D109" s="111" t="str">
+        <x:v>BSTART.TEPL THISTOGRAM, DataType
+B.DATR selected_byte
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E109" s="111" t="str">
+        <x:v>per-row cumulative 256-bin histogram</x:v>
+      </x:c>
+      <x:c r="F109" s="111" t="str">
+        <x:v>U16 or U32 source tile</x:v>
+      </x:c>
+      <x:c r="G109" s="111" t="str">
+        <x:v>filter/index tile</x:v>
+      </x:c>
+      <x:c r="H109" s="111" t="str">
+        <x:v>selected_byte 0..3</x:v>
+      </x:c>
+      <x:c r="I109" s="111" t="str">
+        <x:v>source: U16, U32</x:v>
+      </x:c>
+      <x:c r="J109" s="116" t="str">
+        <x:v>TEPL Mode 3, Function 8, TileOp 0x68;</x:v>
+      </x:c>
+      <x:c r="K109" s="120" t="str">
+        <x:v>THISTOGRAM selects one byte from each U16 or U32 source element, optionally filters higher bytes through the index Tile, counts 256 byte values per row, and writes the cumulative bin counts to the destination. selected_byte is encoded through the B.DATR.PadValueOrByteId union for this operation.</x:v>
+      </x:c>
+      <x:c r="L109" s="121" t="str">
+        <x:v>Destination and source row counts must match; destination valid columns must
+  be at least 256.
+U16 sources allow byte 0 or 1. U32 sources allow byte 0 through 3.
+The index Tile must supply the filter rows required by the selected byte.
+The destination valid region becomes defined after successful completion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="101" customHeight="1">
+      <x:c r="A110" s="127" t="str">
+        <x:v>Complex Layout Transformation
+复杂变换操作</x:v>
+      </x:c>
+      <x:c r="B110" s="101" t="str">
+        <x:v>排序</x:v>
+      </x:c>
+      <x:c r="C110" s="106" t="str">
+        <x:v>TSORT</x:v>
+      </x:c>
+      <x:c r="D110" s="111" t="str">
+        <x:v>BSTART.TEPL TSORT, DataType
+B.DIM sort_width -&gt; LB0
+B.IOT</x:v>
+      </x:c>
+      <x:c r="E110" s="111" t="str">
+        <x:v>sorted values tile
+original-index U32 tile</x:v>
+      </x:c>
+      <x:c r="F110" s="111" t="str">
+        <x:v>source values tile</x:v>
+      </x:c>
+      <x:c r="G110" s="111" t="str">
+        <x:v>sort_width 1..64</x:v>
+      </x:c>
+      <x:c r="H110" s="111" t="str">
+        <x:v>descending control</x:v>
+      </x:c>
+      <x:c r="I110" s="111" t="str">
+        <x:v>values: source/destination dtype match, indices: U32</x:v>
+      </x:c>
+      <x:c r="J110" s="116" t="str">
+        <x:v>TEPL Mode 3, Function 12, TileOp 0x6C;</x:v>
+      </x:c>
+      <x:c r="K110" s="120" t="str">
+        <x:v>TSORT sorts each consecutive group of sort_width elements from the source Tile, writes the ordered values to destination0, and writes each value's original group-relative index to the U32 destination1 Tile. sort_width is in 1..64; the canonical bundle decoder obtains it from LB0 and defaults to 32 when no nonzero width is supplied. The semantic descending operand selects ascending or descending order; the current PTO block transport supplies the operation default (false, ascending).</x:v>
+      </x:c>
+      <x:c r="L110" s="121" t="str">
+        <x:v>The two destinations must be distinct and must have the same element count
+  as the source.
+The values destination dtype must equal the source dtype; the index
+  destination dtype is U32.
+Sorting is stable only where the selected numeric profile defines equal-value
+  ordering; no memory or cross-PE ordering is implied.
+TSORT32 is not an ISA identity in PTO ISA 0.58.0. It is replaced by
+  TSORT with explicit sort_width; the old PTO source page is retained only
+  as provenance for the operation family.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7320,7 +7435,7 @@
     <x:mergeCell ref="A52:A67"/>
     <x:mergeCell ref="A68:A75"/>
     <x:mergeCell ref="A76:A80"/>
-    <x:mergeCell ref="A81:A101"/>
+    <x:mergeCell ref="A81:A99"/>
     <x:mergeCell ref="B2:B6"/>
     <x:mergeCell ref="B8:B14"/>
     <x:mergeCell ref="B15:B18"/>
@@ -7335,10 +7450,10 @@
     <x:mergeCell ref="B72:B75"/>
     <x:mergeCell ref="B76:B78"/>
     <x:mergeCell ref="B79:B80"/>
-    <x:mergeCell ref="B81:B85"/>
-    <x:mergeCell ref="B86:B88"/>
-    <x:mergeCell ref="B89:B95"/>
-    <x:mergeCell ref="B98:B101"/>
+    <x:mergeCell ref="B81:B84"/>
+    <x:mergeCell ref="B85:B87"/>
+    <x:mergeCell ref="B88:B94"/>
+    <x:mergeCell ref="B96:B99"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7354,106 +7469,106 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>471</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>472</x:v>
+        <x:v>455</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26.399999618530273" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>473</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>474</x:v>
+        <x:v>457</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="26.399999618530273" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>475</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>476</x:v>
+        <x:v>459</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" customHeight="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>477</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>478</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.399999618530273" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>479</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>480</x:v>
+        <x:v>463</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>481</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>482</x:v>
+        <x:v>465</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>483</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>484</x:v>
+        <x:v>467</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>485</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>486</x:v>
+        <x:v>469</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>487</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>488</x:v>
+        <x:v>471</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40.5" customHeight="1">
       <x:c r="A10" s="3" t="s">
-        <x:v>489</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
-        <x:v>490</x:v>
+        <x:v>473</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40.5" customHeight="1">
       <x:c r="A11" s="3" t="s">
-        <x:v>491</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>475</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40.5" customHeight="1">
       <x:c r="A12" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>477</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="40.5" customHeight="1">
       <x:c r="A13" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
-        <x:v>496</x:v>
+        <x:v>479</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7471,98 +7586,98 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>497</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>498</x:v>
+        <x:v>481</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="14" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>499</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>500</x:v>
+        <x:v>483</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="14" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>501</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>502</x:v>
+        <x:v>485</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="14" customHeight="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>503</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>504</x:v>
+        <x:v>487</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="14" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>505</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>506</x:v>
+        <x:v>489</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="14" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>507</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>508</x:v>
+        <x:v>491</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>509</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>510</x:v>
+        <x:v>493</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="14" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>511</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>512</x:v>
+        <x:v>495</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="14" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>513</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>514</x:v>
+        <x:v>497</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="14" customHeight="1">
       <x:c r="A10" s="2" t="s">
-        <x:v>515</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
-        <x:v>516</x:v>
+        <x:v>499</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="14" customHeight="1">
       <x:c r="A11" s="2" t="s">
-        <x:v>517</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>518</x:v>
+        <x:v>501</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="14" customHeight="1">
       <x:c r="A12" s="2" t="s">
-        <x:v>519</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>520</x:v>
+        <x:v>503</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: align PTO 0.58 release surfaces
</commit_message>
<xml_diff>
--- a/spec/encoding/PTO-ISA-Encoding.xlsx
+++ b/spec/encoding/PTO-ISA-Encoding.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R77efea90e68d4cb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rd5d2a39aebb44e71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="Rfc64d61f63034444"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rf664057da7f640d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Ra3a3f0a762e44863"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R6213fd2065b34aca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -880,11 +880,6 @@
     <x:t xml:space="preserve">PE-local CUBE matrix multiply: C[i,j] = sum_k(A[i,k] * B[k,j]).</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">1. M/N/K are required 16-bit dims in B.DIM(LB0/LB1/LB2).
-2. M/N/K, fractal/layout, and dtype must satisfy the active CUBE target profile.
-3. ACC lifetime, precision, and export/convert follow the CUBE/ACC contract; ACCCVT writes ACC back to a normal Tile.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">TMATMUL_BIAS</x:t>
   </x:si>
   <x:si>
@@ -894,11 +889,6 @@
     <x:t xml:space="preserve">Matmul with bias add (tile world, ins/outs).</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">1. M/N/K are required 16-bit dims in B.DIM(LB0/LB1/LB2).
-2. M/N/K, fractal/layout, and dtype must satisfy the active CUBE target profile.
-3. ACC lifetime, precision, and export/convert behavior follow the CUBE/ACC contract.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">TMATMUL_ACC</x:t>
   </x:si>
   <x:si>
@@ -906,11 +896,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">PE-local CUBE matrix multiply accumulate; variant operands are profile-specific.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1. M/N/K are required 16-bit dims in B.DIM(LB0/LB1/LB2).
-2. Input 2 appears only when the opcode profile requires an input ACC, bias, scale, or other ExtraTile.
-3. Compiler scratch is not ISA-visible; this row does not define group-level GMMA/barrier semantics.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TMATMUL_MX</x:t>
@@ -5607,15 +5592,25 @@
       <x:c r="K68" s="2" t="s">
         <x:v>280</x:v>
       </x:c>
-      <x:c r="L68" s="3" t="s">
-        <x:v>281</x:v>
+      <x:c r="L68" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+Cooperative form 中 C/D、RowMaxIn/Out、GroupMaxOut 为 MShard4；Bias、vector QuantParam、vector PReLU 是四 PE 上内容相同的完整 Local N-vector；scalar GPR 参数也必须在四 PE 上相等。
+D 必须是显式 ordinary physical Local destination。
+Cooperative TMATMUL 的 Shared read 不修改 descriptor/payload；并发 overlap 由程序避免，且该 rendezvous 不建立 GM ordering。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="118">
       <x:c r="A69" s="46"/>
       <x:c r="B69" s="46"/>
       <x:c r="C69" s="16" t="s">
-        <x:v>282</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="D69" s="17" t="str">
         <x:v>BSTART.CUBE TMATMUL.BIAS AType
@@ -5649,20 +5644,30 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J69" s="41" t="s">
+        <x:v>282</x:v>
+      </x:c>
+      <x:c r="K69" s="2" t="s">
         <x:v>283</x:v>
       </x:c>
-      <x:c r="K69" s="2" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="L69" s="3" t="s">
-        <x:v>285</x:v>
+      <x:c r="L69" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+Cooperative form 中 C/D、RowMaxIn/Out、GroupMaxOut 为 MShard4；Bias、vector QuantParam、vector PReLU 是四 PE 上内容相同的完整 Local N-vector；scalar GPR 参数也必须在四 PE 上相等。
+D 必须是显式 ordinary physical Local destination。
+Cooperative TMATMUL 的 Shared read 不修改 descriptor/payload；并发 overlap 由程序避免，且该 rendezvous 不建立 GM ordering。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="118">
       <x:c r="A70" s="46"/>
       <x:c r="B70" s="46"/>
       <x:c r="C70" s="16" t="s">
-        <x:v>286</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="D70" s="17" t="str">
         <x:v>BSTART.CUBE TMATMUL.ACC AType
@@ -5696,20 +5701,30 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J70" s="41" t="s">
-        <x:v>287</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="K70" s="2" t="s">
-        <x:v>288</x:v>
-      </x:c>
-      <x:c r="L70" s="3" t="s">
-        <x:v>289</x:v>
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="L70" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+Cooperative form 中 C/D、RowMaxIn/Out、GroupMaxOut 为 MShard4；Bias、vector QuantParam、vector PReLU 是四 PE 上内容相同的完整 Local N-vector；scalar GPR 参数也必须在四 PE 上相等。
+D==C 仅在 D 保持 TileAcc role 且 dtype、shape、layout、allocation 完全相同时合法；实现必须 read-old/rename-new，禁止物理原地覆盖。C 不携带 partial-sum provenance 要求。
+Cooperative TMATMUL 的 Shared read 不修改 descriptor/payload；并发 overlap 由程序避免，且该 rendezvous 不建立 GM ordering。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="118.75">
       <x:c r="A71" s="46"/>
       <x:c r="B71" s="46"/>
       <x:c r="C71" s="16" t="s">
-        <x:v>290</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="D71" s="17" t="str">
         <x:v>BSTART.CUBE TMATMULMX AType
@@ -5744,22 +5759,32 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J71" s="41" t="s">
-        <x:v>291</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="K71" s="2" t="s">
-        <x:v>292</x:v>
-      </x:c>
-      <x:c r="L71" s="3" t="s">
-        <x:v>285</x:v>
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="L71" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+Cooperative form 中 C/D、RowMaxIn/Out、GroupMaxOut 为 MShard4；Bias、vector QuantParam、vector PReLU 是四 PE 上内容相同的完整 Local N-vector；scalar GPR 参数也必须在四 PE 上相等。
+D 必须是显式 ordinary physical Local destination。
+Cooperative TMATMUL 的 Shared read 不修改 descriptor/payload；并发 overlap 由程序避免，且该 rendezvous 不建立 GM ordering。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="101">
       <x:c r="A72" s="46"/>
       <x:c r="B72" s="46" t="s">
-        <x:v>293</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="C72" s="13" t="s">
-        <x:v>294</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="D72" s="9" t="str">
         <x:v>BSTART.CUBE TGEMV AType
@@ -5791,20 +5816,30 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J72" s="40" t="s">
-        <x:v>295</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="K72" s="2" t="s">
-        <x:v>296</x:v>
-      </x:c>
-      <x:c r="L72" s="3" t="s">
-        <x:v>285</x:v>
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="L72" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+所有 operand/output 都是单 PE Local Tile；M 固定为 1。
+D 必须是显式 ordinary physical Local destination。
+TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="118">
       <x:c r="A73" s="46"/>
       <x:c r="B73" s="46"/>
       <x:c r="C73" s="16" t="s">
-        <x:v>297</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="D73" s="17" t="str">
         <x:v>BSTART.CUBE TGEMV.BIAS AType
@@ -5837,20 +5872,30 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J73" s="41" t="s">
-        <x:v>298</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="K73" s="2" t="s">
-        <x:v>299</x:v>
-      </x:c>
-      <x:c r="L73" s="3" t="s">
-        <x:v>285</x:v>
+        <x:v>296</x:v>
+      </x:c>
+      <x:c r="L73" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+所有 operand/output 都是单 PE Local Tile；M 固定为 1。
+D 必须是显式 ordinary physical Local destination。
+TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="118">
       <x:c r="A74" s="46"/>
       <x:c r="B74" s="46"/>
       <x:c r="C74" s="16" t="s">
-        <x:v>300</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="D74" s="17" t="str">
         <x:v>BSTART.CUBE TGEMV.ACC AType
@@ -5883,20 +5928,30 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J74" s="41" t="s">
-        <x:v>301</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="K74" s="2" t="s">
-        <x:v>302</x:v>
-      </x:c>
-      <x:c r="L74" s="3" t="s">
-        <x:v>285</x:v>
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="L74" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+所有 operand/output 都是单 PE Local Tile；M 固定为 1。
+D==C 仅在 D 保持 TileAcc role 且 dtype、shape、layout、allocation 完全相同时合法；实现必须 read-old/rename-new，禁止物理原地覆盖。C 不携带 partial-sum provenance 要求。
+TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="101.75">
       <x:c r="A75" s="47"/>
       <x:c r="B75" s="47"/>
       <x:c r="C75" s="24" t="s">
-        <x:v>303</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="D75" s="25" t="str">
         <x:v>BSTART.CUBE TGEMVMX AType
@@ -5930,24 +5985,34 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J75" s="43" t="s">
-        <x:v>304</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="K75" s="2" t="s">
-        <x:v>305</x:v>
-      </x:c>
-      <x:c r="L75" s="3" t="s">
-        <x:v>285</x:v>
+        <x:v>302</x:v>
+      </x:c>
+      <x:c r="L75" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+所有 operand/output 都是单 PE Local Tile；M 固定为 1。
+D 必须是显式 ordinary physical Local destination。
+TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="101">
       <x:c r="A76" s="48" t="s">
-        <x:v>306</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="B76" s="48" t="s">
-        <x:v>307</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="C76" s="13" t="s">
-        <x:v>308</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="D76" s="9" t="str">
         <x:v>Local form
@@ -5977,20 +6042,20 @@
         <x:v>PTO TLOAD dtype/layout combinations supported by the v5 TLSU profile</x:v>
       </x:c>
       <x:c r="J76" s="40" t="s">
-        <x:v>309</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="K76" s="2" t="s">
-        <x:v>310</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="L76" s="3" t="s">
-        <x:v>311</x:v>
+        <x:v>308</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="101">
       <x:c r="A77" s="49"/>
       <x:c r="B77" s="49"/>
       <x:c r="C77" s="16" t="s">
-        <x:v>312</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="D77" s="17" t="str">
         <x:v>Local form
@@ -6028,17 +6093,17 @@
         <x:v>TLSU Function 1; Shared pe_scope Function 14;</x:v>
       </x:c>
       <x:c r="K77" s="2" t="s">
-        <x:v>313</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="L77" s="3" t="s">
-        <x:v>314</x:v>
+        <x:v>311</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="101.75">
       <x:c r="A78" s="49"/>
       <x:c r="B78" s="49"/>
       <x:c r="C78" s="16" t="s">
-        <x:v>315</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="D78" s="17" t="str">
         <x:v>BSTART.TLSU TPREFETCH, DataType
@@ -6049,35 +6114,35 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E78" s="17" t="s">
-        <x:v>316</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="F78" s="17" t="s">
-        <x:v>317</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="G78" s="17" t="s">
-        <x:v>318</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="H78" s="17"/>
       <x:c r="I78" s="17" t="s">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="J78" s="41" t="s">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="K78" s="2" t="s">
+        <x:v>318</x:v>
+      </x:c>
+      <x:c r="L78" s="3" t="s">
         <x:v>319</x:v>
-      </x:c>
-      <x:c r="J78" s="41" t="s">
-        <x:v>320</x:v>
-      </x:c>
-      <x:c r="K78" s="2" t="s">
-        <x:v>321</x:v>
-      </x:c>
-      <x:c r="L78" s="3" t="s">
-        <x:v>322</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="101">
       <x:c r="A79" s="49"/>
       <x:c r="B79" s="48" t="s">
-        <x:v>323</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C79" s="16" t="s">
-        <x:v>324</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D79" s="17" t="str">
         <x:v>BSTART.TLSU MGATHER, DataType
@@ -6091,30 +6156,30 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F79" s="17" t="s">
-        <x:v>325</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="G79" s="17" t="s">
-        <x:v>326</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="H79" s="17"/>
       <x:c r="I79" s="17" t="s">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="J79" s="41" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="K79" s="2" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="L79" s="3" t="s">
         <x:v>327</x:v>
-      </x:c>
-      <x:c r="J79" s="41" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="K79" s="2" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="L79" s="3" t="s">
-        <x:v>330</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="101.75">
       <x:c r="A80" s="50"/>
       <x:c r="B80" s="50"/>
       <x:c r="C80" s="16" t="s">
-        <x:v>331</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="D80" s="17" t="str">
         <x:v>BSTART.TLSU MSCATTER, DataType
@@ -6125,37 +6190,37 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E80" s="17" t="s">
-        <x:v>332</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="F80" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G80" s="17" t="s">
-        <x:v>326</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="H80" s="17"/>
       <x:c r="I80" s="17" t="s">
-        <x:v>333</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="J80" s="41" t="s">
-        <x:v>334</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="K80" s="2" t="s">
-        <x:v>335</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="L80" s="3" t="s">
-        <x:v>330</x:v>
+        <x:v>327</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="101">
       <x:c r="A81" s="51" t="s">
-        <x:v>336</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="B81" s="52" t="s">
-        <x:v>337</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="C81" s="13" t="s">
-        <x:v>338</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="D81" s="9" t="str">
         <x:v>BSTART.TEPL TEXPANDS, DataType
@@ -6169,18 +6234,18 @@
         <x:v>221</x:v>
       </x:c>
       <x:c r="F81" s="9" t="s">
-        <x:v>339</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="G81" s="9"/>
       <x:c r="H81" s="9"/>
       <x:c r="I81" s="9" t="s">
-        <x:v>340</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="J81" s="40" t="s">
-        <x:v>341</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="K81" s="2" t="s">
-        <x:v>342</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="L81" s="3" t="s">
         <x:v>71</x:v>
@@ -6190,7 +6255,7 @@
       <x:c r="A82" s="53"/>
       <x:c r="B82" s="54"/>
       <x:c r="C82" s="16" t="s">
-        <x:v>343</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D82" s="17" t="str">
         <x:v>BSTART.TEPL TCI, DataType
@@ -6201,33 +6266,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E82" s="17" t="s">
-        <x:v>344</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="F82" s="17" t="s">
-        <x:v>345</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="G82" s="17" t="s">
-        <x:v>346</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="H82" s="17"/>
       <x:c r="I82" s="17" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="J82" s="41" t="s">
+        <x:v>345</x:v>
+      </x:c>
+      <x:c r="K82" s="2" t="s">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="L82" s="3" t="s">
         <x:v>347</x:v>
-      </x:c>
-      <x:c r="J82" s="41" t="s">
-        <x:v>348</x:v>
-      </x:c>
-      <x:c r="K82" s="2" t="s">
-        <x:v>349</x:v>
-      </x:c>
-      <x:c r="L82" s="3" t="s">
-        <x:v>350</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="101">
       <x:c r="A83" s="53"/>
       <x:c r="B83" s="54"/>
       <x:c r="C83" s="16" t="s">
-        <x:v>351</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="D83" s="17" t="str">
         <x:v>BSTART.TEPL TTRI, DataType
@@ -6238,33 +6303,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E83" s="17" t="s">
-        <x:v>352</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="F83" s="17" t="s">
-        <x:v>353</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="G83" s="17" t="s">
-        <x:v>354</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="H83" s="17"/>
       <x:c r="I83" s="17" t="s">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="J83" s="41" t="s">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="K83" s="2" t="s">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="L83" s="3" t="s">
         <x:v>355</x:v>
-      </x:c>
-      <x:c r="J83" s="41" t="s">
-        <x:v>356</x:v>
-      </x:c>
-      <x:c r="K83" s="2" t="s">
-        <x:v>357</x:v>
-      </x:c>
-      <x:c r="L83" s="3" t="s">
-        <x:v>358</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="84.75">
       <x:c r="A84" s="53"/>
       <x:c r="B84" s="55"/>
       <x:c r="C84" s="24" t="s">
-        <x:v>359</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="D84" s="25" t="str">
         <x:v>BSTART.TEPL TFILLPAD, DataType
@@ -6274,35 +6339,35 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E84" s="25" t="s">
-        <x:v>360</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="F84" s="25" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G84" s="25" t="s">
-        <x:v>361</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="H84" s="25"/>
       <x:c r="I84" s="25" t="s">
+        <x:v>359</x:v>
+      </x:c>
+      <x:c r="J84" s="43" t="s">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="K84" s="2" t="s">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="L84" s="3" t="s">
         <x:v>362</x:v>
-      </x:c>
-      <x:c r="J84" s="43" t="s">
-        <x:v>363</x:v>
-      </x:c>
-      <x:c r="K84" s="2" t="s">
-        <x:v>364</x:v>
-      </x:c>
-      <x:c r="L84" s="3" t="s">
-        <x:v>365</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="118">
       <x:c r="A85" s="53"/>
       <x:c r="B85" s="52" t="s">
-        <x:v>366</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="C85" s="13" t="s">
-        <x:v>367</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="D85" s="17" t="str">
         <x:v>BSTART.TEPL TCVT, DataType
@@ -6312,33 +6377,33 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E85" s="17" t="s">
-        <x:v>368</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="F85" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G85" s="17" t="s">
-        <x:v>369</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="H85" s="17"/>
       <x:c r="I85" s="17" t="s">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="J85" s="41" t="s">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="K85" s="2" t="s">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="L85" s="3" t="s">
         <x:v>370</x:v>
-      </x:c>
-      <x:c r="J85" s="41" t="s">
-        <x:v>371</x:v>
-      </x:c>
-      <x:c r="K85" s="2" t="s">
-        <x:v>372</x:v>
-      </x:c>
-      <x:c r="L85" s="3" t="s">
-        <x:v>373</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="84">
       <x:c r="A86" s="53"/>
       <x:c r="B86" s="54"/>
       <x:c r="C86" s="16" t="s">
-        <x:v>374</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="D86" s="17" t="str">
         <x:v>BSTART.TEPL TQUANT, DataType
@@ -6348,35 +6413,35 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E86" s="17" t="s">
-        <x:v>375</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="F86" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G86" s="17" t="s">
-        <x:v>376</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="H86" s="17" t="str">
         <x:v>offset/scaling/index Tile (optional)</x:v>
       </x:c>
       <x:c r="I86" s="17" t="s">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="J86" s="41" t="s">
+        <x:v>375</x:v>
+      </x:c>
+      <x:c r="K86" s="2" t="s">
+        <x:v>376</x:v>
+      </x:c>
+      <x:c r="L86" s="3" t="s">
         <x:v>377</x:v>
-      </x:c>
-      <x:c r="J86" s="41" t="s">
-        <x:v>378</x:v>
-      </x:c>
-      <x:c r="K86" s="2" t="s">
-        <x:v>379</x:v>
-      </x:c>
-      <x:c r="L86" s="3" t="s">
-        <x:v>380</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="84.75">
       <x:c r="A87" s="53"/>
       <x:c r="B87" s="55"/>
       <x:c r="C87" s="16" t="s">
-        <x:v>381</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="D87" s="17" t="str">
         <x:v>BSTART.TEPL TDEQUANT, DataType
@@ -6386,37 +6451,37 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E87" s="17" t="s">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="F87" s="17" t="s">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="G87" s="17" t="s">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="H87" s="17" t="s">
         <x:v>382</x:v>
       </x:c>
-      <x:c r="F87" s="17" t="s">
+      <x:c r="I87" s="17" t="s">
         <x:v>383</x:v>
       </x:c>
-      <x:c r="G87" s="17" t="s">
+      <x:c r="J87" s="41" t="s">
         <x:v>384</x:v>
       </x:c>
-      <x:c r="H87" s="17" t="s">
+      <x:c r="K87" s="2" t="s">
         <x:v>385</x:v>
       </x:c>
-      <x:c r="I87" s="17" t="s">
+      <x:c r="L87" s="3" t="s">
         <x:v>386</x:v>
-      </x:c>
-      <x:c r="J87" s="41" t="s">
-        <x:v>387</x:v>
-      </x:c>
-      <x:c r="K87" s="2" t="s">
-        <x:v>388</x:v>
-      </x:c>
-      <x:c r="L87" s="3" t="s">
-        <x:v>389</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="101">
       <x:c r="A88" s="53"/>
       <x:c r="B88" s="52" t="s">
-        <x:v>390</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="C88" s="56" t="s">
-        <x:v>391</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="D88" s="56" t="str">
         <x:v>BSTART.TEPL TEXTRACT, DataType
@@ -6427,33 +6492,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E88" s="9" t="s">
-        <x:v>392</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="F88" s="9" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G88" s="9" t="s">
-        <x:v>393</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="H88" s="9"/>
       <x:c r="I88" s="9" t="s">
+        <x:v>391</x:v>
+      </x:c>
+      <x:c r="J88" s="40" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="K88" s="2" t="s">
+        <x:v>393</x:v>
+      </x:c>
+      <x:c r="L88" s="3" t="s">
         <x:v>394</x:v>
-      </x:c>
-      <x:c r="J88" s="40" t="s">
-        <x:v>395</x:v>
-      </x:c>
-      <x:c r="K88" s="2" t="s">
-        <x:v>396</x:v>
-      </x:c>
-      <x:c r="L88" s="3" t="s">
-        <x:v>397</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="101">
       <x:c r="A89" s="53"/>
       <x:c r="B89" s="54"/>
       <x:c r="C89" s="57" t="s">
-        <x:v>398</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D89" s="57" t="str">
         <x:v>BSTART.TEPL TINSERT, DataType
@@ -6467,30 +6532,30 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F89" s="17" t="s">
-        <x:v>399</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G89" s="17" t="s">
-        <x:v>393</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="H89" s="17"/>
       <x:c r="I89" s="17" t="s">
+        <x:v>397</x:v>
+      </x:c>
+      <x:c r="J89" s="41" t="s">
+        <x:v>398</x:v>
+      </x:c>
+      <x:c r="K89" s="2" t="s">
+        <x:v>399</x:v>
+      </x:c>
+      <x:c r="L89" s="3" t="s">
         <x:v>400</x:v>
-      </x:c>
-      <x:c r="J89" s="41" t="s">
-        <x:v>401</x:v>
-      </x:c>
-      <x:c r="K89" s="2" t="s">
-        <x:v>402</x:v>
-      </x:c>
-      <x:c r="L89" s="3" t="s">
-        <x:v>403</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="101">
       <x:c r="A90" s="53"/>
       <x:c r="B90" s="54"/>
       <x:c r="C90" s="57" t="s">
-        <x:v>404</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="D90" s="57" t="str">
         <x:v>BSTART.TEPL TGATHER, DataType
@@ -6500,33 +6565,33 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E90" s="17" t="s">
-        <x:v>405</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="F90" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G90" s="17" t="s">
-        <x:v>406</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="H90" s="17"/>
       <x:c r="I90" s="17" t="s">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="J90" s="41" t="s">
+        <x:v>405</x:v>
+      </x:c>
+      <x:c r="K90" s="2" t="s">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="L90" s="3" t="s">
         <x:v>407</x:v>
-      </x:c>
-      <x:c r="J90" s="41" t="s">
-        <x:v>408</x:v>
-      </x:c>
-      <x:c r="K90" s="2" t="s">
-        <x:v>409</x:v>
-      </x:c>
-      <x:c r="L90" s="3" t="s">
-        <x:v>410</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="84">
       <x:c r="A91" s="53"/>
       <x:c r="B91" s="54"/>
       <x:c r="C91" s="57" t="s">
-        <x:v>411</x:v>
+        <x:v>408</x:v>
       </x:c>
       <x:c r="D91" s="57" t="str">
         <x:v>BSTART.TEPL TSCATTER, DataType
@@ -6536,33 +6601,33 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E91" s="17" t="s">
-        <x:v>412</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="F91" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G91" s="17" t="s">
-        <x:v>413</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="H91" s="17"/>
       <x:c r="I91" s="17" t="s">
+        <x:v>411</x:v>
+      </x:c>
+      <x:c r="J91" s="41" t="s">
+        <x:v>412</x:v>
+      </x:c>
+      <x:c r="K91" s="2" t="s">
+        <x:v>413</x:v>
+      </x:c>
+      <x:c r="L91" s="3" t="s">
         <x:v>414</x:v>
-      </x:c>
-      <x:c r="J91" s="41" t="s">
-        <x:v>415</x:v>
-      </x:c>
-      <x:c r="K91" s="2" t="s">
-        <x:v>416</x:v>
-      </x:c>
-      <x:c r="L91" s="3" t="s">
-        <x:v>417</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="84">
       <x:c r="A92" s="53"/>
       <x:c r="B92" s="54"/>
       <x:c r="C92" s="57" t="s">
-        <x:v>418</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="D92" s="57" t="str">
         <x:v>BSTART.TEPL TCONCAT, DataType
@@ -6585,10 +6650,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="J92" s="41" t="s">
-        <x:v>419</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="K92" s="2" t="s">
-        <x:v>420</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="L92" s="3" t="s">
         <x:v>26</x:v>
@@ -6598,7 +6663,7 @@
       <x:c r="A93" s="53"/>
       <x:c r="B93" s="54"/>
       <x:c r="C93" s="57" t="s">
-        <x:v>421</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="D93" s="57" t="str">
         <x:v>BSTART.TEPL TTRANS, DataType
@@ -6608,7 +6673,7 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E93" s="17" t="s">
-        <x:v>422</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="F93" s="17" t="s">
         <x:v>74</x:v>
@@ -6616,23 +6681,23 @@
       <x:c r="G93" s="17"/>
       <x:c r="H93" s="17"/>
       <x:c r="I93" s="17" t="s">
+        <x:v>420</x:v>
+      </x:c>
+      <x:c r="J93" s="41" t="s">
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="K93" s="2" t="s">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="L93" s="3" t="s">
         <x:v>423</x:v>
-      </x:c>
-      <x:c r="J93" s="41" t="s">
-        <x:v>424</x:v>
-      </x:c>
-      <x:c r="K93" s="2" t="s">
-        <x:v>425</x:v>
-      </x:c>
-      <x:c r="L93" s="3" t="s">
-        <x:v>426</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="101.75">
       <x:c r="A94" s="53"/>
       <x:c r="B94" s="55"/>
       <x:c r="C94" s="58" t="s">
-        <x:v>427</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="D94" s="58" t="str">
         <x:v>BSTART.TEPL TIMG2COL, DataType
@@ -6643,33 +6708,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E94" s="25" t="s">
-        <x:v>428</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="F94" s="25" t="s">
-        <x:v>429</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="G94" s="25" t="s">
-        <x:v>430</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="H94" s="25"/>
       <x:c r="I94" s="25" t="s">
         <x:v>223</x:v>
       </x:c>
       <x:c r="J94" s="43" t="s">
-        <x:v>431</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="K94" s="2" t="s">
-        <x:v>432</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="L94" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>430</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="101.75">
       <x:c r="A95" s="53"/>
       <x:c r="B95" s="55"/>
       <x:c r="C95" s="43" t="s">
-        <x:v>434</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="D95" s="58" t="str">
         <x:v>BSTART.TEPL TMRGSORT, DataType
@@ -6680,35 +6745,35 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E95" s="25" t="s">
-        <x:v>435</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="F95" s="25" t="s">
-        <x:v>436</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="G95" s="25" t="s">
-        <x:v>437</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="H95" s="25"/>
       <x:c r="I95" s="25" t="s">
         <x:v>171</x:v>
       </x:c>
       <x:c r="J95" s="43" t="s">
-        <x:v>438</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="K95" s="2" t="s">
-        <x:v>439</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="L95" s="3" t="s">
-        <x:v>440</x:v>
+        <x:v>437</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="84">
       <x:c r="A96" s="53"/>
       <x:c r="B96" s="52" t="s">
-        <x:v>441</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="C96" s="40" t="s">
-        <x:v>442</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="D96" s="56" t="str">
         <x:v>BSTART.TEPL TPARTADD, DataType
@@ -6731,10 +6796,10 @@
         <x:v>117</x:v>
       </x:c>
       <x:c r="J96" s="40" t="s">
-        <x:v>443</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="K96" s="2" t="s">
-        <x:v>444</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="L96" s="3" t="s">
         <x:v>26</x:v>
@@ -6744,7 +6809,7 @@
       <x:c r="A97" s="53"/>
       <x:c r="B97" s="54"/>
       <x:c r="C97" s="41" t="s">
-        <x:v>445</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="D97" s="57" t="str">
         <x:v>BSTART.TEPL TPARTMUL, DataType
@@ -6767,10 +6832,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="J97" s="41" t="s">
-        <x:v>446</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="K97" s="2" t="s">
-        <x:v>447</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="L97" s="3" t="s">
         <x:v>26</x:v>
@@ -6780,7 +6845,7 @@
       <x:c r="A98" s="53"/>
       <x:c r="B98" s="54"/>
       <x:c r="C98" s="41" t="s">
-        <x:v>448</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D98" s="57" t="str">
         <x:v>BSTART.TEPL TPARTMAX, DataType
@@ -6803,10 +6868,10 @@
         <x:v>223</x:v>
       </x:c>
       <x:c r="J98" s="41" t="s">
-        <x:v>449</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="K98" s="2" t="s">
-        <x:v>450</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="L98" s="3" t="s">
         <x:v>26</x:v>
@@ -6816,7 +6881,7 @@
       <x:c r="A99" s="59"/>
       <x:c r="B99" s="55"/>
       <x:c r="C99" s="43" t="s">
-        <x:v>451</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="D99" s="58" t="str">
         <x:v>BSTART.TEPL TPARTMIN, DataType
@@ -6839,10 +6904,10 @@
         <x:v>223</x:v>
       </x:c>
       <x:c r="J99" s="43" t="s">
-        <x:v>452</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="K99" s="2" t="s">
-        <x:v>453</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="L99" s="3" t="s">
         <x:v>26</x:v>
@@ -7469,106 +7534,106 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>454</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>455</x:v>
+        <x:v>452</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26.399999618530273" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>456</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>457</x:v>
+        <x:v>454</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="26.399999618530273" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>458</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>459</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" customHeight="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>460</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>461</x:v>
+        <x:v>458</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.399999618530273" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>462</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>463</x:v>
+        <x:v>460</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>464</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>465</x:v>
+        <x:v>462</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>466</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>467</x:v>
+        <x:v>464</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>468</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>469</x:v>
+        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>470</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>471</x:v>
+        <x:v>468</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40.5" customHeight="1">
       <x:c r="A10" s="3" t="s">
-        <x:v>472</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
-        <x:v>473</x:v>
+        <x:v>470</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40.5" customHeight="1">
       <x:c r="A11" s="3" t="s">
-        <x:v>474</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
-        <x:v>475</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40.5" customHeight="1">
       <x:c r="A12" s="3" t="s">
-        <x:v>476</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
-        <x:v>477</x:v>
+        <x:v>474</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="40.5" customHeight="1">
       <x:c r="A13" s="3" t="s">
-        <x:v>478</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
-        <x:v>479</x:v>
+        <x:v>476</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7586,98 +7651,98 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>480</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>481</x:v>
+        <x:v>478</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="14" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>482</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>483</x:v>
+        <x:v>480</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="14" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>484</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>485</x:v>
+        <x:v>482</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="14" customHeight="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>486</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>487</x:v>
+        <x:v>484</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="14" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>488</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>489</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="14" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>490</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>491</x:v>
+        <x:v>488</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>492</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>493</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="14" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>494</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>495</x:v>
+        <x:v>492</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="14" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>496</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>497</x:v>
+        <x:v>494</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="14" customHeight="1">
       <x:c r="A10" s="2" t="s">
-        <x:v>498</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
-        <x:v>499</x:v>
+        <x:v>496</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="14" customHeight="1">
       <x:c r="A11" s="2" t="s">
-        <x:v>500</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>501</x:v>
+        <x:v>498</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="14" customHeight="1">
       <x:c r="A12" s="2" t="s">
-        <x:v>502</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>503</x:v>
+        <x:v>500</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: align PTO 0.58 release surfaces (#47)
## Summary
- remove stale implicit-ACC and 0.57.1 wording from active PTO 0.58
release surfaces
- correct active maturity counts to 87 TEPL and 12 CUBE operations while
retaining 10 TLSU operations, including masked gather/scatter and
gather-CAS
- refresh the controlled Excel projection and release manifest without
changing catalog, ASL, encodings, or CI

## Exact head
- commit: 072f33ae456db9980685296feaa2d2debe0f3a5b
- tree: 6819f712cd3a385bc1c26bf03793743547c08732

## Local validation
- intrinsic sync repeat dry-run: zero changes
- intrinsic sync audit: pass
- intrinsic documentation tests: 24/24 pass
- publication hygiene: pass
- repository gate: pass
- release manifest: PTO ISA 0.58.0, encoding
0d9dda5c9830c126f31febb67186067792e2994f5dae998c0e248c4bbe419e13
- workbook formula-error scan and rendered layout verification: pass

Co-authored-by: Codex Review <codex-review@example.invalid>
</commit_message>
<xml_diff>
--- a/spec/encoding/PTO-ISA-Encoding.xlsx
+++ b/spec/encoding/PTO-ISA-Encoding.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R77efea90e68d4cb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rd5d2a39aebb44e71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="Rfc64d61f63034444"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rf664057da7f640d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Ra3a3f0a762e44863"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R6213fd2065b34aca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -880,11 +880,6 @@
     <x:t xml:space="preserve">PE-local CUBE matrix multiply: C[i,j] = sum_k(A[i,k] * B[k,j]).</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">1. M/N/K are required 16-bit dims in B.DIM(LB0/LB1/LB2).
-2. M/N/K, fractal/layout, and dtype must satisfy the active CUBE target profile.
-3. ACC lifetime, precision, and export/convert follow the CUBE/ACC contract; ACCCVT writes ACC back to a normal Tile.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">TMATMUL_BIAS</x:t>
   </x:si>
   <x:si>
@@ -894,11 +889,6 @@
     <x:t xml:space="preserve">Matmul with bias add (tile world, ins/outs).</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">1. M/N/K are required 16-bit dims in B.DIM(LB0/LB1/LB2).
-2. M/N/K, fractal/layout, and dtype must satisfy the active CUBE target profile.
-3. ACC lifetime, precision, and export/convert behavior follow the CUBE/ACC contract.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">TMATMUL_ACC</x:t>
   </x:si>
   <x:si>
@@ -906,11 +896,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">PE-local CUBE matrix multiply accumulate; variant operands are profile-specific.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1. M/N/K are required 16-bit dims in B.DIM(LB0/LB1/LB2).
-2. Input 2 appears only when the opcode profile requires an input ACC, bias, scale, or other ExtraTile.
-3. Compiler scratch is not ISA-visible; this row does not define group-level GMMA/barrier semantics.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TMATMUL_MX</x:t>
@@ -5607,15 +5592,25 @@
       <x:c r="K68" s="2" t="s">
         <x:v>280</x:v>
       </x:c>
-      <x:c r="L68" s="3" t="s">
-        <x:v>281</x:v>
+      <x:c r="L68" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+Cooperative form 中 C/D、RowMaxIn/Out、GroupMaxOut 为 MShard4；Bias、vector QuantParam、vector PReLU 是四 PE 上内容相同的完整 Local N-vector；scalar GPR 参数也必须在四 PE 上相等。
+D 必须是显式 ordinary physical Local destination。
+Cooperative TMATMUL 的 Shared read 不修改 descriptor/payload；并发 overlap 由程序避免，且该 rendezvous 不建立 GM ordering。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="118">
       <x:c r="A69" s="46"/>
       <x:c r="B69" s="46"/>
       <x:c r="C69" s="16" t="s">
-        <x:v>282</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="D69" s="17" t="str">
         <x:v>BSTART.CUBE TMATMUL.BIAS AType
@@ -5649,20 +5644,30 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J69" s="41" t="s">
+        <x:v>282</x:v>
+      </x:c>
+      <x:c r="K69" s="2" t="s">
         <x:v>283</x:v>
       </x:c>
-      <x:c r="K69" s="2" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="L69" s="3" t="s">
-        <x:v>285</x:v>
+      <x:c r="L69" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+Cooperative form 中 C/D、RowMaxIn/Out、GroupMaxOut 为 MShard4；Bias、vector QuantParam、vector PReLU 是四 PE 上内容相同的完整 Local N-vector；scalar GPR 参数也必须在四 PE 上相等。
+D 必须是显式 ordinary physical Local destination。
+Cooperative TMATMUL 的 Shared read 不修改 descriptor/payload；并发 overlap 由程序避免，且该 rendezvous 不建立 GM ordering。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="118">
       <x:c r="A70" s="46"/>
       <x:c r="B70" s="46"/>
       <x:c r="C70" s="16" t="s">
-        <x:v>286</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="D70" s="17" t="str">
         <x:v>BSTART.CUBE TMATMUL.ACC AType
@@ -5696,20 +5701,30 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J70" s="41" t="s">
-        <x:v>287</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="K70" s="2" t="s">
-        <x:v>288</x:v>
-      </x:c>
-      <x:c r="L70" s="3" t="s">
-        <x:v>289</x:v>
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="L70" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+Cooperative form 中 C/D、RowMaxIn/Out、GroupMaxOut 为 MShard4；Bias、vector QuantParam、vector PReLU 是四 PE 上内容相同的完整 Local N-vector；scalar GPR 参数也必须在四 PE 上相等。
+D==C 仅在 D 保持 TileAcc role 且 dtype、shape、layout、allocation 完全相同时合法；实现必须 read-old/rename-new，禁止物理原地覆盖。C 不携带 partial-sum provenance 要求。
+Cooperative TMATMUL 的 Shared read 不修改 descriptor/payload；并发 overlap 由程序避免，且该 rendezvous 不建立 GM ordering。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="118.75">
       <x:c r="A71" s="46"/>
       <x:c r="B71" s="46"/>
       <x:c r="C71" s="16" t="s">
-        <x:v>290</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="D71" s="17" t="str">
         <x:v>BSTART.CUBE TMATMULMX AType
@@ -5744,22 +5759,32 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J71" s="41" t="s">
-        <x:v>291</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="K71" s="2" t="s">
-        <x:v>292</x:v>
-      </x:c>
-      <x:c r="L71" s="3" t="s">
-        <x:v>285</x:v>
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="L71" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+Cooperative form 中 C/D、RowMaxIn/Out、GroupMaxOut 为 MShard4；Bias、vector QuantParam、vector PReLU 是四 PE 上内容相同的完整 Local N-vector；scalar GPR 参数也必须在四 PE 上相等。
+D 必须是显式 ordinary physical Local destination。
+Cooperative TMATMUL 的 Shared read 不修改 descriptor/payload；并发 overlap 由程序避免，且该 rendezvous 不建立 GM ordering。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="101">
       <x:c r="A72" s="46"/>
       <x:c r="B72" s="46" t="s">
-        <x:v>293</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="C72" s="13" t="s">
-        <x:v>294</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="D72" s="9" t="str">
         <x:v>BSTART.CUBE TGEMV AType
@@ -5791,20 +5816,30 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J72" s="40" t="s">
-        <x:v>295</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="K72" s="2" t="s">
-        <x:v>296</x:v>
-      </x:c>
-      <x:c r="L72" s="3" t="s">
-        <x:v>285</x:v>
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="L72" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+所有 operand/output 都是单 PE Local Tile；M 固定为 1。
+D 必须是显式 ordinary physical Local destination。
+TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="118">
       <x:c r="A73" s="46"/>
       <x:c r="B73" s="46"/>
       <x:c r="C73" s="16" t="s">
-        <x:v>297</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="D73" s="17" t="str">
         <x:v>BSTART.CUBE TGEMV.BIAS AType
@@ -5837,20 +5872,30 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J73" s="41" t="s">
-        <x:v>298</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="K73" s="2" t="s">
-        <x:v>299</x:v>
-      </x:c>
-      <x:c r="L73" s="3" t="s">
-        <x:v>285</x:v>
+        <x:v>296</x:v>
+      </x:c>
+      <x:c r="L73" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+所有 operand/output 都是单 PE Local Tile；M 固定为 1。
+D 必须是显式 ordinary physical Local destination。
+TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="118">
       <x:c r="A74" s="46"/>
       <x:c r="B74" s="46"/>
       <x:c r="C74" s="16" t="s">
-        <x:v>300</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="D74" s="17" t="str">
         <x:v>BSTART.CUBE TGEMV.ACC AType
@@ -5883,20 +5928,30 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J74" s="41" t="s">
-        <x:v>301</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="K74" s="2" t="s">
-        <x:v>302</x:v>
-      </x:c>
-      <x:c r="L74" s="3" t="s">
-        <x:v>285</x:v>
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="L74" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+所有 operand/output 都是单 PE Local Tile；M 固定为 1。
+D==C 仅在 D 保持 TileAcc role 且 dtype、shape、layout、allocation 完全相同时合法；实现必须 read-old/rename-new，禁止物理原地覆盖。C 不携带 partial-sum provenance 要求。
+TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="101.75">
       <x:c r="A75" s="47"/>
       <x:c r="B75" s="47"/>
       <x:c r="C75" s="24" t="s">
-        <x:v>303</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="D75" s="25" t="str">
         <x:v>BSTART.CUBE TGEMVMX AType
@@ -5930,24 +5985,34 @@
         <x:v>AccType S32 or F32; DType is AccType for canonical None and otherwise follows PostProcessConfig</x:v>
       </x:c>
       <x:c r="J75" s="43" t="s">
-        <x:v>304</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="K75" s="2" t="s">
-        <x:v>305</x:v>
-      </x:c>
-      <x:c r="L75" s="3" t="s">
-        <x:v>285</x:v>
+        <x:v>302</x:v>
+      </x:c>
+      <x:c r="L75" s="3" t="str">
+        <x:v>AccType 只允许 S32/F32；C（若存在）必须为 M×N ND AccType Local Tile。U32 accumulator 非法。
+canonical None 为 PreQuant=None、ReLU=None、RMode=NONE、Sat=0；D 保持 AccType 与逻辑 TileAcc role。RowMax/GroupMax 可独立启用且不改变 D role。
+任一 quant、convert 或 ReLU 使 D 成为由 PostProcess 推导 dtype 的 ordinary ND Tile。
+RowMax/GroupMax 在 ReLU、quant、convert 前观察 P。RowMaxIn/Out 为 M×1；GroupMaxOut 为 M×ceil(N/GroupN)。
+verifier 必须按 config 检查精确 source/destination arity，不接受闲置 operand。
+D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
+所有 operand/output 都是单 PE Local Tile；M 固定为 1。
+D 必须是显式 ordinary physical Local destination。
+TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
+nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="101">
       <x:c r="A76" s="48" t="s">
-        <x:v>306</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="B76" s="48" t="s">
-        <x:v>307</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="C76" s="13" t="s">
-        <x:v>308</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="D76" s="9" t="str">
         <x:v>Local form
@@ -5977,20 +6042,20 @@
         <x:v>PTO TLOAD dtype/layout combinations supported by the v5 TLSU profile</x:v>
       </x:c>
       <x:c r="J76" s="40" t="s">
-        <x:v>309</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="K76" s="2" t="s">
-        <x:v>310</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="L76" s="3" t="s">
-        <x:v>311</x:v>
+        <x:v>308</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="101">
       <x:c r="A77" s="49"/>
       <x:c r="B77" s="49"/>
       <x:c r="C77" s="16" t="s">
-        <x:v>312</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="D77" s="17" t="str">
         <x:v>Local form
@@ -6028,17 +6093,17 @@
         <x:v>TLSU Function 1; Shared pe_scope Function 14;</x:v>
       </x:c>
       <x:c r="K77" s="2" t="s">
-        <x:v>313</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="L77" s="3" t="s">
-        <x:v>314</x:v>
+        <x:v>311</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="101.75">
       <x:c r="A78" s="49"/>
       <x:c r="B78" s="49"/>
       <x:c r="C78" s="16" t="s">
-        <x:v>315</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="D78" s="17" t="str">
         <x:v>BSTART.TLSU TPREFETCH, DataType
@@ -6049,35 +6114,35 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E78" s="17" t="s">
-        <x:v>316</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="F78" s="17" t="s">
-        <x:v>317</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="G78" s="17" t="s">
-        <x:v>318</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="H78" s="17"/>
       <x:c r="I78" s="17" t="s">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="J78" s="41" t="s">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="K78" s="2" t="s">
+        <x:v>318</x:v>
+      </x:c>
+      <x:c r="L78" s="3" t="s">
         <x:v>319</x:v>
-      </x:c>
-      <x:c r="J78" s="41" t="s">
-        <x:v>320</x:v>
-      </x:c>
-      <x:c r="K78" s="2" t="s">
-        <x:v>321</x:v>
-      </x:c>
-      <x:c r="L78" s="3" t="s">
-        <x:v>322</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="101">
       <x:c r="A79" s="49"/>
       <x:c r="B79" s="48" t="s">
-        <x:v>323</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C79" s="16" t="s">
-        <x:v>324</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="D79" s="17" t="str">
         <x:v>BSTART.TLSU MGATHER, DataType
@@ -6091,30 +6156,30 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F79" s="17" t="s">
-        <x:v>325</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="G79" s="17" t="s">
-        <x:v>326</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="H79" s="17"/>
       <x:c r="I79" s="17" t="s">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="J79" s="41" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="K79" s="2" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="L79" s="3" t="s">
         <x:v>327</x:v>
-      </x:c>
-      <x:c r="J79" s="41" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="K79" s="2" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="L79" s="3" t="s">
-        <x:v>330</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="101.75">
       <x:c r="A80" s="50"/>
       <x:c r="B80" s="50"/>
       <x:c r="C80" s="16" t="s">
-        <x:v>331</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="D80" s="17" t="str">
         <x:v>BSTART.TLSU MSCATTER, DataType
@@ -6125,37 +6190,37 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E80" s="17" t="s">
-        <x:v>332</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="F80" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G80" s="17" t="s">
-        <x:v>326</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="H80" s="17"/>
       <x:c r="I80" s="17" t="s">
-        <x:v>333</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="J80" s="41" t="s">
-        <x:v>334</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="K80" s="2" t="s">
-        <x:v>335</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="L80" s="3" t="s">
-        <x:v>330</x:v>
+        <x:v>327</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="101">
       <x:c r="A81" s="51" t="s">
-        <x:v>336</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="B81" s="52" t="s">
-        <x:v>337</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="C81" s="13" t="s">
-        <x:v>338</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="D81" s="9" t="str">
         <x:v>BSTART.TEPL TEXPANDS, DataType
@@ -6169,18 +6234,18 @@
         <x:v>221</x:v>
       </x:c>
       <x:c r="F81" s="9" t="s">
-        <x:v>339</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="G81" s="9"/>
       <x:c r="H81" s="9"/>
       <x:c r="I81" s="9" t="s">
-        <x:v>340</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="J81" s="40" t="s">
-        <x:v>341</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="K81" s="2" t="s">
-        <x:v>342</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="L81" s="3" t="s">
         <x:v>71</x:v>
@@ -6190,7 +6255,7 @@
       <x:c r="A82" s="53"/>
       <x:c r="B82" s="54"/>
       <x:c r="C82" s="16" t="s">
-        <x:v>343</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D82" s="17" t="str">
         <x:v>BSTART.TEPL TCI, DataType
@@ -6201,33 +6266,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E82" s="17" t="s">
-        <x:v>344</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="F82" s="17" t="s">
-        <x:v>345</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="G82" s="17" t="s">
-        <x:v>346</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="H82" s="17"/>
       <x:c r="I82" s="17" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="J82" s="41" t="s">
+        <x:v>345</x:v>
+      </x:c>
+      <x:c r="K82" s="2" t="s">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="L82" s="3" t="s">
         <x:v>347</x:v>
-      </x:c>
-      <x:c r="J82" s="41" t="s">
-        <x:v>348</x:v>
-      </x:c>
-      <x:c r="K82" s="2" t="s">
-        <x:v>349</x:v>
-      </x:c>
-      <x:c r="L82" s="3" t="s">
-        <x:v>350</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="101">
       <x:c r="A83" s="53"/>
       <x:c r="B83" s="54"/>
       <x:c r="C83" s="16" t="s">
-        <x:v>351</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="D83" s="17" t="str">
         <x:v>BSTART.TEPL TTRI, DataType
@@ -6238,33 +6303,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E83" s="17" t="s">
-        <x:v>352</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="F83" s="17" t="s">
-        <x:v>353</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="G83" s="17" t="s">
-        <x:v>354</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="H83" s="17"/>
       <x:c r="I83" s="17" t="s">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="J83" s="41" t="s">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="K83" s="2" t="s">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="L83" s="3" t="s">
         <x:v>355</x:v>
-      </x:c>
-      <x:c r="J83" s="41" t="s">
-        <x:v>356</x:v>
-      </x:c>
-      <x:c r="K83" s="2" t="s">
-        <x:v>357</x:v>
-      </x:c>
-      <x:c r="L83" s="3" t="s">
-        <x:v>358</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="84.75">
       <x:c r="A84" s="53"/>
       <x:c r="B84" s="55"/>
       <x:c r="C84" s="24" t="s">
-        <x:v>359</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="D84" s="25" t="str">
         <x:v>BSTART.TEPL TFILLPAD, DataType
@@ -6274,35 +6339,35 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E84" s="25" t="s">
-        <x:v>360</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="F84" s="25" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G84" s="25" t="s">
-        <x:v>361</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="H84" s="25"/>
       <x:c r="I84" s="25" t="s">
+        <x:v>359</x:v>
+      </x:c>
+      <x:c r="J84" s="43" t="s">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="K84" s="2" t="s">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="L84" s="3" t="s">
         <x:v>362</x:v>
-      </x:c>
-      <x:c r="J84" s="43" t="s">
-        <x:v>363</x:v>
-      </x:c>
-      <x:c r="K84" s="2" t="s">
-        <x:v>364</x:v>
-      </x:c>
-      <x:c r="L84" s="3" t="s">
-        <x:v>365</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="118">
       <x:c r="A85" s="53"/>
       <x:c r="B85" s="52" t="s">
-        <x:v>366</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="C85" s="13" t="s">
-        <x:v>367</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="D85" s="17" t="str">
         <x:v>BSTART.TEPL TCVT, DataType
@@ -6312,33 +6377,33 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E85" s="17" t="s">
-        <x:v>368</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="F85" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G85" s="17" t="s">
-        <x:v>369</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="H85" s="17"/>
       <x:c r="I85" s="17" t="s">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="J85" s="41" t="s">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="K85" s="2" t="s">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="L85" s="3" t="s">
         <x:v>370</x:v>
-      </x:c>
-      <x:c r="J85" s="41" t="s">
-        <x:v>371</x:v>
-      </x:c>
-      <x:c r="K85" s="2" t="s">
-        <x:v>372</x:v>
-      </x:c>
-      <x:c r="L85" s="3" t="s">
-        <x:v>373</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="84">
       <x:c r="A86" s="53"/>
       <x:c r="B86" s="54"/>
       <x:c r="C86" s="16" t="s">
-        <x:v>374</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="D86" s="17" t="str">
         <x:v>BSTART.TEPL TQUANT, DataType
@@ -6348,35 +6413,35 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E86" s="17" t="s">
-        <x:v>375</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="F86" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G86" s="17" t="s">
-        <x:v>376</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="H86" s="17" t="str">
         <x:v>offset/scaling/index Tile (optional)</x:v>
       </x:c>
       <x:c r="I86" s="17" t="s">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="J86" s="41" t="s">
+        <x:v>375</x:v>
+      </x:c>
+      <x:c r="K86" s="2" t="s">
+        <x:v>376</x:v>
+      </x:c>
+      <x:c r="L86" s="3" t="s">
         <x:v>377</x:v>
-      </x:c>
-      <x:c r="J86" s="41" t="s">
-        <x:v>378</x:v>
-      </x:c>
-      <x:c r="K86" s="2" t="s">
-        <x:v>379</x:v>
-      </x:c>
-      <x:c r="L86" s="3" t="s">
-        <x:v>380</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="84.75">
       <x:c r="A87" s="53"/>
       <x:c r="B87" s="55"/>
       <x:c r="C87" s="16" t="s">
-        <x:v>381</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="D87" s="17" t="str">
         <x:v>BSTART.TEPL TDEQUANT, DataType
@@ -6386,37 +6451,37 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E87" s="17" t="s">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="F87" s="17" t="s">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="G87" s="17" t="s">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="H87" s="17" t="s">
         <x:v>382</x:v>
       </x:c>
-      <x:c r="F87" s="17" t="s">
+      <x:c r="I87" s="17" t="s">
         <x:v>383</x:v>
       </x:c>
-      <x:c r="G87" s="17" t="s">
+      <x:c r="J87" s="41" t="s">
         <x:v>384</x:v>
       </x:c>
-      <x:c r="H87" s="17" t="s">
+      <x:c r="K87" s="2" t="s">
         <x:v>385</x:v>
       </x:c>
-      <x:c r="I87" s="17" t="s">
+      <x:c r="L87" s="3" t="s">
         <x:v>386</x:v>
-      </x:c>
-      <x:c r="J87" s="41" t="s">
-        <x:v>387</x:v>
-      </x:c>
-      <x:c r="K87" s="2" t="s">
-        <x:v>388</x:v>
-      </x:c>
-      <x:c r="L87" s="3" t="s">
-        <x:v>389</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="101">
       <x:c r="A88" s="53"/>
       <x:c r="B88" s="52" t="s">
-        <x:v>390</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="C88" s="56" t="s">
-        <x:v>391</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="D88" s="56" t="str">
         <x:v>BSTART.TEPL TEXTRACT, DataType
@@ -6427,33 +6492,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E88" s="9" t="s">
-        <x:v>392</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="F88" s="9" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G88" s="9" t="s">
-        <x:v>393</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="H88" s="9"/>
       <x:c r="I88" s="9" t="s">
+        <x:v>391</x:v>
+      </x:c>
+      <x:c r="J88" s="40" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="K88" s="2" t="s">
+        <x:v>393</x:v>
+      </x:c>
+      <x:c r="L88" s="3" t="s">
         <x:v>394</x:v>
-      </x:c>
-      <x:c r="J88" s="40" t="s">
-        <x:v>395</x:v>
-      </x:c>
-      <x:c r="K88" s="2" t="s">
-        <x:v>396</x:v>
-      </x:c>
-      <x:c r="L88" s="3" t="s">
-        <x:v>397</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="101">
       <x:c r="A89" s="53"/>
       <x:c r="B89" s="54"/>
       <x:c r="C89" s="57" t="s">
-        <x:v>398</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D89" s="57" t="str">
         <x:v>BSTART.TEPL TINSERT, DataType
@@ -6467,30 +6532,30 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F89" s="17" t="s">
-        <x:v>399</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G89" s="17" t="s">
-        <x:v>393</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="H89" s="17"/>
       <x:c r="I89" s="17" t="s">
+        <x:v>397</x:v>
+      </x:c>
+      <x:c r="J89" s="41" t="s">
+        <x:v>398</x:v>
+      </x:c>
+      <x:c r="K89" s="2" t="s">
+        <x:v>399</x:v>
+      </x:c>
+      <x:c r="L89" s="3" t="s">
         <x:v>400</x:v>
-      </x:c>
-      <x:c r="J89" s="41" t="s">
-        <x:v>401</x:v>
-      </x:c>
-      <x:c r="K89" s="2" t="s">
-        <x:v>402</x:v>
-      </x:c>
-      <x:c r="L89" s="3" t="s">
-        <x:v>403</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="101">
       <x:c r="A90" s="53"/>
       <x:c r="B90" s="54"/>
       <x:c r="C90" s="57" t="s">
-        <x:v>404</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="D90" s="57" t="str">
         <x:v>BSTART.TEPL TGATHER, DataType
@@ -6500,33 +6565,33 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E90" s="17" t="s">
-        <x:v>405</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="F90" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G90" s="17" t="s">
-        <x:v>406</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="H90" s="17"/>
       <x:c r="I90" s="17" t="s">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="J90" s="41" t="s">
+        <x:v>405</x:v>
+      </x:c>
+      <x:c r="K90" s="2" t="s">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="L90" s="3" t="s">
         <x:v>407</x:v>
-      </x:c>
-      <x:c r="J90" s="41" t="s">
-        <x:v>408</x:v>
-      </x:c>
-      <x:c r="K90" s="2" t="s">
-        <x:v>409</x:v>
-      </x:c>
-      <x:c r="L90" s="3" t="s">
-        <x:v>410</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="84">
       <x:c r="A91" s="53"/>
       <x:c r="B91" s="54"/>
       <x:c r="C91" s="57" t="s">
-        <x:v>411</x:v>
+        <x:v>408</x:v>
       </x:c>
       <x:c r="D91" s="57" t="str">
         <x:v>BSTART.TEPL TSCATTER, DataType
@@ -6536,33 +6601,33 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E91" s="17" t="s">
-        <x:v>412</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="F91" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G91" s="17" t="s">
-        <x:v>413</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="H91" s="17"/>
       <x:c r="I91" s="17" t="s">
+        <x:v>411</x:v>
+      </x:c>
+      <x:c r="J91" s="41" t="s">
+        <x:v>412</x:v>
+      </x:c>
+      <x:c r="K91" s="2" t="s">
+        <x:v>413</x:v>
+      </x:c>
+      <x:c r="L91" s="3" t="s">
         <x:v>414</x:v>
-      </x:c>
-      <x:c r="J91" s="41" t="s">
-        <x:v>415</x:v>
-      </x:c>
-      <x:c r="K91" s="2" t="s">
-        <x:v>416</x:v>
-      </x:c>
-      <x:c r="L91" s="3" t="s">
-        <x:v>417</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="84">
       <x:c r="A92" s="53"/>
       <x:c r="B92" s="54"/>
       <x:c r="C92" s="57" t="s">
-        <x:v>418</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="D92" s="57" t="str">
         <x:v>BSTART.TEPL TCONCAT, DataType
@@ -6585,10 +6650,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="J92" s="41" t="s">
-        <x:v>419</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="K92" s="2" t="s">
-        <x:v>420</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="L92" s="3" t="s">
         <x:v>26</x:v>
@@ -6598,7 +6663,7 @@
       <x:c r="A93" s="53"/>
       <x:c r="B93" s="54"/>
       <x:c r="C93" s="57" t="s">
-        <x:v>421</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="D93" s="57" t="str">
         <x:v>BSTART.TEPL TTRANS, DataType
@@ -6608,7 +6673,7 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E93" s="17" t="s">
-        <x:v>422</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="F93" s="17" t="s">
         <x:v>74</x:v>
@@ -6616,23 +6681,23 @@
       <x:c r="G93" s="17"/>
       <x:c r="H93" s="17"/>
       <x:c r="I93" s="17" t="s">
+        <x:v>420</x:v>
+      </x:c>
+      <x:c r="J93" s="41" t="s">
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="K93" s="2" t="s">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="L93" s="3" t="s">
         <x:v>423</x:v>
-      </x:c>
-      <x:c r="J93" s="41" t="s">
-        <x:v>424</x:v>
-      </x:c>
-      <x:c r="K93" s="2" t="s">
-        <x:v>425</x:v>
-      </x:c>
-      <x:c r="L93" s="3" t="s">
-        <x:v>426</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="101.75">
       <x:c r="A94" s="53"/>
       <x:c r="B94" s="55"/>
       <x:c r="C94" s="58" t="s">
-        <x:v>427</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="D94" s="58" t="str">
         <x:v>BSTART.TEPL TIMG2COL, DataType
@@ -6643,33 +6708,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E94" s="25" t="s">
-        <x:v>428</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="F94" s="25" t="s">
-        <x:v>429</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="G94" s="25" t="s">
-        <x:v>430</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="H94" s="25"/>
       <x:c r="I94" s="25" t="s">
         <x:v>223</x:v>
       </x:c>
       <x:c r="J94" s="43" t="s">
-        <x:v>431</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="K94" s="2" t="s">
-        <x:v>432</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="L94" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>430</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="101.75">
       <x:c r="A95" s="53"/>
       <x:c r="B95" s="55"/>
       <x:c r="C95" s="43" t="s">
-        <x:v>434</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="D95" s="58" t="str">
         <x:v>BSTART.TEPL TMRGSORT, DataType
@@ -6680,35 +6745,35 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E95" s="25" t="s">
-        <x:v>435</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="F95" s="25" t="s">
-        <x:v>436</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="G95" s="25" t="s">
-        <x:v>437</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="H95" s="25"/>
       <x:c r="I95" s="25" t="s">
         <x:v>171</x:v>
       </x:c>
       <x:c r="J95" s="43" t="s">
-        <x:v>438</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="K95" s="2" t="s">
-        <x:v>439</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="L95" s="3" t="s">
-        <x:v>440</x:v>
+        <x:v>437</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="84">
       <x:c r="A96" s="53"/>
       <x:c r="B96" s="52" t="s">
-        <x:v>441</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="C96" s="40" t="s">
-        <x:v>442</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="D96" s="56" t="str">
         <x:v>BSTART.TEPL TPARTADD, DataType
@@ -6731,10 +6796,10 @@
         <x:v>117</x:v>
       </x:c>
       <x:c r="J96" s="40" t="s">
-        <x:v>443</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="K96" s="2" t="s">
-        <x:v>444</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="L96" s="3" t="s">
         <x:v>26</x:v>
@@ -6744,7 +6809,7 @@
       <x:c r="A97" s="53"/>
       <x:c r="B97" s="54"/>
       <x:c r="C97" s="41" t="s">
-        <x:v>445</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="D97" s="57" t="str">
         <x:v>BSTART.TEPL TPARTMUL, DataType
@@ -6767,10 +6832,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="J97" s="41" t="s">
-        <x:v>446</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="K97" s="2" t="s">
-        <x:v>447</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="L97" s="3" t="s">
         <x:v>26</x:v>
@@ -6780,7 +6845,7 @@
       <x:c r="A98" s="53"/>
       <x:c r="B98" s="54"/>
       <x:c r="C98" s="41" t="s">
-        <x:v>448</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D98" s="57" t="str">
         <x:v>BSTART.TEPL TPARTMAX, DataType
@@ -6803,10 +6868,10 @@
         <x:v>223</x:v>
       </x:c>
       <x:c r="J98" s="41" t="s">
-        <x:v>449</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="K98" s="2" t="s">
-        <x:v>450</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="L98" s="3" t="s">
         <x:v>26</x:v>
@@ -6816,7 +6881,7 @@
       <x:c r="A99" s="59"/>
       <x:c r="B99" s="55"/>
       <x:c r="C99" s="43" t="s">
-        <x:v>451</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="D99" s="58" t="str">
         <x:v>BSTART.TEPL TPARTMIN, DataType
@@ -6839,10 +6904,10 @@
         <x:v>223</x:v>
       </x:c>
       <x:c r="J99" s="43" t="s">
-        <x:v>452</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="K99" s="2" t="s">
-        <x:v>453</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="L99" s="3" t="s">
         <x:v>26</x:v>
@@ -7469,106 +7534,106 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>454</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>455</x:v>
+        <x:v>452</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26.399999618530273" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>456</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>457</x:v>
+        <x:v>454</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="26.399999618530273" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>458</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>459</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" customHeight="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>460</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>461</x:v>
+        <x:v>458</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.399999618530273" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>462</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>463</x:v>
+        <x:v>460</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>464</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>465</x:v>
+        <x:v>462</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>466</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>467</x:v>
+        <x:v>464</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>468</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>469</x:v>
+        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>470</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>471</x:v>
+        <x:v>468</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40.5" customHeight="1">
       <x:c r="A10" s="3" t="s">
-        <x:v>472</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
-        <x:v>473</x:v>
+        <x:v>470</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40.5" customHeight="1">
       <x:c r="A11" s="3" t="s">
-        <x:v>474</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
-        <x:v>475</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40.5" customHeight="1">
       <x:c r="A12" s="3" t="s">
-        <x:v>476</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
-        <x:v>477</x:v>
+        <x:v>474</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="40.5" customHeight="1">
       <x:c r="A13" s="3" t="s">
-        <x:v>478</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
-        <x:v>479</x:v>
+        <x:v>476</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7586,98 +7651,98 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>480</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>481</x:v>
+        <x:v>478</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="14" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>482</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>483</x:v>
+        <x:v>480</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="14" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>484</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>485</x:v>
+        <x:v>482</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="14" customHeight="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>486</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>487</x:v>
+        <x:v>484</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="14" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>488</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>489</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="14" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>490</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>491</x:v>
+        <x:v>488</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>492</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>493</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="14" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>494</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>495</x:v>
+        <x:v>492</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="14" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>496</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>497</x:v>
+        <x:v>494</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="14" customHeight="1">
       <x:c r="A10" s="2" t="s">
-        <x:v>498</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
-        <x:v>499</x:v>
+        <x:v>496</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="14" customHeight="1">
       <x:c r="A11" s="2" t="s">
-        <x:v>500</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>501</x:v>
+        <x:v>498</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="14" customHeight="1">
       <x:c r="A12" s="2" t="s">
-        <x:v>502</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>503</x:v>
+        <x:v>500</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
spec: reissue 0.58 with PE-local B.IOS
</commit_message>
<xml_diff>
--- a/spec/encoding/PTO-ISA-Encoding.xlsx
+++ b/spec/encoding/PTO-ISA-Encoding.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rf664057da7f640d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Ra3a3f0a762e44863"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R6213fd2065b34aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5db740adfcf441f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="R3dd93611e07a44e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R391f2a71df774264"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1487,9 +1487,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Common allocation size</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">DavinciOO active PE-local profile permits B.IOT.imm4=3..9 only, corresponding to output Tile allocation size 128 B..8 KB. Source: intrinsic/header/B.IOT.md</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Common B.DIM contract</x:t>
@@ -5563,7 +5560,7 @@
 B.DIM LB0 M
 B.DIM LB1 N
 B.DIM LB2 K
-C.B.IOS Shared operand binder (optional)
+B.IOS Shared operand binder (optional)
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
@@ -5619,7 +5616,7 @@
 B.DIM LB0 M
 B.DIM LB1 N
 B.DIM LB2 K
-C.B.IOS Shared operand binder (optional)
+B.IOS Shared operand binder (optional)
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
@@ -5676,7 +5673,7 @@
 B.DIM LB0 M
 B.DIM LB1 N
 B.DIM LB2 K
-C.B.IOS Shared operand binder (optional)
+B.IOS Shared operand binder (optional)
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
@@ -5733,7 +5730,7 @@
 B.DIM LB0 M
 B.DIM LB1 N
 B.DIM LB2 K
-C.B.IOS Shared operand binder (optional)
+B.IOS Shared operand binder (optional)
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
@@ -5830,7 +5827,7 @@
 D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
 所有 operand/output 都是单 PE Local Tile；M 固定为 1。
 D 必须是显式 ordinary physical Local destination。
-TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+TGEMV 禁止所有 SharedTile、B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
 一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
@@ -5886,7 +5883,7 @@
 D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
 所有 operand/output 都是单 PE Local Tile；M 固定为 1。
 D 必须是显式 ordinary physical Local destination。
-TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+TGEMV 禁止所有 SharedTile、B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
 一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
@@ -5942,7 +5939,7 @@
 D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
 所有 operand/output 都是单 PE Local Tile；M 固定为 1。
 D==C 仅在 D 保持 TileAcc role 且 dtype、shape、layout、allocation 完全相同时合法；实现必须 read-old/rename-new，禁止物理原地覆盖。C 不携带 partial-sum provenance 要求。
-TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+TGEMV 禁止所有 SharedTile、B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
 一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
@@ -5999,7 +5996,7 @@
 D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
 所有 operand/output 都是单 PE Local Tile；M 固定为 1。
 D 必须是显式 ordinary physical Local destination。
-TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+TGEMV 禁止所有 SharedTile、B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
 一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
@@ -6023,7 +6020,7 @@
 Shared form
 BSTART.TLSU TLOAD
 B.DATR/B.DIM
-C.B.IOS
+B.IOS
 B.IOR</x:v>
       </x:c>
       <x:c r="E76" s="9" t="str">
@@ -6065,11 +6062,11 @@
 B.IOR
 Shared full form
 BSTART.TLSU Function 1
-C.B.IOS
+B.IOS
 B.IOR
 Shared pe_scope form
 BSTART.TLSU Function 14
-C.B.IOS
+B.IOS
 B.IOR</x:v>
       </x:c>
       <x:c r="E77" s="17" t="str">
@@ -6971,7 +6968,7 @@
 D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
 所有 operand/output 都是单 PE Local Tile；M 固定为 1。
 D==C 仅在 D 保持 TileAcc role 且 dtype、shape、layout、allocation 完全相同时合法；实现必须 read-old/rename-new，禁止物理原地覆盖。C 不携带 partial-sum provenance 要求。
-TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+TGEMV 禁止所有 SharedTile、B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
 一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
@@ -7034,7 +7031,7 @@
 D、RowMaxOut、GroupMaxOut 同时 ready，并在 retire/flush 上作为一个原子结果组处理。
 所有 operand/output 都是单 PE Local Tile；M 固定为 1。
 D 必须是显式 ordinary physical Local destination。
-TGEMV 禁止所有 SharedTile、C.B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
+TGEMV 禁止所有 SharedTile、B.IOS 和 core rendezvous；K blocking 通过每 PE 显式 TGEMV_ACC(D,C,A,B) 链完成。
 一个 block 中最后一条 B.IOT 必须设置 last；M/N/K、fractal、layout 与 Tile size 必须满足 CUBE profile。
 nondefault AccPhase 一律拒绝；K blocking 使用显式 _ACC(D,C,...)。</x:v>
       </x:c>
@@ -7057,7 +7054,7 @@
 B.DIM LB0 M
 B.DIM LB1 N
 B.DIM LB2 K
-C.B.IOS Shared operand binder (optional)
+B.IOS Shared operand binder (optional)
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
@@ -7121,7 +7118,7 @@
 B.DIM LB0 M
 B.DIM LB1 N
 B.DIM LB2 K
-C.B.IOS Shared operand binder (optional)
+B.IOS Shared operand binder (optional)
 B.IOT Local sources and Local outputs
 B.IOR scalar PostProcess parameter (optional)</x:v>
       </x:c>
@@ -7240,7 +7237,7 @@
         <x:v>byte-preserving; descriptors must be compatible</x:v>
       </x:c>
       <x:c r="J105" s="83" t="str">
-        <x:v>TLSU Function 2, Shared Functions 8–11;</x:v>
+        <x:v>TLSU Function 2, Shared Functions 9–12;</x:v>
       </x:c>
       <x:c r="K105" s="90" t="str">
         <x:v>Ordinary PTO TMOV(dst,src) remains a Local Tile move/conversion. DavinciOO v5 adds strongly typed Local↔Shared forms under the same intrinsic name; no _SHARED operation is introduced.</x:v>
@@ -7616,24 +7613,24 @@
       <x:c r="A11" s="3" t="s">
         <x:v>471</x:v>
       </x:c>
-      <x:c r="B11" s="3" t="s">
-        <x:v>472</x:v>
+      <x:c r="B11" s="3" t="str">
+        <x:v>PTO ISA 0.58 uses B.IOT.TSize=001..111 for 128 B..8 KiB per selected PE; B.IOS uses the same per-PE TSize table for Shared destinations. Core allocation is popcount(PE_MASK) times the per-PE size. Source: docs/instructions/block/operands/B.IOT.md and B.IOS.md</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40.5" customHeight="1">
       <x:c r="A12" s="3" t="s">
+        <x:v>472</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="s">
         <x:v>473</x:v>
-      </x:c>
-      <x:c r="B12" s="3" t="s">
-        <x:v>474</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="40.5" customHeight="1">
       <x:c r="A13" s="3" t="s">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="s">
         <x:v>475</x:v>
-      </x:c>
-      <x:c r="B13" s="3" t="s">
-        <x:v>476</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7651,98 +7648,98 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
+        <x:v>476</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
         <x:v>477</x:v>
-      </x:c>
-      <x:c r="B1" s="1" t="s">
-        <x:v>478</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="14" customHeight="1">
       <x:c r="A2" s="2" t="s">
+        <x:v>478</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="s">
         <x:v>479</x:v>
-      </x:c>
-      <x:c r="B2" s="2" t="s">
-        <x:v>480</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="14" customHeight="1">
       <x:c r="A3" s="2" t="s">
+        <x:v>480</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
         <x:v>481</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>482</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="14" customHeight="1">
       <x:c r="A4" s="2" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="s">
         <x:v>483</x:v>
-      </x:c>
-      <x:c r="B4" s="2" t="s">
-        <x:v>484</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="14" customHeight="1">
       <x:c r="A5" s="2" t="s">
+        <x:v>484</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="s">
         <x:v>485</x:v>
-      </x:c>
-      <x:c r="B5" s="2" t="s">
-        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="14" customHeight="1">
       <x:c r="A6" s="2" t="s">
+        <x:v>486</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="s">
         <x:v>487</x:v>
-      </x:c>
-      <x:c r="B6" s="2" t="s">
-        <x:v>488</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="s">
         <x:v>489</x:v>
-      </x:c>
-      <x:c r="B7" s="2" t="s">
-        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="14" customHeight="1">
       <x:c r="A8" s="2" t="s">
+        <x:v>490</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="s">
         <x:v>491</x:v>
-      </x:c>
-      <x:c r="B8" s="2" t="s">
-        <x:v>492</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="14" customHeight="1">
       <x:c r="A9" s="2" t="s">
+        <x:v>492</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="s">
         <x:v>493</x:v>
-      </x:c>
-      <x:c r="B9" s="2" t="s">
-        <x:v>494</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="14" customHeight="1">
       <x:c r="A10" s="2" t="s">
+        <x:v>494</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="s">
         <x:v>495</x:v>
-      </x:c>
-      <x:c r="B10" s="2" t="s">
-        <x:v>496</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="14" customHeight="1">
       <x:c r="A11" s="2" t="s">
+        <x:v>496</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="s">
         <x:v>497</x:v>
-      </x:c>
-      <x:c r="B11" s="2" t="s">
-        <x:v>498</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="14" customHeight="1">
       <x:c r="A12" s="2" t="s">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="s">
         <x:v>499</x:v>
-      </x:c>
-      <x:c r="B12" s="2" t="s">
-        <x:v>500</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
arch: reconcile PTO ISA 0.58 draft contracts
</commit_message>
<xml_diff>
--- a/spec/encoding/PTO-ISA-Encoding.xlsx
+++ b/spec/encoding/PTO-ISA-Encoding.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6f8d8ab6d45b4199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rce61c905a5d940fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R691a09b226ca4fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2405572ca20642db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="R7687975b46a142b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R71e1682035664704"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -977,20 +977,10 @@
     <x:t xml:space="preserve">PTO data load operation (Dimension Collapse: PartitionView -&gt; TileBuf).</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">1. 1D may declare B.DIM LB0 only; 2D uses B.DIM LB0/LB1/LB2 and ValidCol &lt;= Col.
-2. TLOAD has no Tile source operand; B.IOT declares the destination Tile only.
-3. GM address/stride, alignment, layout conversion, dtype, and access size must satisfy the PTO page and active TLSU target profile.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">TSTORE</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">PTO data store operation (TileBuf -&gt; PartitionView).</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1. 1D may declare B.DIM LB0 only; 2D uses B.DIM LB0/LB1/LB2 and ValidCol &lt;= Col.
-2. TSTORE has no ordinary Tile destination; the result is a memory side effect.
-3. GM address/stride, alignment, layout conversion, dtype, and access size must satisfy the PTO page and active TLSU target profile.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TPREFETCH</x:t>
@@ -1028,23 +1018,12 @@
     <x:t xml:space="preserve">global memory/partition-view src</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">indexes tile</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">data: U8, S8, U16, S16, U32, S32, F16, BF16, F32; index: S32, U32</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TLSU Function 4;</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Gather-load elements from memory into a tile using per-element indices (tile world, ins/outs).</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1. 1D may declare B.DIM LB0 only; 2D uses B.DIM LB0/LB1/LB2 and ValidCol &lt;= Col.
-2. Tile operand order and destination presence follow the TLSU opcode profile.
-3. GM address/stride, alignment, layout conversion, dtype, and access size must satisfy the PTO page and active TLSU target profile.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">MSCATTER</x:t>
   </x:si>
   <x:si>
@@ -1055,9 +1034,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TLSU Function 5;</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Scatter-store elements from a tile into memory using per-element indices (tile world, ins/outs).</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Complex Layout Transformation
@@ -6004,7 +5980,7 @@
 Shared form
 BSTART.TLSU TLOAD
 B.DATR/B.DIM
-C.B.IOS
+B.IOS
 B.IOR</x:v>
       </x:c>
       <x:c r="E76" s="9" t="str">
@@ -6014,7 +5990,7 @@
         <x:v>full logical GlobalTensor/partition-view source</x:v>
       </x:c>
       <x:c r="G76" s="9" t="str">
-        <x:v>base, row stride, pad/layout attributes</x:v>
+        <x:v>base byte address, byte row stride, pad/layout attributes</x:v>
       </x:c>
       <x:c r="H76" s="9" t="str">
         <x:v>Shared full form requires exactly-one issuer</x:v>
@@ -6028,15 +6004,22 @@
       <x:c r="K76" s="2" t="s">
         <x:v>310</x:v>
       </x:c>
-      <x:c r="L76" s="3" t="s">
-        <x:v>311</x:v>
+      <x:c r="L76" s="3" t="str">
+        <x:v>Local and Shared destinations are distinguished by static type; no runtime storage switch is allowed.
+Shared TLOAD updates selected quarters atomically. Partial writes to an
+  initialized Sx require descriptor compatibility; a partial first write
+  establishes the descriptor and leaves unselected quarters uninitialized.
+The issuer pointer addresses the full object; it is not a per-PE fragment pointer.
+Shared destination TSize is 128 B–8 KiB per participating PE and cannot be implicit.
+GM alignment, dtype, layout, shape and valid-region constraints remain those of PTO TLOAD and the TLSU target.
+RecordEvent completion controls operation readiness but is not a cross-PE GM visibility fence.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="101">
       <x:c r="A77" s="49"/>
       <x:c r="B77" s="49"/>
       <x:c r="C77" s="16" t="s">
-        <x:v>312</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="D77" s="17" t="str">
         <x:v>Local form
@@ -6044,13 +6027,9 @@
 B.DATR/B.DIM
 B.IOT
 B.IOR
-Shared full form
+Shared form
 BSTART.TLSU Function 1
-C.B.IOS
-B.IOR
-Shared pe_scope form
-BSTART.TLSU Function 12
-C.B.IOS
+B.IOS
 B.IOR</x:v>
       </x:c>
       <x:c r="E77" s="17" t="str">
@@ -6060,31 +6039,36 @@
         <x:v>Local tile or SharedTile source</x:v>
       </x:c>
       <x:c r="G77" s="17" t="str">
-        <x:v>base GPR
-row-stride GPR
+        <x:v>base-byte-address GPR
+byte-row-stride GPR
 ordinary quantized-store scalar (optional)</x:v>
       </x:c>
-      <x:c r="H77" s="17" t="str">
-        <x:v>default full/core or compile-time pe_scope</x:v>
-      </x:c>
+      <x:c r="H77" s="17"/>
       <x:c r="I77" s="17" t="str">
         <x:v>PTO TSTORE dtype/layout combinations supported by the v5 TLSU profile</x:v>
       </x:c>
       <x:c r="J77" s="41" t="str">
-        <x:v>TLSU Function 1; Shared pe_scope Function 12;</x:v>
+        <x:v>TLSU Function 1</x:v>
       </x:c>
       <x:c r="K77" s="2" t="s">
-        <x:v>313</x:v>
-      </x:c>
-      <x:c r="L77" s="3" t="s">
-        <x:v>314</x:v>
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="L77" s="3" t="str">
+        <x:v>Each selected PE uses its own private GPR base and row stride. Programs must
+  ensure the resulting GM byte ranges do not conflict; the architecture does
+  not impose an order between participating PEs.
+Shared stores use zero B.IOR.RegDst; source size comes from the descriptor.
+Reading an uninitialized selected quarter is legal and produces an
+  undefined-register value without modifying the Shared descriptor.
+Source storage and scope are compile-time. Unsupported combinations are diagnostics, not runtime modes.
+GM alignment, dtype, layout, shape, atomic and ordinary quantized-store rules remain PTO/target-specific.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="101.75">
       <x:c r="A78" s="49"/>
       <x:c r="B78" s="49"/>
       <x:c r="C78" s="16" t="s">
-        <x:v>315</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="D78" s="17" t="str">
         <x:v>BSTART.TLSU TPREFETCH, DataType
@@ -6095,35 +6079,35 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E78" s="17" t="s">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="F78" s="17" t="s">
+        <x:v>315</x:v>
+      </x:c>
+      <x:c r="G78" s="17" t="s">
         <x:v>316</x:v>
-      </x:c>
-      <x:c r="F78" s="17" t="s">
-        <x:v>317</x:v>
-      </x:c>
-      <x:c r="G78" s="17" t="s">
-        <x:v>318</x:v>
       </x:c>
       <x:c r="H78" s="17"/>
       <x:c r="I78" s="17" t="s">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="J78" s="41" t="s">
+        <x:v>318</x:v>
+      </x:c>
+      <x:c r="K78" s="2" t="s">
         <x:v>319</x:v>
       </x:c>
-      <x:c r="J78" s="41" t="s">
+      <x:c r="L78" s="3" t="s">
         <x:v>320</x:v>
-      </x:c>
-      <x:c r="K78" s="2" t="s">
-        <x:v>321</x:v>
-      </x:c>
-      <x:c r="L78" s="3" t="s">
-        <x:v>322</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="101">
       <x:c r="A79" s="49"/>
       <x:c r="B79" s="48" t="s">
-        <x:v>323</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="C79" s="16" t="s">
-        <x:v>324</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="D79" s="17" t="str">
         <x:v>BSTART.TLSU MGATHER, DataType
@@ -6137,30 +6121,37 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F79" s="17" t="s">
-        <x:v>325</x:v>
-      </x:c>
-      <x:c r="G79" s="17" t="s">
-        <x:v>326</x:v>
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="G79" s="17" t="str">
+        <x:v>signed/unsigned byte-displacement index tile</x:v>
       </x:c>
       <x:c r="H79" s="17"/>
       <x:c r="I79" s="17" t="s">
-        <x:v>327</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="J79" s="41" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="K79" s="2" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="L79" s="3" t="s">
-        <x:v>330</x:v>
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="K79" s="2" t="str">
+        <x:v>PTO 来源页：../pto/MGATHER.md PTO 指令名：MGATHER C++ intrinsic / RecordEvent 签名摘录：</x:v>
+      </x:c>
+      <x:c r="L79" s="3" t="str">
+        <x:v>Tile operand 使用 Linx-style 6-bit / 64-entry TReg namespace：T#1..T#16、U#1..U#16、M#1..M#16、N#1..N#16。
+B.IOT 中表达的 operand 顺序必须与 MGATHER operand role 保持一致。
+一个 block 中最后一条 B.IOT 必须设置 last；只有一条 B.IOT 时也必须设置 last。
+B.IOT.TSize=001..111 encodes a 512 B..32 KB logical Tile (128 B..8 KB per PE fragment).
+二维 MGATHER 的 ValidCol/ValidRow/Col 均为 16-bit dimension 值，并应满足 ValidCol &lt;= Col。
+IndexTile 使用整数 dtype；其元素直接作为 byte displacement。Packed four-bit transfer dtype 因缺少 nibble selector 而在访存前拒绝。
+GM base、byte displacement、alignment、dtype、mask 和 access size 约束由 PTO/Linx 来源页和当前 TLSU target profile 共同约束。
+本指令不隐含 cross-PE visibility 或 group-level barrier。</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="101.75">
       <x:c r="A80" s="50"/>
       <x:c r="B80" s="50"/>
       <x:c r="C80" s="16" t="s">
-        <x:v>331</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="D80" s="17" t="str">
         <x:v>BSTART.TLSU MSCATTER, DataType
@@ -6171,37 +6162,43 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E80" s="17" t="s">
-        <x:v>332</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="F80" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="G80" s="17" t="s">
-        <x:v>326</x:v>
+      <x:c r="G80" s="17" t="str">
+        <x:v>signed/unsigned byte-displacement index tile</x:v>
       </x:c>
       <x:c r="H80" s="17"/>
       <x:c r="I80" s="17" t="s">
-        <x:v>333</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="J80" s="41" t="s">
-        <x:v>334</x:v>
-      </x:c>
-      <x:c r="K80" s="2" t="s">
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="L80" s="3" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="K80" s="2" t="str">
+        <x:v>PTO 来源页：../pto/MSCATTER.md PTO 指令名：MSCATTER C++ intrinsic / RecordEvent 签名摘录：</x:v>
+      </x:c>
+      <x:c r="L80" s="3" t="str">
+        <x:v>Tile operand 使用 Linx-style 6-bit / 64-entry TReg namespace：T#1..T#16、U#1..U#16、M#1..M#16、N#1..N#16。
+B.IOT 中表达的 operand 顺序必须与 MSCATTER operand role 保持一致。
+一个 block 中最后一条 B.IOT 必须设置 last；只有一条 B.IOT 时也必须设置 last。
+二维 MSCATTER 的 ValidCol/ValidRow/Col 均为 16-bit dimension 值，并应满足 ValidCol &lt;= Col。
+IndexTile 使用整数 dtype；其元素直接作为 byte displacement。Packed four-bit transfer dtype 因缺少 nibble selector 而在访存前拒绝。
+GM base、byte displacement、alignment、dtype、mask 和 access size 约束由 PTO/Linx 来源页和当前 TLSU target profile 共同约束。
+本指令不隐含 cross-PE visibility 或 group-level barrier。</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="101">
       <x:c r="A81" s="51" t="s">
-        <x:v>336</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="B81" s="52" t="s">
-        <x:v>337</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="C81" s="13" t="s">
-        <x:v>338</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="D81" s="9" t="str">
         <x:v>BSTART.TEPL TEXPANDS, DataType
@@ -6215,18 +6212,18 @@
         <x:v>221</x:v>
       </x:c>
       <x:c r="F81" s="9" t="s">
-        <x:v>339</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="G81" s="9"/>
       <x:c r="H81" s="9"/>
       <x:c r="I81" s="9" t="s">
-        <x:v>340</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="J81" s="40" t="s">
-        <x:v>341</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="K81" s="2" t="s">
-        <x:v>342</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="L81" s="3" t="s">
         <x:v>71</x:v>
@@ -6236,7 +6233,7 @@
       <x:c r="A82" s="53"/>
       <x:c r="B82" s="54"/>
       <x:c r="C82" s="16" t="s">
-        <x:v>343</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="D82" s="17" t="str">
         <x:v>BSTART.TEPL TCI, DataType
@@ -6247,33 +6244,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E82" s="17" t="s">
-        <x:v>344</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="F82" s="17" t="s">
-        <x:v>345</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="G82" s="17" t="s">
-        <x:v>346</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="H82" s="17"/>
       <x:c r="I82" s="17" t="s">
-        <x:v>347</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="J82" s="41" t="s">
-        <x:v>348</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="K82" s="2" t="s">
-        <x:v>349</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="L82" s="3" t="s">
-        <x:v>350</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="101">
       <x:c r="A83" s="53"/>
       <x:c r="B83" s="54"/>
       <x:c r="C83" s="16" t="s">
-        <x:v>351</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="D83" s="17" t="str">
         <x:v>BSTART.TEPL TTRI, DataType
@@ -6284,33 +6281,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E83" s="17" t="s">
-        <x:v>352</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="F83" s="17" t="s">
-        <x:v>353</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="G83" s="17" t="s">
-        <x:v>354</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="H83" s="17"/>
       <x:c r="I83" s="17" t="s">
-        <x:v>355</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="J83" s="41" t="s">
-        <x:v>356</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="K83" s="2" t="s">
-        <x:v>357</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="L83" s="3" t="s">
-        <x:v>358</x:v>
+        <x:v>352</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="101">
       <x:c r="A84" s="53"/>
       <x:c r="B84" s="54"/>
       <x:c r="C84" s="16" t="s">
-        <x:v>359</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="D84" s="17" t="str">
         <x:v>BSTART.TEPL TRANDOM, DataType
@@ -6321,33 +6318,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E84" s="17" t="s">
-        <x:v>360</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="F84" s="17" t="s">
-        <x:v>361</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="G84" s="17" t="s">
-        <x:v>362</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="H84" s="17"/>
       <x:c r="I84" s="17" t="s">
-        <x:v>363</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="J84" s="41" t="s">
-        <x:v>364</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="K84" s="2" t="s">
-        <x:v>365</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="L84" s="3" t="s">
-        <x:v>366</x:v>
+        <x:v>360</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="84.75">
       <x:c r="A85" s="53"/>
       <x:c r="B85" s="55"/>
       <x:c r="C85" s="24" t="s">
-        <x:v>367</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="D85" s="25" t="str">
         <x:v>BSTART.TEPL TFILLPAD, DataType
@@ -6357,35 +6354,35 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E85" s="25" t="s">
-        <x:v>368</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="F85" s="25" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G85" s="25" t="s">
-        <x:v>369</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="H85" s="25"/>
       <x:c r="I85" s="25" t="s">
-        <x:v>370</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="J85" s="43" t="s">
-        <x:v>371</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="K85" s="2" t="s">
-        <x:v>372</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="L85" s="3" t="s">
-        <x:v>373</x:v>
+        <x:v>367</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="118">
       <x:c r="A86" s="53"/>
       <x:c r="B86" s="52" t="s">
-        <x:v>374</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="C86" s="13" t="s">
-        <x:v>375</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="D86" s="17" t="str">
         <x:v>BSTART.TEPL TCVT, DataType
@@ -6395,33 +6392,33 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E86" s="17" t="s">
-        <x:v>376</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="F86" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G86" s="17" t="s">
-        <x:v>377</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="H86" s="17"/>
       <x:c r="I86" s="17" t="s">
-        <x:v>378</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="J86" s="41" t="s">
-        <x:v>379</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="K86" s="2" t="s">
-        <x:v>380</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="L86" s="3" t="s">
-        <x:v>381</x:v>
+        <x:v>375</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="84">
       <x:c r="A87" s="53"/>
       <x:c r="B87" s="54"/>
       <x:c r="C87" s="16" t="s">
-        <x:v>382</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="D87" s="17" t="str">
         <x:v>BSTART.TEPL TQUANT, DataType
@@ -6431,35 +6428,35 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E87" s="17" t="s">
-        <x:v>383</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="F87" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G87" s="17" t="s">
-        <x:v>384</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="H87" s="17" t="str">
         <x:v>offset/scaling/index Tile (optional)</x:v>
       </x:c>
       <x:c r="I87" s="17" t="s">
-        <x:v>385</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="J87" s="41" t="s">
-        <x:v>386</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="K87" s="2" t="s">
-        <x:v>387</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="L87" s="3" t="s">
-        <x:v>388</x:v>
+        <x:v>382</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="84.75">
       <x:c r="A88" s="53"/>
       <x:c r="B88" s="55"/>
       <x:c r="C88" s="16" t="s">
-        <x:v>389</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="D88" s="17" t="str">
         <x:v>BSTART.TEPL TDEQUANT, DataType
@@ -6469,37 +6466,37 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E88" s="17" t="s">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="F88" s="17" t="s">
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="G88" s="17" t="s">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="H88" s="17" t="s">
+        <x:v>387</x:v>
+      </x:c>
+      <x:c r="I88" s="17" t="s">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="J88" s="41" t="s">
+        <x:v>389</x:v>
+      </x:c>
+      <x:c r="K88" s="2" t="s">
         <x:v>390</x:v>
       </x:c>
-      <x:c r="F88" s="17" t="s">
+      <x:c r="L88" s="3" t="s">
         <x:v>391</x:v>
-      </x:c>
-      <x:c r="G88" s="17" t="s">
-        <x:v>392</x:v>
-      </x:c>
-      <x:c r="H88" s="17" t="s">
-        <x:v>393</x:v>
-      </x:c>
-      <x:c r="I88" s="17" t="s">
-        <x:v>394</x:v>
-      </x:c>
-      <x:c r="J88" s="41" t="s">
-        <x:v>395</x:v>
-      </x:c>
-      <x:c r="K88" s="2" t="s">
-        <x:v>396</x:v>
-      </x:c>
-      <x:c r="L88" s="3" t="s">
-        <x:v>397</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="101">
       <x:c r="A89" s="53"/>
       <x:c r="B89" s="52" t="s">
-        <x:v>398</x:v>
+        <x:v>392</x:v>
       </x:c>
       <x:c r="C89" s="56" t="s">
-        <x:v>399</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="D89" s="56" t="str">
         <x:v>BSTART.TEPL TEXTRACT, DataType
@@ -6510,33 +6507,33 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E89" s="9" t="s">
-        <x:v>400</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="F89" s="9" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G89" s="9" t="s">
-        <x:v>401</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="H89" s="9"/>
       <x:c r="I89" s="9" t="s">
-        <x:v>402</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="J89" s="40" t="s">
-        <x:v>403</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="K89" s="2" t="s">
-        <x:v>404</x:v>
+        <x:v>398</x:v>
       </x:c>
       <x:c r="L89" s="3" t="s">
-        <x:v>405</x:v>
+        <x:v>399</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="101">
       <x:c r="A90" s="53"/>
       <x:c r="B90" s="54"/>
       <x:c r="C90" s="57" t="s">
-        <x:v>406</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="D90" s="57" t="str">
         <x:v>BSTART.TEPL TINSERT, DataType
@@ -6550,30 +6547,30 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F90" s="17" t="s">
-        <x:v>407</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="G90" s="17" t="s">
-        <x:v>401</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="H90" s="17"/>
       <x:c r="I90" s="17" t="s">
-        <x:v>408</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="J90" s="41" t="s">
-        <x:v>409</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="K90" s="2" t="s">
-        <x:v>410</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="L90" s="3" t="s">
-        <x:v>411</x:v>
+        <x:v>405</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="101">
       <x:c r="A91" s="53"/>
       <x:c r="B91" s="54"/>
       <x:c r="C91" s="57" t="s">
-        <x:v>412</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="D91" s="57" t="str">
         <x:v>BSTART.TEPL TGATHER, DataType
@@ -6583,33 +6580,33 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E91" s="17" t="s">
-        <x:v>413</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="F91" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G91" s="17" t="s">
-        <x:v>414</x:v>
+        <x:v>408</x:v>
       </x:c>
       <x:c r="H91" s="17"/>
       <x:c r="I91" s="17" t="s">
-        <x:v>415</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="J91" s="41" t="s">
-        <x:v>416</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="K91" s="2" t="s">
-        <x:v>417</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="L91" s="3" t="s">
-        <x:v>418</x:v>
+        <x:v>412</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="84">
       <x:c r="A92" s="53"/>
       <x:c r="B92" s="54"/>
       <x:c r="C92" s="57" t="s">
-        <x:v>419</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="D92" s="57" t="str">
         <x:v>BSTART.TEPL TSCATTER, DataType
@@ -6619,33 +6616,33 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E92" s="17" t="s">
-        <x:v>420</x:v>
+        <x:v>414</x:v>
       </x:c>
       <x:c r="F92" s="17" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="G92" s="17" t="s">
-        <x:v>421</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="H92" s="17"/>
       <x:c r="I92" s="17" t="s">
-        <x:v>422</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="J92" s="41" t="s">
-        <x:v>423</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="K92" s="2" t="s">
-        <x:v>424</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="L92" s="3" t="s">
-        <x:v>425</x:v>
+        <x:v>419</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="84">
       <x:c r="A93" s="53"/>
       <x:c r="B93" s="54"/>
       <x:c r="C93" s="57" t="s">
-        <x:v>426</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="D93" s="57" t="str">
         <x:v>BSTART.TEPL TCONCAT, DataType
@@ -6668,10 +6665,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="J93" s="41" t="s">
-        <x:v>427</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="K93" s="2" t="s">
-        <x:v>428</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="L93" s="3" t="s">
         <x:v>26</x:v>
@@ -6681,7 +6678,7 @@
       <x:c r="A94" s="53"/>
       <x:c r="B94" s="54"/>
       <x:c r="C94" s="57" t="s">
-        <x:v>429</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="D94" s="57" t="str">
         <x:v>BSTART.TEPL TTRANS, DataType
@@ -6691,7 +6688,7 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E94" s="17" t="s">
-        <x:v>430</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="F94" s="17" t="s">
         <x:v>74</x:v>
@@ -6699,23 +6696,23 @@
       <x:c r="G94" s="17"/>
       <x:c r="H94" s="17"/>
       <x:c r="I94" s="17" t="s">
-        <x:v>431</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="J94" s="41" t="s">
-        <x:v>432</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="K94" s="2" t="s">
-        <x:v>433</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="L94" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>428</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="101.75">
       <x:c r="A95" s="53"/>
       <x:c r="B95" s="55"/>
       <x:c r="C95" s="58" t="s">
-        <x:v>435</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="D95" s="58" t="str">
         <x:v>BSTART.TEPL TIMG2COL, DataType
@@ -6726,35 +6723,35 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E95" s="25" t="s">
-        <x:v>436</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="F95" s="25" t="s">
-        <x:v>437</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="G95" s="25" t="s">
-        <x:v>438</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="H95" s="25"/>
       <x:c r="I95" s="25" t="s">
         <x:v>223</x:v>
       </x:c>
       <x:c r="J95" s="43" t="s">
-        <x:v>439</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="K95" s="2" t="s">
-        <x:v>440</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="L95" s="3" t="s">
-        <x:v>441</x:v>
+        <x:v>435</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="84">
       <x:c r="A96" s="53"/>
       <x:c r="B96" s="52" t="s">
-        <x:v>442</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="C96" s="40" t="s">
-        <x:v>443</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="D96" s="56" t="str">
         <x:v>BSTART.TEPL TSORT32, DataType
@@ -6764,33 +6761,33 @@
 B.IOT</x:v>
       </x:c>
       <x:c r="E96" s="9" t="s">
-        <x:v>444</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="F96" s="9" t="s">
-        <x:v>445</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="G96" s="9" t="s">
-        <x:v>446</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="H96" s="9"/>
       <x:c r="I96" s="9" t="s">
-        <x:v>447</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="J96" s="40" t="s">
-        <x:v>448</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="K96" s="2" t="s">
-        <x:v>449</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="L96" s="3" t="s">
-        <x:v>450</x:v>
+        <x:v>444</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="101.75">
       <x:c r="A97" s="53"/>
       <x:c r="B97" s="55"/>
       <x:c r="C97" s="43" t="s">
-        <x:v>451</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D97" s="58" t="str">
         <x:v>BSTART.TEPL TMRGSORT, DataType
@@ -6801,35 +6798,35 @@
 B.IOR</x:v>
       </x:c>
       <x:c r="E97" s="25" t="s">
-        <x:v>452</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="F97" s="25" t="s">
-        <x:v>453</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="G97" s="25" t="s">
-        <x:v>454</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="H97" s="25"/>
       <x:c r="I97" s="25" t="s">
         <x:v>171</x:v>
       </x:c>
       <x:c r="J97" s="43" t="s">
-        <x:v>455</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="K97" s="2" t="s">
-        <x:v>456</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="L97" s="3" t="s">
-        <x:v>457</x:v>
+        <x:v>451</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="84">
       <x:c r="A98" s="53"/>
       <x:c r="B98" s="52" t="s">
-        <x:v>458</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="C98" s="40" t="s">
-        <x:v>459</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="D98" s="56" t="str">
         <x:v>BSTART.TEPL TPARTADD, DataType
@@ -6852,10 +6849,10 @@
         <x:v>117</x:v>
       </x:c>
       <x:c r="J98" s="40" t="s">
-        <x:v>460</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="K98" s="2" t="s">
-        <x:v>461</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="L98" s="3" t="s">
         <x:v>26</x:v>
@@ -6865,7 +6862,7 @@
       <x:c r="A99" s="53"/>
       <x:c r="B99" s="54"/>
       <x:c r="C99" s="41" t="s">
-        <x:v>462</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D99" s="57" t="str">
         <x:v>BSTART.TEPL TPARTMUL, DataType
@@ -6888,10 +6885,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="J99" s="41" t="s">
-        <x:v>463</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="K99" s="2" t="s">
-        <x:v>464</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="L99" s="3" t="s">
         <x:v>26</x:v>
@@ -6901,7 +6898,7 @@
       <x:c r="A100" s="53"/>
       <x:c r="B100" s="54"/>
       <x:c r="C100" s="41" t="s">
-        <x:v>465</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="D100" s="57" t="str">
         <x:v>BSTART.TEPL TPARTMAX, DataType
@@ -6924,10 +6921,10 @@
         <x:v>223</x:v>
       </x:c>
       <x:c r="J100" s="41" t="s">
-        <x:v>466</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="K100" s="2" t="s">
-        <x:v>467</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="L100" s="3" t="s">
         <x:v>26</x:v>
@@ -6937,7 +6934,7 @@
       <x:c r="A101" s="59"/>
       <x:c r="B101" s="55"/>
       <x:c r="C101" s="43" t="s">
-        <x:v>468</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="D101" s="58" t="str">
         <x:v>BSTART.TEPL TPARTMIN, DataType
@@ -6960,10 +6957,10 @@
         <x:v>223</x:v>
       </x:c>
       <x:c r="J101" s="43" t="s">
-        <x:v>469</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="K101" s="2" t="s">
-        <x:v>470</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="L101" s="3" t="s">
         <x:v>26</x:v>
@@ -7354,106 +7351,106 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>471</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>472</x:v>
+        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26.399999618530273" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>473</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>474</x:v>
+        <x:v>468</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="26.399999618530273" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>475</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>476</x:v>
+        <x:v>470</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" customHeight="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>477</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>478</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.399999618530273" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>479</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>480</x:v>
+        <x:v>474</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>481</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>482</x:v>
+        <x:v>476</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>483</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>484</x:v>
+        <x:v>478</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>485</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>486</x:v>
+        <x:v>480</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>487</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>488</x:v>
+        <x:v>482</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40.5" customHeight="1">
       <x:c r="A10" s="3" t="s">
-        <x:v>489</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
-        <x:v>490</x:v>
+        <x:v>484</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40.5" customHeight="1">
       <x:c r="A11" s="3" t="s">
-        <x:v>491</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>486</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40.5" customHeight="1">
       <x:c r="A12" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>488</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="40.5" customHeight="1">
       <x:c r="A13" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
-        <x:v>496</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7471,98 +7468,98 @@
   <x:sheetData>
     <x:row r="1" ht="14" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>497</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="14" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>499</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>500</x:v>
+        <x:v>494</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="14" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>501</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>502</x:v>
+        <x:v>496</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="14" customHeight="1">
       <x:c r="A4" s="2" t="s">
-        <x:v>503</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>504</x:v>
+        <x:v>498</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="14" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>505</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>506</x:v>
+        <x:v>500</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="14" customHeight="1">
       <x:c r="A6" s="2" t="s">
-        <x:v>507</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>508</x:v>
+        <x:v>502</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="14" customHeight="1">
       <x:c r="A7" s="2" t="s">
-        <x:v>509</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>510</x:v>
+        <x:v>504</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="14" customHeight="1">
       <x:c r="A8" s="2" t="s">
-        <x:v>511</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>512</x:v>
+        <x:v>506</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="14" customHeight="1">
       <x:c r="A9" s="2" t="s">
-        <x:v>513</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>514</x:v>
+        <x:v>508</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="14" customHeight="1">
       <x:c r="A10" s="2" t="s">
-        <x:v>515</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
-        <x:v>516</x:v>
+        <x:v>510</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="14" customHeight="1">
       <x:c r="A11" s="2" t="s">
-        <x:v>517</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>518</x:v>
+        <x:v>512</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="14" customHeight="1">
       <x:c r="A12" s="2" t="s">
-        <x:v>519</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>520</x:v>
+        <x:v>514</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>